<commit_message>
Derive years 2-5 growth from a regional build
PR #1's regional algorithm, adapted: the guided year-1 total is split
across Americas, EIMEA and Asia-Pacific by FY2025 revenue times one plus
the regional rate, regional rates run in years 2-5 and fade in years
6-10, and the build is compressed to the one rate the Ginzu takes,
keeping year-1 and year-5 revenue. Regional rates are anchored on
FY2022-FY2025 segment history (added with its source); PR #1's rates
reproduce its own 6.1544% Base rate here and are kept as a
sensitivity. The 17.0m gap between reported and guidance-base revenue
moves the rate by at most 0.05 pp. Measured alone: Bear -2.08,
Base -0.96, Bull +9.27.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/models/excel/wd40_valuation.xlsx
+++ b/models/excel/wd40_valuation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\sunesis-ai\models\out\valuation_book\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3EC6663E-8796-480F-BEDA-DCD0FA5C3926}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{93ED054F-6A65-4899-B0FE-F88E6D8A444F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4310" yWindow="4570" windowWidth="7500" windowHeight="6000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1244,13 +1244,13 @@
         <v>0.05</v>
       </c>
       <c r="C12">
-        <v>0.04</v>
+        <v>3.2465449091496852E-2</v>
       </c>
       <c r="D12">
-        <v>0.06</v>
+        <v>5.8096824069499453E-2</v>
       </c>
       <c r="E12">
-        <v>7.0000000000000007E-2</v>
+        <v>7.9772924907641762E-2</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
@@ -2708,7 +2708,7 @@
         <v>101</v>
       </c>
       <c r="B2">
-        <v>66.1328125</v>
+        <v>65.8935546875</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
@@ -2725,7 +2725,7 @@
       </c>
       <c r="B4">
         <f>B2*B3</f>
-        <v>901.60602574218751</v>
+        <v>898.3441610595703</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
@@ -2758,7 +2758,7 @@
       </c>
       <c r="B8">
         <f>B4+B5-B6</f>
-        <v>930.47102574218752</v>
+        <v>927.20916105957031</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
@@ -2775,7 +2775,7 @@
       </c>
       <c r="B10">
         <f>B8/B9</f>
-        <v>8.3089640104138773</v>
+        <v>8.2798360574686587</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">
@@ -2842,7 +2842,7 @@
       </c>
       <c r="B18">
         <f>B4+B5+B8*B16+B12*B17</f>
-        <v>1019.8086462570313</v>
+        <v>1016.4815442807617</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.35">
@@ -2860,7 +2860,7 @@
       </c>
       <c r="B20">
         <f>B18-B12-B19</f>
-        <v>487.75064625703135</v>
+        <v>484.42354428076169</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.35">
@@ -2873,19 +2873,19 @@
       </c>
       <c r="D21">
         <f>'DCF Base'!D4</f>
-        <v>681.05000000000007</v>
+        <v>679.82720946465338</v>
       </c>
       <c r="E21">
         <f>'DCF Base'!E4</f>
-        <v>721.91300000000012</v>
+        <v>719.32301125058007</v>
       </c>
       <c r="F21">
         <f>'DCF Base'!F4</f>
-        <v>765.22778000000017</v>
+        <v>761.11339368434756</v>
       </c>
       <c r="G21">
         <f>'DCF Base'!G4</f>
-        <v>811.14144680000027</v>
+        <v>805.33166461416681</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.35">
@@ -2898,19 +2898,19 @@
       </c>
       <c r="D22">
         <f>'DCF Base'!D6+D21*(B39-B38)</f>
-        <v>124.71904650703914</v>
+        <v>124.49511982082481</v>
       </c>
       <c r="E22">
         <f>'DCF Base'!E6+E21*(B39-B38)</f>
-        <v>133.74901196412819</v>
+        <v>133.26916406523574</v>
       </c>
       <c r="F22">
         <f>'DCF Base'!F6+F21*(B39-B38)</f>
-        <v>143.41358470864253</v>
+        <v>142.64249549073159</v>
       </c>
       <c r="G22">
         <f>'DCF Base'!G6+G21*(B39-B38)</f>
-        <v>153.75640973942777</v>
+        <v>152.65513294758597</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.35">
@@ -2919,23 +2919,23 @@
       </c>
       <c r="C23">
         <f>'DCF Base'!C11</f>
-        <v>64.475333333333282</v>
+        <v>65.086728601006627</v>
       </c>
       <c r="D23">
         <f>'DCF Base'!D11</f>
-        <v>70.591123999999965</v>
+        <v>71.111296628614184</v>
       </c>
       <c r="E23">
         <f>'DCF Base'!E11</f>
-        <v>76.017644893333326</v>
+        <v>76.429417459616076</v>
       </c>
       <c r="F23">
         <f>'DCF Base'!F11</f>
-        <v>81.841220247466623</v>
+        <v>82.125452389621302</v>
       </c>
       <c r="G23">
         <f>'DCF Base'!G11</f>
-        <v>90.928956186280061</v>
+        <v>90.890754739313536</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.35">
@@ -2948,19 +2948,19 @@
       </c>
       <c r="D24">
         <f>B15*C29</f>
-        <v>36.838105306180267</v>
+        <v>36.790171917194677</v>
       </c>
       <c r="E24">
         <f>B15*D29</f>
-        <v>33.527603925703765</v>
+        <v>33.435995359808537</v>
       </c>
       <c r="F24">
         <f>B15*E29</f>
-        <v>29.591814959853313</v>
+        <v>29.462393198855555</v>
       </c>
       <c r="G24">
         <f>B15*F29</f>
-        <v>24.961861977948356</v>
+        <v>24.802343484137754</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.35">
@@ -2998,19 +2998,19 @@
       </c>
       <c r="D26">
         <f>D24*(1-D25)</f>
-        <v>28.365341085758807</v>
+        <v>28.328432376239903</v>
       </c>
       <c r="E26">
         <f>E24*(1-E25)</f>
-        <v>25.8162550227919</v>
+        <v>25.745716427052574</v>
       </c>
       <c r="F26">
         <f>F24*(1-F25)</f>
-        <v>22.785697519087051</v>
+        <v>22.686042763118778</v>
       </c>
       <c r="G26">
         <f>G24*(1-G25)</f>
-        <v>19.220633723020235</v>
+        <v>19.097804482786071</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.35">
@@ -3019,23 +3019,23 @@
       </c>
       <c r="C27">
         <f>C23-C26</f>
-        <v>34.054207829333279</v>
+        <v>34.665603097006624</v>
       </c>
       <c r="D27">
         <f>D23-D26</f>
-        <v>42.225782914241158</v>
+        <v>42.782864252374281</v>
       </c>
       <c r="E27">
         <f>E23-E26</f>
-        <v>50.201389870541426</v>
+        <v>50.683701032563505</v>
       </c>
       <c r="F27">
         <f>F23-F26</f>
-        <v>59.055522728379572</v>
+        <v>59.439409626502524</v>
       </c>
       <c r="G27">
         <f>G23-G26</f>
-        <v>71.708322463259833</v>
+        <v>71.792950256527462</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.35">
@@ -3044,23 +3044,23 @@
       </c>
       <c r="C28">
         <f>IF(C27&gt;B12,B12,C27)</f>
-        <v>34.054207829333279</v>
+        <v>34.665603097006624</v>
       </c>
       <c r="D28">
         <f>IF(D27&gt;C29,C29,D27)</f>
-        <v>42.225782914241158</v>
+        <v>42.782864252374281</v>
       </c>
       <c r="E28">
         <f>IF(E27&gt;D29,D29,E27)</f>
-        <v>50.201389870541426</v>
+        <v>50.683701032563505</v>
       </c>
       <c r="F28">
         <f>IF(F27&gt;E29,E29,F27)</f>
-        <v>59.055522728379572</v>
+        <v>59.439409626502524</v>
       </c>
       <c r="G28">
         <f>IF(G27&gt;F29,F29,G27)</f>
-        <v>71.708322463259833</v>
+        <v>71.792950256527462</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.35">
@@ -3073,23 +3073,23 @@
       </c>
       <c r="C29">
         <f>B12-C28</f>
-        <v>469.87379217066672</v>
+        <v>469.26239690299337</v>
       </c>
       <c r="D29">
         <f>C29-D28</f>
-        <v>427.64800925642555</v>
+        <v>426.47953265061909</v>
       </c>
       <c r="E29">
         <f>D29-E28</f>
-        <v>377.44661938588411</v>
+        <v>375.79583161805556</v>
       </c>
       <c r="F29">
         <f>E29-F28</f>
-        <v>318.39109665750453</v>
+        <v>316.35642199155302</v>
       </c>
       <c r="G29">
         <f>F29-G28</f>
-        <v>246.6827741942447</v>
+        <v>244.56347173502556</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.35">
@@ -3106,11 +3106,11 @@
       </c>
       <c r="D30">
         <f>C30+D27-D28</f>
-        <v>30.000000000000007</v>
+        <v>30</v>
       </c>
       <c r="E30">
         <f>D30+E27-E28</f>
-        <v>30.000000000000007</v>
+        <v>30</v>
       </c>
       <c r="F30">
         <f>E30+F27-F28</f>
@@ -3135,7 +3135,7 @@
       </c>
       <c r="B32">
         <f>B31*G22</f>
-        <v>1705.257983713919</v>
+        <v>1693.0441121442741</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.35">
@@ -3144,7 +3144,7 @@
       </c>
       <c r="B33">
         <f>B32-G29+G30</f>
-        <v>1488.5752095196742</v>
+        <v>1478.4806404092485</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.35">
@@ -3153,7 +3153,7 @@
       </c>
       <c r="B34">
         <f>B33/B20</f>
-        <v>3.0519184770802652</v>
+        <v>3.0520412516373323</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.35">
@@ -3162,7 +3162,7 @@
       </c>
       <c r="B35">
         <f>B34^(1/5)-1</f>
-        <v>0.25001316136525809</v>
+        <v>0.25002321847155828</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.35">
@@ -3234,7 +3234,7 @@
         <v>101</v>
       </c>
       <c r="B2">
-        <v>76.15234375</v>
+        <v>75.859375</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
@@ -3251,7 +3251,7 @@
       </c>
       <c r="B4">
         <f>B2*B3</f>
-        <v>1038.2049304101563</v>
+        <v>1034.2108103906251</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
@@ -3284,7 +3284,7 @@
       </c>
       <c r="B8">
         <f>B4+B5-B6</f>
-        <v>1067.0699304101563</v>
+        <v>1063.0758103906251</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
@@ -3301,7 +3301,7 @@
       </c>
       <c r="B10">
         <f>B8/B9</f>
-        <v>9.528771345997253</v>
+        <v>9.4931044648398437</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">
@@ -3368,7 +3368,7 @@
       </c>
       <c r="B18">
         <f>B4+B5+B8*B16+B12*B17</f>
-        <v>1160.5393290183597</v>
+        <v>1156.4653265984377</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.35">
@@ -3386,7 +3386,7 @@
       </c>
       <c r="B20">
         <f>B18-B12-B19</f>
-        <v>572.48932901835974</v>
+        <v>568.41532659843779</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.35">
@@ -3399,19 +3399,19 @@
       </c>
       <c r="D21">
         <f>'DCF Base'!D4</f>
-        <v>681.05000000000007</v>
+        <v>679.82720946465338</v>
       </c>
       <c r="E21">
         <f>'DCF Base'!E4</f>
-        <v>721.91300000000012</v>
+        <v>719.32301125058007</v>
       </c>
       <c r="F21">
         <f>'DCF Base'!F4</f>
-        <v>765.22778000000017</v>
+        <v>761.11339368434756</v>
       </c>
       <c r="G21">
         <f>'DCF Base'!G4</f>
-        <v>811.14144680000027</v>
+        <v>805.33166461416681</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.35">
@@ -3424,19 +3424,19 @@
       </c>
       <c r="D22">
         <f>'DCF Base'!D6+D21*(B39-B38)</f>
-        <v>124.71904650703914</v>
+        <v>124.49511982082481</v>
       </c>
       <c r="E22">
         <f>'DCF Base'!E6+E21*(B39-B38)</f>
-        <v>133.74901196412819</v>
+        <v>133.26916406523574</v>
       </c>
       <c r="F22">
         <f>'DCF Base'!F6+F21*(B39-B38)</f>
-        <v>143.41358470864253</v>
+        <v>142.64249549073159</v>
       </c>
       <c r="G22">
         <f>'DCF Base'!G6+G21*(B39-B38)</f>
-        <v>153.75640973942777</v>
+        <v>152.65513294758597</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.35">
@@ -3445,23 +3445,23 @@
       </c>
       <c r="C23">
         <f>'DCF Base'!C11</f>
-        <v>64.475333333333282</v>
+        <v>65.086728601006627</v>
       </c>
       <c r="D23">
         <f>'DCF Base'!D11</f>
-        <v>70.591123999999965</v>
+        <v>71.111296628614184</v>
       </c>
       <c r="E23">
         <f>'DCF Base'!E11</f>
-        <v>76.017644893333326</v>
+        <v>76.429417459616076</v>
       </c>
       <c r="F23">
         <f>'DCF Base'!F11</f>
-        <v>81.841220247466623</v>
+        <v>82.125452389621302</v>
       </c>
       <c r="G23">
         <f>'DCF Base'!G11</f>
-        <v>90.928956186280061</v>
+        <v>90.890754739313536</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.35">
@@ -3474,19 +3474,19 @@
       </c>
       <c r="D24">
         <f>B15*C29</f>
-        <v>41.492879910570664</v>
+        <v>41.444946521585074</v>
       </c>
       <c r="E24">
         <f>B15*D29</f>
-        <v>38.463377963411993</v>
+        <v>38.371769397516772</v>
       </c>
       <c r="F24">
         <f>B15*E29</f>
-        <v>34.825551804669914</v>
+        <v>34.696130043672163</v>
       </c>
       <c r="G24">
         <f>B15*F29</f>
-        <v>30.511549048612846</v>
+        <v>30.352030554802255</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.35">
@@ -3524,19 +3524,19 @@
       </c>
       <c r="D26">
         <f>D24*(1-D25)</f>
-        <v>31.949517531139414</v>
+        <v>31.912608821620509</v>
       </c>
       <c r="E26">
         <f>E24*(1-E25)</f>
-        <v>29.616801031827237</v>
+        <v>29.546262436087915</v>
       </c>
       <c r="F26">
         <f>F24*(1-F25)</f>
-        <v>26.815674889595833</v>
+        <v>26.716020133627566</v>
       </c>
       <c r="G26">
         <f>G24*(1-G25)</f>
-        <v>23.493892767431891</v>
+        <v>23.371063527197737</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.35">
@@ -3545,23 +3545,23 @@
       </c>
       <c r="C27">
         <f>C23-C26</f>
-        <v>30.674082773333289</v>
+        <v>31.285478041006634</v>
       </c>
       <c r="D27">
         <f>D23-D26</f>
-        <v>38.641606468860552</v>
+        <v>39.198687806993675</v>
       </c>
       <c r="E27">
         <f>E23-E26</f>
-        <v>46.40084386150609</v>
+        <v>46.883155023528161</v>
       </c>
       <c r="F27">
         <f>F23-F26</f>
-        <v>55.02554535787079</v>
+        <v>55.409432255993735</v>
       </c>
       <c r="G27">
         <f>G23-G26</f>
-        <v>67.435063418848173</v>
+        <v>67.519691212115802</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.35">
@@ -3570,23 +3570,23 @@
       </c>
       <c r="C28">
         <f>IF(C27&gt;B12,B12,C27)</f>
-        <v>30.674082773333289</v>
+        <v>31.285478041006634</v>
       </c>
       <c r="D28">
         <f>IF(D27&gt;C29,C29,D27)</f>
-        <v>38.641606468860552</v>
+        <v>39.198687806993675</v>
       </c>
       <c r="E28">
         <f>IF(E27&gt;D29,D29,E27)</f>
-        <v>46.40084386150609</v>
+        <v>46.883155023528161</v>
       </c>
       <c r="F28">
         <f>IF(F27&gt;E29,E29,F27)</f>
-        <v>55.02554535787079</v>
+        <v>55.409432255993735</v>
       </c>
       <c r="G28">
         <f>IF(G27&gt;F29,F29,G27)</f>
-        <v>67.435063418848173</v>
+        <v>67.519691212115802</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.35">
@@ -3599,23 +3599,23 @@
       </c>
       <c r="C29">
         <f>B12-C28</f>
-        <v>529.24591722666662</v>
+        <v>528.63452195899333</v>
       </c>
       <c r="D29">
         <f>C29-D28</f>
-        <v>490.60431075780605</v>
+        <v>489.43583415199964</v>
       </c>
       <c r="E29">
         <f>D29-E28</f>
-        <v>444.20346689629997</v>
+        <v>442.55267912847148</v>
       </c>
       <c r="F29">
         <f>E29-F28</f>
-        <v>389.17792153842919</v>
+        <v>387.14324687247773</v>
       </c>
       <c r="G29">
         <f>F29-G28</f>
-        <v>321.742858119581</v>
+        <v>319.62355566036194</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.35">
@@ -3632,19 +3632,19 @@
       </c>
       <c r="D30">
         <f>C30+D27-D28</f>
-        <v>29.999999999999993</v>
+        <v>30</v>
       </c>
       <c r="E30">
         <f>D30+E27-E28</f>
-        <v>29.999999999999986</v>
+        <v>30</v>
       </c>
       <c r="F30">
         <f>E30+F27-F28</f>
-        <v>29.999999999999993</v>
+        <v>30</v>
       </c>
       <c r="G30">
         <f>F30+G27-G28</f>
-        <v>29.999999999999986</v>
+        <v>30</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.35">
@@ -3661,7 +3661,7 @@
       </c>
       <c r="B32">
         <f>B31*G22</f>
-        <v>1716.3810998123329</v>
+        <v>1704.0875591763192</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.35">
@@ -3670,7 +3670,7 @@
       </c>
       <c r="B33">
         <f>B32-G29+G30</f>
-        <v>1424.6382416927518</v>
+        <v>1414.4640035159573</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.35">
@@ -3679,7 +3679,7 @@
       </c>
       <c r="B34">
         <f>B33/B20</f>
-        <v>2.4884974609667592</v>
+        <v>2.488433962505058</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.35">
@@ -3688,7 +3688,7 @@
       </c>
       <c r="B35">
         <f>B34^(1/5)-1</f>
-        <v>0.20001711573153358</v>
+        <v>0.20001099155260116</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.35">
@@ -3760,7 +3760,7 @@
         <v>101</v>
       </c>
       <c r="B2">
-        <v>108.408203125</v>
+        <v>107.8955078125</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
@@ -3777,7 +3777,7 @@
       </c>
       <c r="B4">
         <f>B2*B3</f>
-        <v>1477.9575445605469</v>
+        <v>1470.9678345263671</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
@@ -3810,7 +3810,7 @@
       </c>
       <c r="B8">
         <f>B4+B5-B6</f>
-        <v>1506.8225445605467</v>
+        <v>1499.8328345263672</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
@@ -3827,7 +3827,7 @@
       </c>
       <c r="B10">
         <f>B8/B9</f>
-        <v>13.455694961427943</v>
+        <v>13.393277919402479</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">
@@ -3894,7 +3894,7 @@
       </c>
       <c r="B18">
         <f>B4+B5+B8*B16+B12*B17</f>
-        <v>1610.4867954517576</v>
+        <v>1603.3572912168945</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.35">
@@ -3912,7 +3912,7 @@
       </c>
       <c r="B20">
         <f>B18-B12-B19</f>
-        <v>966.44479545175773</v>
+        <v>959.31529121689459</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.35">
@@ -3925,19 +3925,19 @@
       </c>
       <c r="D21">
         <f>'DCF Base'!D4</f>
-        <v>681.05000000000007</v>
+        <v>679.82720946465338</v>
       </c>
       <c r="E21">
         <f>'DCF Base'!E4</f>
-        <v>721.91300000000012</v>
+        <v>719.32301125058007</v>
       </c>
       <c r="F21">
         <f>'DCF Base'!F4</f>
-        <v>765.22778000000017</v>
+        <v>761.11339368434756</v>
       </c>
       <c r="G21">
         <f>'DCF Base'!G4</f>
-        <v>811.14144680000027</v>
+        <v>805.33166461416681</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.35">
@@ -3950,19 +3950,19 @@
       </c>
       <c r="D22">
         <f>'DCF Base'!D6+D21*(B39-B38)</f>
-        <v>124.71904650703914</v>
+        <v>124.49511982082481</v>
       </c>
       <c r="E22">
         <f>'DCF Base'!E6+E21*(B39-B38)</f>
-        <v>133.74901196412819</v>
+        <v>133.26916406523574</v>
       </c>
       <c r="F22">
         <f>'DCF Base'!F6+F21*(B39-B38)</f>
-        <v>143.41358470864253</v>
+        <v>142.64249549073159</v>
       </c>
       <c r="G22">
         <f>'DCF Base'!G6+G21*(B39-B38)</f>
-        <v>153.75640973942777</v>
+        <v>152.65513294758597</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.35">
@@ -3971,23 +3971,23 @@
       </c>
       <c r="C23">
         <f>'DCF Base'!C11</f>
-        <v>64.475333333333282</v>
+        <v>65.086728601006627</v>
       </c>
       <c r="D23">
         <f>'DCF Base'!D11</f>
-        <v>70.591123999999965</v>
+        <v>71.111296628614184</v>
       </c>
       <c r="E23">
         <f>'DCF Base'!E11</f>
-        <v>76.017644893333326</v>
+        <v>76.429417459616076</v>
       </c>
       <c r="F23">
         <f>'DCF Base'!F11</f>
-        <v>81.841220247466623</v>
+        <v>82.125452389621302</v>
       </c>
       <c r="G23">
         <f>'DCF Base'!G11</f>
-        <v>90.928956186280061</v>
+        <v>90.890754739313536</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.35">
@@ -4000,19 +4000,19 @@
       </c>
       <c r="D24">
         <f>B15*C29</f>
-        <v>46.147654514961062</v>
+        <v>46.099721125975471</v>
       </c>
       <c r="E24">
         <f>B15*D29</f>
-        <v>43.399152001120235</v>
+        <v>43.307543435225007</v>
       </c>
       <c r="F24">
         <f>B15*E29</f>
-        <v>40.059288649486525</v>
+        <v>39.929866888488775</v>
       </c>
       <c r="G24">
         <f>B15*F29</f>
-        <v>36.061236119277346</v>
+        <v>35.901717625466752</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.35">
@@ -4050,19 +4050,19 @@
       </c>
       <c r="D26">
         <f>D24*(1-D25)</f>
-        <v>35.53369397652002</v>
+        <v>35.496785267001115</v>
       </c>
       <c r="E26">
         <f>E24*(1-E25)</f>
-        <v>33.41734704086258</v>
+        <v>33.346808445123258</v>
       </c>
       <c r="F26">
         <f>F24*(1-F25)</f>
-        <v>30.845652260104625</v>
+        <v>30.745997504136358</v>
       </c>
       <c r="G26">
         <f>G24*(1-G25)</f>
-        <v>27.767151811843558</v>
+        <v>27.644322571609401</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.35">
@@ -4071,23 +4071,23 @@
       </c>
       <c r="C27">
         <f>C23-C26</f>
-        <v>27.293957717333292</v>
+        <v>27.905352985006637</v>
       </c>
       <c r="D27">
         <f>D23-D26</f>
-        <v>35.057430023479945</v>
+        <v>35.614511361613069</v>
       </c>
       <c r="E27">
         <f>E23-E26</f>
-        <v>42.600297852470746</v>
+        <v>43.082609014492817</v>
       </c>
       <c r="F27">
         <f>F23-F26</f>
-        <v>50.995567987361994</v>
+        <v>51.379454885484947</v>
       </c>
       <c r="G27">
         <f>G23-G26</f>
-        <v>63.1618043744365</v>
+        <v>63.246432167704135</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.35">
@@ -4096,23 +4096,23 @@
       </c>
       <c r="C28">
         <f>IF(C27&gt;B12,B12,C27)</f>
-        <v>27.293957717333292</v>
+        <v>27.905352985006637</v>
       </c>
       <c r="D28">
         <f>IF(D27&gt;C29,C29,D27)</f>
-        <v>35.057430023479945</v>
+        <v>35.614511361613069</v>
       </c>
       <c r="E28">
         <f>IF(E27&gt;D29,D29,E27)</f>
-        <v>42.600297852470746</v>
+        <v>43.082609014492817</v>
       </c>
       <c r="F28">
         <f>IF(F27&gt;E29,E29,F27)</f>
-        <v>50.995567987361994</v>
+        <v>51.379454885484947</v>
       </c>
       <c r="G28">
         <f>IF(G27&gt;F29,F29,G27)</f>
-        <v>63.1618043744365</v>
+        <v>63.246432167704135</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.35">
@@ -4125,23 +4125,23 @@
       </c>
       <c r="C29">
         <f>B12-C28</f>
-        <v>588.61804228266658</v>
+        <v>588.00664701499329</v>
       </c>
       <c r="D29">
         <f>C29-D28</f>
-        <v>553.56061225918666</v>
+        <v>552.39213565338025</v>
       </c>
       <c r="E29">
         <f>D29-E28</f>
-        <v>510.9603144067159</v>
+        <v>509.30952663888741</v>
       </c>
       <c r="F29">
         <f>E29-F28</f>
-        <v>459.9647464193539</v>
+        <v>457.93007175340244</v>
       </c>
       <c r="G29">
         <f>F29-G28</f>
-        <v>396.80294204491742</v>
+        <v>394.6836395856983</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.35">
@@ -4158,19 +4158,19 @@
       </c>
       <c r="D30">
         <f>C30+D27-D28</f>
-        <v>30.000000000000007</v>
+        <v>30</v>
       </c>
       <c r="E30">
         <f>D30+E27-E28</f>
-        <v>30.000000000000014</v>
+        <v>30</v>
       </c>
       <c r="F30">
         <f>E30+F27-F28</f>
-        <v>30.000000000000014</v>
+        <v>30</v>
       </c>
       <c r="G30">
         <f>F30+G27-G28</f>
-        <v>30.000000000000014</v>
+        <v>30.000000000000007</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.35">
@@ -4187,7 +4187,7 @@
       </c>
       <c r="B32">
         <f>B31*G22</f>
-        <v>2531.4847449574277</v>
+        <v>2513.3530429799443</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.35">
@@ -4196,7 +4196,7 @@
       </c>
       <c r="B33">
         <f>B32-G29+G30</f>
-        <v>2164.6818029125102</v>
+        <v>2148.6694033942458</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.35">
@@ -4205,7 +4205,7 @@
       </c>
       <c r="B34">
         <f>B33/B20</f>
-        <v>2.2398400954714077</v>
+        <v>2.2397948026749908</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.35">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="B35">
         <f>B34^(1/5)-1</f>
-        <v>0.17501497885164818</v>
+        <v>0.17501022671377831</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.35">
@@ -4306,39 +4306,39 @@
       </c>
       <c r="D2">
         <f>'DCF Base'!D4</f>
-        <v>681.05000000000007</v>
+        <v>679.82720946465338</v>
       </c>
       <c r="E2">
         <f>'DCF Base'!E4</f>
-        <v>721.91300000000012</v>
+        <v>719.32301125058007</v>
       </c>
       <c r="F2">
         <f>'DCF Base'!F4</f>
-        <v>765.22778000000017</v>
+        <v>761.11339368434756</v>
       </c>
       <c r="G2">
         <f>'DCF Base'!G4</f>
-        <v>811.14144680000027</v>
+        <v>805.33166461416681</v>
       </c>
       <c r="H2">
         <f>'DCF Base'!H4</f>
-        <v>854.1319434804002</v>
+        <v>846.78809256658678</v>
       </c>
       <c r="I2">
         <f>'DCF Base'!I4</f>
-        <v>893.42201288049864</v>
+        <v>884.77339279504542</v>
       </c>
       <c r="J2">
         <f>'DCF Base'!J4</f>
-        <v>928.26547138283797</v>
+        <v>918.60600334400624</v>
       </c>
       <c r="K2">
         <f>'DCF Base'!K4</f>
-        <v>957.96996646708885</v>
+        <v>947.6517416839788</v>
       </c>
       <c r="L2">
         <f>'DCF Base'!L4</f>
-        <v>981.91921562876598</v>
+        <v>971.3430352260782</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.35">
@@ -4386,39 +4386,39 @@
       </c>
       <c r="D4">
         <f>D2*B10*D3</f>
-        <v>21.96935483870968</v>
+        <v>21.929909982730752</v>
       </c>
       <c r="E4">
         <f>E2*B10*E3</f>
-        <v>23.287516129032262</v>
+        <v>23.20396810485742</v>
       </c>
       <c r="F4">
         <f>F2*B10*F3</f>
-        <v>24.684767096774198</v>
+        <v>24.552044957559598</v>
       </c>
       <c r="G4">
         <f>G2*B10*G3</f>
-        <v>26.165853122580653</v>
+        <v>25.97844079400538</v>
       </c>
       <c r="H4">
         <f>H2*B10*H3</f>
-        <v>27.552643338077424</v>
+        <v>27.315744921502798</v>
       </c>
       <c r="I4">
         <f>I2*B10*I3</f>
-        <v>28.820064931628988</v>
+        <v>28.541077186936949</v>
       </c>
       <c r="J4">
         <f>J2*B10*J3</f>
-        <v>29.944047463962516</v>
+        <v>29.632451720774394</v>
       </c>
       <c r="K4">
         <f>K2*B10*K3</f>
-        <v>30.902256982809316</v>
+        <v>30.569411022063832</v>
       </c>
       <c r="L4">
         <f>L2*B10*L3</f>
-        <v>31.674813407379546</v>
+        <v>31.333646297615424</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.35">
@@ -4427,11 +4427,11 @@
       </c>
       <c r="C5">
         <f>0.5*B11*D2*B10</f>
-        <v>10.98467741935484</v>
+        <v>10.964954991365376</v>
       </c>
       <c r="D5">
         <f>0.5*B11*D2*B10</f>
-        <v>10.98467741935484</v>
+        <v>10.964954991365376</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -4509,43 +4509,43 @@
       </c>
       <c r="C7">
         <f t="shared" ref="C7:L7" si="0">(C4-C5)*(1-C6)</f>
-        <v>-0.47876612903225896</v>
+        <v>-0.46357985948037161</v>
       </c>
       <c r="D7">
         <f t="shared" si="0"/>
-        <v>8.4582016129032276</v>
+        <v>8.4430153433513393</v>
       </c>
       <c r="E7">
         <f t="shared" si="0"/>
-        <v>17.931387419354841</v>
+        <v>17.867055440740213</v>
       </c>
       <c r="F7">
         <f t="shared" si="0"/>
-        <v>19.007270664516135</v>
+        <v>18.905074617320892</v>
       </c>
       <c r="G7">
         <f t="shared" si="0"/>
-        <v>20.147706904387103</v>
+        <v>20.003399411384144</v>
       </c>
       <c r="H7">
         <f t="shared" si="0"/>
-        <v>21.105324796967306</v>
+        <v>20.923860609871145</v>
       </c>
       <c r="I7">
         <f t="shared" si="0"/>
-        <v>21.96088947790129</v>
+        <v>21.748300816445955</v>
       </c>
       <c r="J7">
         <f t="shared" si="0"/>
-        <v>22.697587977683586</v>
+        <v>22.461398404346991</v>
       </c>
       <c r="K7">
         <f t="shared" si="0"/>
-        <v>23.300301765038224</v>
+        <v>23.049335910636131</v>
       </c>
       <c r="L7">
         <f t="shared" si="0"/>
-        <v>23.756110055534659</v>
+        <v>23.50023472321157</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.35">
@@ -4599,43 +4599,43 @@
       </c>
       <c r="C9">
         <f t="shared" ref="C9:L9" si="1">C7*C8</f>
-        <v>-0.44577282433239629</v>
+        <v>-0.43163308917004989</v>
       </c>
       <c r="D9">
         <f t="shared" si="1"/>
-        <v>7.3326064228840986</v>
+        <v>7.3194411020804484</v>
       </c>
       <c r="E9">
         <f t="shared" si="1"/>
-        <v>14.473861308197401</v>
+        <v>14.42193380730893</v>
       </c>
       <c r="F9">
         <f t="shared" si="1"/>
-        <v>14.285006523405839</v>
+        <v>14.208200588107843</v>
       </c>
       <c r="G9">
         <f t="shared" si="1"/>
-        <v>14.098615913790423</v>
+        <v>13.997634897589135</v>
       </c>
       <c r="H9">
         <f t="shared" si="1"/>
-        <v>13.750961492892165</v>
+        <v>13.632730332125718</v>
       </c>
       <c r="I9">
         <f t="shared" si="1"/>
-        <v>13.322358712694149</v>
+        <v>13.193393881419468</v>
       </c>
       <c r="J9">
         <f t="shared" si="1"/>
-        <v>12.820385253246609</v>
+        <v>12.686977186893818</v>
       </c>
       <c r="K9">
         <f t="shared" si="1"/>
-        <v>12.253864803262037</v>
+        <v>12.121879317361898</v>
       </c>
       <c r="L9">
         <f t="shared" si="1"/>
-        <v>11.632606527530735</v>
+        <v>11.507312569300304</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.35">
@@ -4678,7 +4678,7 @@
       </c>
       <c r="B14">
         <f>L4*(1+B12)*(1-'DCF Base'!M7)/(B13-B12)</f>
-        <v>496.7999398044621</v>
+        <v>491.44894381234081</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.35">
@@ -4687,7 +4687,7 @@
       </c>
       <c r="B15">
         <f>B14*L8</f>
-        <v>243.2670251626428</v>
+        <v>240.64681374077162</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.35">
@@ -4696,7 +4696,7 @@
       </c>
       <c r="B16">
         <f>SUM(C9:L9)</f>
-        <v>113.52449413357107</v>
+        <v>112.65787059301752</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.35">
@@ -4705,7 +4705,7 @@
       </c>
       <c r="B17">
         <f>B16+B15</f>
-        <v>356.79151929621389</v>
+        <v>353.30468433378917</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.35">
@@ -4722,7 +4722,7 @@
       </c>
       <c r="B19">
         <f>B17/B18</f>
-        <v>26.17066210020403</v>
+        <v>25.914902715057224</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.35">
@@ -4731,7 +4731,7 @@
       </c>
       <c r="B20">
         <f>'DCF Base'!B30</f>
-        <v>126.29998915646284</v>
+        <v>125.33517043256788</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.35">
@@ -4740,7 +4740,7 @@
       </c>
       <c r="B21">
         <f>B20+B19</f>
-        <v>152.47065125666688</v>
+        <v>151.2500731476251</v>
       </c>
     </row>
   </sheetData>
@@ -4799,39 +4799,39 @@
       </c>
       <c r="D2">
         <f>'DCF Base'!D4</f>
-        <v>681.05000000000007</v>
+        <v>679.82720946465338</v>
       </c>
       <c r="E2">
         <f>'DCF Base'!E4</f>
-        <v>721.91300000000012</v>
+        <v>719.32301125058007</v>
       </c>
       <c r="F2">
         <f>'DCF Base'!F4</f>
-        <v>765.22778000000017</v>
+        <v>761.11339368434756</v>
       </c>
       <c r="G2">
         <f>'DCF Base'!G4</f>
-        <v>811.14144680000027</v>
+        <v>805.33166461416681</v>
       </c>
       <c r="H2">
         <f>'DCF Base'!H4</f>
-        <v>854.1319434804002</v>
+        <v>846.78809256658678</v>
       </c>
       <c r="I2">
         <f>'DCF Base'!I4</f>
-        <v>893.42201288049864</v>
+        <v>884.77339279504542</v>
       </c>
       <c r="J2">
         <f>'DCF Base'!J4</f>
-        <v>928.26547138283797</v>
+        <v>918.60600334400624</v>
       </c>
       <c r="K2">
         <f>'DCF Base'!K4</f>
-        <v>957.96996646708885</v>
+        <v>947.6517416839788</v>
       </c>
       <c r="L2">
         <f>'DCF Base'!L4</f>
-        <v>981.91921562876598</v>
+        <v>971.3430352260782</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.35">
@@ -4879,39 +4879,39 @@
       </c>
       <c r="D4">
         <f>D2*B10*D3</f>
-        <v>32.828650586701436</v>
+        <v>32.769708419128392</v>
       </c>
       <c r="E4">
         <f>E2*B10*E3</f>
-        <v>34.798369621903525</v>
+        <v>34.673524403963292</v>
       </c>
       <c r="F4">
         <f>F2*B10*F3</f>
-        <v>36.886271799217738</v>
+        <v>36.687946051129835</v>
       </c>
       <c r="G4">
         <f>G2*B10*G3</f>
-        <v>39.099448107170808</v>
+        <v>38.81939919833362</v>
       </c>
       <c r="H4">
         <f>H2*B10*H3</f>
-        <v>41.171718856850859</v>
+        <v>40.81772323889269</v>
       </c>
       <c r="I4">
         <f>I2*B10*I3</f>
-        <v>43.065617924266</v>
+        <v>42.648728522838098</v>
       </c>
       <c r="J4">
         <f>J2*B10*J3</f>
-        <v>44.745177023312365</v>
+        <v>44.279561721792334</v>
       </c>
       <c r="K4">
         <f>K2*B10*K3</f>
-        <v>46.177022688058365</v>
+        <v>45.67965333767328</v>
       </c>
       <c r="L4">
         <f>L2*B10*L3</f>
-        <v>47.331448255259822</v>
+        <v>46.821644671115109</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.35">
@@ -4920,11 +4920,11 @@
       </c>
       <c r="C5">
         <f>0.5*B11*D2*B10</f>
-        <v>16.414325293350718</v>
+        <v>16.384854209564196</v>
       </c>
       <c r="D5">
         <f>0.5*B11*D2*B10</f>
-        <v>16.414325293350718</v>
+        <v>16.384854209564196</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -5002,43 +5002,43 @@
       </c>
       <c r="C7">
         <f t="shared" ref="C7:L7" si="0">(C4-C5)*(1-C6)</f>
-        <v>-0.71541681938943735</v>
+        <v>-0.69272408487381565</v>
       </c>
       <c r="D7">
         <f t="shared" si="0"/>
-        <v>12.639030475880054</v>
+        <v>12.616337741364431</v>
       </c>
       <c r="E7">
         <f t="shared" si="0"/>
-        <v>26.794744608865717</v>
+        <v>26.698613791051734</v>
       </c>
       <c r="F7">
         <f t="shared" si="0"/>
-        <v>28.402429285397659</v>
+        <v>28.249718459369973</v>
       </c>
       <c r="G7">
         <f t="shared" si="0"/>
-        <v>30.106575042521523</v>
+        <v>29.890937382716888</v>
       </c>
       <c r="H7">
         <f t="shared" si="0"/>
-        <v>31.53753664434776</v>
+        <v>31.266376000991801</v>
       </c>
       <c r="I7">
         <f t="shared" si="0"/>
-        <v>32.816000858290693</v>
+        <v>32.498331134402633</v>
       </c>
       <c r="J7">
         <f t="shared" si="0"/>
-        <v>33.916844183670776</v>
+        <v>33.563907785118587</v>
       </c>
       <c r="K7">
         <f t="shared" si="0"/>
-        <v>34.81747510679601</v>
+        <v>34.442458616605656</v>
       </c>
       <c r="L7">
         <f t="shared" si="0"/>
-        <v>35.498586191444865</v>
+        <v>35.116233503336332</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.35">
@@ -5092,43 +5092,43 @@
       </c>
       <c r="C9">
         <f t="shared" ref="C9:L9" si="1">C7*C8</f>
-        <v>-0.66611515897909546</v>
+        <v>-0.64498625335391846</v>
       </c>
       <c r="D9">
         <f t="shared" si="1"/>
-        <v>10.957061593930852</v>
+        <v>10.937388748747283</v>
       </c>
       <c r="E9">
         <f t="shared" si="1"/>
-        <v>21.628187947056581</v>
+        <v>21.550593052030145</v>
       </c>
       <c r="F9">
         <f t="shared" si="1"/>
-        <v>21.34598358616088</v>
+        <v>21.231213023648046</v>
       </c>
       <c r="G9">
         <f t="shared" si="1"/>
-        <v>21.067461424694162</v>
+        <v>20.916566210833764</v>
       </c>
       <c r="H9">
         <f t="shared" si="1"/>
-        <v>20.547963897689804</v>
+        <v>20.371291915569376</v>
       </c>
       <c r="I9">
         <f t="shared" si="1"/>
-        <v>19.907505813467068</v>
+        <v>19.714794583894243</v>
       </c>
       <c r="J9">
         <f t="shared" si="1"/>
-        <v>19.157410445397129</v>
+        <v>18.95805972126815</v>
       </c>
       <c r="K9">
         <f t="shared" si="1"/>
-        <v>18.310862968727729</v>
+        <v>18.113637996445103</v>
       </c>
       <c r="L9">
         <f t="shared" si="1"/>
-        <v>17.382521148596361</v>
+        <v>17.195295278489148</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.35">
@@ -5171,7 +5171,7 @@
       </c>
       <c r="B14">
         <f>L4*(1+B12)*(1-'DCF Base'!M7)/(B13-B12)</f>
-        <v>742.36461448555156</v>
+        <v>734.36865925582993</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.35">
@@ -5180,7 +5180,7 @@
       </c>
       <c r="B15">
         <f>B14*L8</f>
-        <v>363.51218444791419</v>
+        <v>359.59682116740805</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.35">
@@ -5189,7 +5189,7 @@
       </c>
       <c r="B16">
         <f>SUM(C9:L9)</f>
-        <v>169.63884366674148</v>
+        <v>168.34385427757132</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.35">
@@ -5198,7 +5198,7 @@
       </c>
       <c r="B17">
         <f>B16+B15</f>
-        <v>533.15102811465567</v>
+        <v>527.94067544497943</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.35">
@@ -5215,7 +5215,7 @@
       </c>
       <c r="B19">
         <f>B17/B18</f>
-        <v>39.106634128209492</v>
+        <v>38.724454699141319</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.35">
@@ -5224,7 +5224,7 @@
       </c>
       <c r="B20">
         <f>'DCF Base'!B30</f>
-        <v>126.29998915646284</v>
+        <v>125.33517043256788</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.35">
@@ -5233,7 +5233,7 @@
       </c>
       <c r="B21">
         <f>B20+B19</f>
-        <v>165.40662328467232</v>
+        <v>164.0596251317092</v>
       </c>
     </row>
   </sheetData>
@@ -5292,39 +5292,39 @@
       </c>
       <c r="D2">
         <f>'DCF Base'!D4</f>
-        <v>681.05000000000007</v>
+        <v>679.82720946465338</v>
       </c>
       <c r="E2">
         <f>'DCF Base'!E4</f>
-        <v>721.91300000000012</v>
+        <v>719.32301125058007</v>
       </c>
       <c r="F2">
         <f>'DCF Base'!F4</f>
-        <v>765.22778000000017</v>
+        <v>761.11339368434756</v>
       </c>
       <c r="G2">
         <f>'DCF Base'!G4</f>
-        <v>811.14144680000027</v>
+        <v>805.33166461416681</v>
       </c>
       <c r="H2">
         <f>'DCF Base'!H4</f>
-        <v>854.1319434804002</v>
+        <v>846.78809256658678</v>
       </c>
       <c r="I2">
         <f>'DCF Base'!I4</f>
-        <v>893.42201288049864</v>
+        <v>884.77339279504542</v>
       </c>
       <c r="J2">
         <f>'DCF Base'!J4</f>
-        <v>928.26547138283797</v>
+        <v>918.60600334400624</v>
       </c>
       <c r="K2">
         <f>'DCF Base'!K4</f>
-        <v>957.96996646708885</v>
+        <v>947.6517416839788</v>
       </c>
       <c r="L2">
         <f>'DCF Base'!L4</f>
-        <v>981.91921562876598</v>
+        <v>971.3430352260782</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.35">
@@ -5372,39 +5372,39 @@
       </c>
       <c r="D4">
         <f>D2*B10*D3</f>
-        <v>47.515116279069773</v>
+        <v>47.429805311487442</v>
       </c>
       <c r="E4">
         <f>E2*B10*E3</f>
-        <v>50.366023255813964</v>
+        <v>50.185326366319536</v>
       </c>
       <c r="F4">
         <f>F2*B10*F3</f>
-        <v>53.387984651162803</v>
+        <v>53.100934443094012</v>
       </c>
       <c r="G4">
         <f>G2*B10*G3</f>
-        <v>56.591263730232576</v>
+        <v>56.185930089360475</v>
       </c>
       <c r="H4">
         <f>H2*B10*H3</f>
-        <v>59.590600707934897</v>
+        <v>59.078239016273493</v>
       </c>
       <c r="I4">
         <f>I2*B10*I3</f>
-        <v>62.331768340499906</v>
+        <v>61.728376241514795</v>
       </c>
       <c r="J4">
         <f>J2*B10*J3</f>
-        <v>64.762707305779387</v>
+        <v>64.088790930977183</v>
       </c>
       <c r="K4">
         <f>K2*B10*K3</f>
-        <v>66.835113939564337</v>
+        <v>66.1152377919055</v>
       </c>
       <c r="L4">
         <f>L2*B10*L3</f>
-        <v>68.505991788053436</v>
+        <v>67.76811873670313</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.35">
@@ -5413,11 +5413,11 @@
       </c>
       <c r="C5">
         <f>0.5*B11*D2*B10</f>
-        <v>23.757558139534886</v>
+        <v>23.714902655743721</v>
       </c>
       <c r="D5">
         <f>0.5*B11*D2*B10</f>
-        <v>23.757558139534886</v>
+        <v>23.714902655743721</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -5495,43 +5495,43 @@
       </c>
       <c r="C7">
         <f t="shared" ref="C7:L7" si="0">(C4-C5)*(1-C6)</f>
-        <v>-1.0354709302325613</v>
+        <v>-1.0026262077133641</v>
       </c>
       <c r="D7">
         <f t="shared" si="0"/>
-        <v>18.293319767441862</v>
+        <v>18.260475044922664</v>
       </c>
       <c r="E7">
         <f t="shared" si="0"/>
-        <v>38.781837906976754</v>
+        <v>38.642701302066044</v>
       </c>
       <c r="F7">
         <f t="shared" si="0"/>
-        <v>41.108748181395356</v>
+        <v>40.88771952118239</v>
       </c>
       <c r="G7">
         <f t="shared" si="0"/>
-        <v>43.575273072279082</v>
+        <v>43.263166168807565</v>
       </c>
       <c r="H7">
         <f t="shared" si="0"/>
-        <v>45.646400142278132</v>
+        <v>45.253931086465499</v>
       </c>
       <c r="I7">
         <f t="shared" si="0"/>
-        <v>47.496807475460926</v>
+        <v>47.037022696034278</v>
       </c>
       <c r="J7">
         <f t="shared" si="0"/>
-        <v>49.090132137780778</v>
+        <v>48.579303525680707</v>
       </c>
       <c r="K7">
         <f t="shared" si="0"/>
-        <v>50.393675910431512</v>
+        <v>49.850889295096749</v>
       </c>
       <c r="L7">
         <f t="shared" si="0"/>
-        <v>51.379493841040073</v>
+        <v>50.826089052527351</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.35">
@@ -5585,43 +5585,43 @@
       </c>
       <c r="C9">
         <f t="shared" ref="C9:L9" si="1">C7*C8</f>
-        <v>-0.96411331774216058</v>
+        <v>-0.93353203006545882</v>
       </c>
       <c r="D9">
         <f t="shared" si="1"/>
-        <v>15.85889296112142</v>
+        <v>15.830419127755388</v>
       </c>
       <c r="E9">
         <f t="shared" si="1"/>
-        <v>31.303932596799033</v>
+        <v>31.191624280923968</v>
       </c>
       <c r="F9">
         <f t="shared" si="1"/>
-        <v>30.895479225040532</v>
+        <v>30.729364062651843</v>
       </c>
       <c r="G9">
         <f t="shared" si="1"/>
-        <v>30.492355348430451</v>
+        <v>30.273954545948595</v>
       </c>
       <c r="H9">
         <f t="shared" si="1"/>
-        <v>29.740451600906312</v>
+        <v>29.484742346225392</v>
       </c>
       <c r="I9">
         <f t="shared" si="1"/>
-        <v>28.813473494896645</v>
+        <v>28.534549557488617</v>
       </c>
       <c r="J9">
         <f t="shared" si="1"/>
-        <v>27.72780996632406</v>
+        <v>27.439276241421521</v>
       </c>
       <c r="K9">
         <f t="shared" si="1"/>
-        <v>26.502544807055102</v>
+        <v>26.217087825922249</v>
       </c>
       <c r="L9">
         <f t="shared" si="1"/>
-        <v>25.15889318745019</v>
+        <v>24.887908580114612</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.35">
@@ -5664,7 +5664,7 @@
       </c>
       <c r="B14">
         <f>L4*(1+B12)*(1-'DCF Base'!M7)/(B13-B12)</f>
-        <v>1074.474288414302</v>
+        <v>1062.9012040592488</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.35">
@@ -5673,7 +5673,7 @@
       </c>
       <c r="B15">
         <f>B14*L8</f>
-        <v>526.13565907269265</v>
+        <v>520.46869018352936</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.35">
@@ -5682,7 +5682,7 @@
       </c>
       <c r="B16">
         <f>SUM(C9:L9)</f>
-        <v>245.52971987028158</v>
+        <v>243.65539453838673</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.35">
@@ -5691,7 +5691,7 @@
       </c>
       <c r="B17">
         <f>B16+B15</f>
-        <v>771.66537894297426</v>
+        <v>764.12408472191612</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.35">
@@ -5708,7 +5708,7 @@
       </c>
       <c r="B19">
         <f>B17/B18</f>
-        <v>56.601664542301741</v>
+        <v>56.048510523263296</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.35">
@@ -5717,7 +5717,7 @@
       </c>
       <c r="B20">
         <f>'DCF Base'!B30</f>
-        <v>126.29998915646284</v>
+        <v>125.33517043256788</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.35">
@@ -5726,7 +5726,7 @@
       </c>
       <c r="B21">
         <f>B20+B19</f>
-        <v>182.90165369876459</v>
+        <v>181.38368095583118</v>
       </c>
     </row>
   </sheetData>
@@ -7612,35 +7612,35 @@
       </c>
       <c r="D3">
         <f>'Scenario inputs'!C12</f>
-        <v>0.04</v>
+        <v>3.2465449091496852E-2</v>
       </c>
       <c r="E3">
         <f>'Scenario inputs'!C12</f>
-        <v>0.04</v>
+        <v>3.2465449091496852E-2</v>
       </c>
       <c r="F3">
         <f>'Scenario inputs'!C12</f>
-        <v>0.04</v>
+        <v>3.2465449091496852E-2</v>
       </c>
       <c r="G3">
         <f>'Scenario inputs'!C12</f>
-        <v>0.04</v>
+        <v>3.2465449091496852E-2</v>
       </c>
       <c r="H3">
         <f>G3-((G3-M3)/5)*1</f>
-        <v>3.6000000000000004E-2</v>
+        <v>2.9972359273197482E-2</v>
       </c>
       <c r="I3">
         <f>G3-((G3-M3)/5)*2</f>
-        <v>3.2000000000000001E-2</v>
+        <v>2.7479269454898113E-2</v>
       </c>
       <c r="J3">
         <f>G3-((G3-M3)/5)*3</f>
-        <v>2.8000000000000001E-2</v>
+        <v>2.498617963659874E-2</v>
       </c>
       <c r="K3">
         <f>G3-((G3-M3)/5)*4</f>
-        <v>2.4E-2</v>
+        <v>2.249308981829937E-2</v>
       </c>
       <c r="L3">
         <f>G3-((G3-M3)/5)*5</f>
@@ -7665,43 +7665,43 @@
       </c>
       <c r="D4">
         <f t="shared" si="0"/>
-        <v>655.20000000000005</v>
+        <v>650.45323292764306</v>
       </c>
       <c r="E4">
         <f t="shared" si="0"/>
-        <v>681.40800000000002</v>
+        <v>671.57048924765502</v>
       </c>
       <c r="F4">
         <f t="shared" si="0"/>
-        <v>708.66432000000009</v>
+        <v>693.37332677767643</v>
       </c>
       <c r="G4">
         <f t="shared" si="0"/>
-        <v>737.01089280000008</v>
+        <v>715.88400321957886</v>
       </c>
       <c r="H4">
         <f t="shared" si="0"/>
-        <v>763.54328494080005</v>
+        <v>737.34073576201092</v>
       </c>
       <c r="I4">
         <f t="shared" si="0"/>
-        <v>787.97667005890571</v>
+        <v>757.60232052008814</v>
       </c>
       <c r="J4">
         <f t="shared" si="0"/>
-        <v>810.04001682055514</v>
+        <v>776.53190819370707</v>
       </c>
       <c r="K4">
         <f t="shared" si="0"/>
-        <v>829.48097722424848</v>
+        <v>793.99851015148352</v>
       </c>
       <c r="L4">
         <f t="shared" si="0"/>
-        <v>846.07059676873348</v>
+        <v>809.87848035451316</v>
       </c>
       <c r="M4">
         <f t="shared" si="0"/>
-        <v>862.99200870410812</v>
+        <v>826.07604996160342</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.35">
@@ -7771,43 +7771,43 @@
       </c>
       <c r="D6">
         <f t="shared" si="1"/>
-        <v>109.47733333333335</v>
+        <v>108.68419627436491</v>
       </c>
       <c r="E6">
         <f t="shared" si="1"/>
-        <v>113.85642666666668</v>
+        <v>112.21267751556056</v>
       </c>
       <c r="F6">
         <f t="shared" si="1"/>
-        <v>118.41068373333336</v>
+        <v>115.85571248486255</v>
       </c>
       <c r="G6">
         <f t="shared" si="1"/>
-        <v>123.14711108266668</v>
+        <v>119.61702022049894</v>
       </c>
       <c r="H6">
         <f t="shared" si="1"/>
-        <v>127.58040708164268</v>
+        <v>123.20222452573707</v>
       </c>
       <c r="I6">
         <f t="shared" si="1"/>
-        <v>131.66298010825525</v>
+        <v>126.58773165092266</v>
       </c>
       <c r="J6">
         <f t="shared" si="1"/>
-        <v>135.34954355128642</v>
+        <v>129.75067545374216</v>
       </c>
       <c r="K6">
         <f t="shared" si="1"/>
-        <v>138.5979325965173</v>
+        <v>132.66916905070821</v>
       </c>
       <c r="L6">
         <f t="shared" si="1"/>
-        <v>141.36989124844763</v>
+        <v>135.32255243172236</v>
       </c>
       <c r="M6">
         <f t="shared" si="1"/>
-        <v>144.19728907341658</v>
+        <v>138.02900348035681</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.35">
@@ -7877,43 +7877,43 @@
       </c>
       <c r="D8">
         <f t="shared" si="2"/>
-        <v>83.750160000000008</v>
+        <v>83.143410149889149</v>
       </c>
       <c r="E8">
         <f t="shared" si="2"/>
-        <v>87.100166400000006</v>
+        <v>85.842698299403821</v>
       </c>
       <c r="F8">
         <f t="shared" si="2"/>
-        <v>90.584173056000026</v>
+        <v>88.629620050919854</v>
       </c>
       <c r="G8">
         <f t="shared" si="2"/>
-        <v>94.207539978240021</v>
+        <v>91.507020468681688</v>
       </c>
       <c r="H8">
         <f t="shared" si="2"/>
-        <v>97.216270196211724</v>
+        <v>93.88009508861164</v>
       </c>
       <c r="I8">
         <f t="shared" si="2"/>
-        <v>99.932201902165744</v>
+        <v>96.080088323050305</v>
       </c>
       <c r="J8">
         <f t="shared" si="2"/>
-        <v>102.32425492477253</v>
+        <v>98.091510643029068</v>
       </c>
       <c r="K8">
         <f t="shared" si="2"/>
-        <v>104.36424324517752</v>
+        <v>99.899884295183284</v>
       </c>
       <c r="L8">
         <f t="shared" si="2"/>
-        <v>106.02741843633572</v>
+        <v>101.49191432379178</v>
       </c>
       <c r="M8">
         <f>M6*(1-M7)</f>
-        <v>108.14796680506244</v>
+        <v>103.52175261026761</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.35">
@@ -7967,47 +7967,47 @@
       </c>
       <c r="C10">
         <f t="shared" ref="C10:L10" si="3">(D4-C4)/C9</f>
-        <v>12.600000000000023</v>
+        <v>10.226616463821529</v>
       </c>
       <c r="D10">
         <f t="shared" si="3"/>
-        <v>13.103999999999985</v>
+        <v>10.558628160005981</v>
       </c>
       <c r="E10">
         <f t="shared" si="3"/>
-        <v>13.628160000000037</v>
+        <v>10.901418765010703</v>
       </c>
       <c r="F10">
         <f t="shared" si="3"/>
-        <v>14.173286399999995</v>
+        <v>11.255338220951216</v>
       </c>
       <c r="G10">
         <f t="shared" si="3"/>
-        <v>13.266196070399985</v>
+        <v>10.728366271216032</v>
       </c>
       <c r="H10">
         <f t="shared" si="3"/>
-        <v>12.216692559052831</v>
+        <v>10.13079237903861</v>
       </c>
       <c r="I10">
         <f t="shared" si="3"/>
-        <v>11.031673380824714</v>
+        <v>9.4647938368094628</v>
       </c>
       <c r="J10">
         <f t="shared" si="3"/>
-        <v>9.7204802018466694</v>
+        <v>8.7333009788882237</v>
       </c>
       <c r="K10">
         <f t="shared" si="3"/>
-        <v>8.2948097722425018</v>
+        <v>7.9399851015148215</v>
       </c>
       <c r="L10">
         <f t="shared" si="3"/>
-        <v>8.4607059676873178</v>
+        <v>8.0987848035451293</v>
       </c>
       <c r="M10">
         <f>IF(M3&gt;0,(M3/B17)*M8,0)</f>
-        <v>25.992928433729084</v>
+        <v>24.881036476470626</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.35">
@@ -8016,47 +8016,47 @@
       </c>
       <c r="C11">
         <f t="shared" ref="C11:M11" si="4">C8-C10</f>
-        <v>67.928999999999974</v>
+        <v>70.302383536178468</v>
       </c>
       <c r="D11">
         <f t="shared" si="4"/>
-        <v>70.646160000000023</v>
+        <v>72.584781989883169</v>
       </c>
       <c r="E11">
         <f t="shared" si="4"/>
-        <v>73.47200639999997</v>
+        <v>74.941279534393118</v>
       </c>
       <c r="F11">
         <f t="shared" si="4"/>
-        <v>76.410886656000031</v>
+        <v>77.374281829968638</v>
       </c>
       <c r="G11">
         <f t="shared" si="4"/>
-        <v>80.941343907840036</v>
+        <v>80.778654197465656</v>
       </c>
       <c r="H11">
         <f t="shared" si="4"/>
-        <v>84.999577637158893</v>
+        <v>83.74930270957303</v>
       </c>
       <c r="I11">
         <f t="shared" si="4"/>
-        <v>88.90052852134103</v>
+        <v>86.615294486240842</v>
       </c>
       <c r="J11">
         <f t="shared" si="4"/>
-        <v>92.603774722925863</v>
+        <v>89.358209664140844</v>
       </c>
       <c r="K11">
         <f t="shared" si="4"/>
-        <v>96.069433472935017</v>
+        <v>91.959899193668463</v>
       </c>
       <c r="L11">
         <f t="shared" si="4"/>
-        <v>97.566712468648404</v>
+        <v>93.393129520246646</v>
       </c>
       <c r="M11">
         <f t="shared" si="4"/>
-        <v>82.155038371333347</v>
+        <v>78.640716133796985</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.35">
@@ -8159,43 +8159,43 @@
       </c>
       <c r="C14">
         <f t="shared" ref="C14:L14" si="6">C11*C13</f>
-        <v>63.07120357355349</v>
+        <v>65.274859687561261</v>
       </c>
       <c r="D14">
         <f t="shared" si="6"/>
-        <v>60.903234097738761</v>
+        <v>62.574497601330144</v>
       </c>
       <c r="E14">
         <f t="shared" si="6"/>
-        <v>58.809785027144741</v>
+        <v>59.985847059660848</v>
       </c>
       <c r="F14">
         <f t="shared" si="6"/>
-        <v>56.788294844713256</v>
+        <v>57.504286656686389</v>
       </c>
       <c r="G14">
         <f t="shared" si="6"/>
-        <v>55.853436300228488</v>
+        <v>55.741172543087956</v>
       </c>
       <c r="H14">
         <f t="shared" si="6"/>
-        <v>54.396759148666078</v>
+        <v>53.59662688923504</v>
       </c>
       <c r="I14">
         <f t="shared" si="6"/>
-        <v>52.70342268241339</v>
+        <v>51.34865396187412</v>
       </c>
       <c r="J14">
         <f t="shared" si="6"/>
-        <v>50.797624691679061</v>
+        <v>49.017276144744798</v>
       </c>
       <c r="K14">
         <f t="shared" si="6"/>
-        <v>48.706034513105557</v>
+        <v>46.622550607736883</v>
       </c>
       <c r="L14">
         <f t="shared" si="6"/>
-        <v>45.66518272053635</v>
+        <v>43.711776449936394</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.35">
@@ -8208,43 +8208,43 @@
       </c>
       <c r="C15">
         <f t="shared" ref="C15:L15" si="7">B15+C10</f>
-        <v>326.03700000000003</v>
+        <v>323.66361646382154</v>
       </c>
       <c r="D15">
         <f t="shared" si="7"/>
-        <v>339.14100000000002</v>
+        <v>334.22224462382752</v>
       </c>
       <c r="E15">
         <f t="shared" si="7"/>
-        <v>352.76916000000006</v>
+        <v>345.12366338883822</v>
       </c>
       <c r="F15">
         <f t="shared" si="7"/>
-        <v>366.94244640000005</v>
+        <v>356.37900160978944</v>
       </c>
       <c r="G15">
         <f t="shared" si="7"/>
-        <v>380.20864247040004</v>
+        <v>367.10736788100547</v>
       </c>
       <c r="H15">
         <f t="shared" si="7"/>
-        <v>392.42533502945287</v>
+        <v>377.23816026004408</v>
       </c>
       <c r="I15">
         <f t="shared" si="7"/>
-        <v>403.45700841027758</v>
+        <v>386.70295409685355</v>
       </c>
       <c r="J15">
         <f t="shared" si="7"/>
-        <v>413.17748861212425</v>
+        <v>395.43625507574177</v>
       </c>
       <c r="K15">
         <f t="shared" si="7"/>
-        <v>421.47229838436675</v>
+        <v>403.37624017725659</v>
       </c>
       <c r="L15">
         <f t="shared" si="7"/>
-        <v>429.93300435205407</v>
+        <v>411.47502498080172</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.35">
@@ -8261,39 +8261,39 @@
       </c>
       <c r="D16">
         <f t="shared" si="8"/>
-        <v>0.25687317697071194</v>
+        <v>0.25688216382882428</v>
       </c>
       <c r="E16">
         <f t="shared" si="8"/>
-        <v>0.25682582288782541</v>
+        <v>0.25684316253701528</v>
       </c>
       <c r="F16">
         <f t="shared" si="8"/>
-        <v>0.25678030657781992</v>
+        <v>0.25680539891309656</v>
       </c>
       <c r="G16">
         <f t="shared" si="8"/>
-        <v>0.25673655610707241</v>
+        <v>0.25676883333568457</v>
       </c>
       <c r="H16">
         <f t="shared" si="8"/>
-        <v>0.25569190001718645</v>
+        <v>0.2557292588010438</v>
       </c>
       <c r="I16">
         <f t="shared" si="8"/>
-        <v>0.25465277845699102</v>
+        <v>0.25469344950897538</v>
       </c>
       <c r="J16">
         <f t="shared" si="8"/>
-        <v>0.25361873208735652</v>
+        <v>0.25366113603171775</v>
       </c>
       <c r="K16">
         <f t="shared" si="8"/>
-        <v>0.25258937411072463</v>
+        <v>0.25263208168924339</v>
       </c>
       <c r="L16">
         <f t="shared" si="8"/>
-        <v>0.25156438238710233</v>
+        <v>0.25160607942399615</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.35">
@@ -8311,7 +8311,7 @@
       </c>
       <c r="B18">
         <f>M11/(M12-M3)</f>
-        <v>1299.6464216864545</v>
+        <v>1244.0518238235315</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.35">
@@ -8320,7 +8320,7 @@
       </c>
       <c r="B19">
         <f>B18*L13</f>
-        <v>608.28729201543979</v>
+        <v>582.26676303122395</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.35">
@@ -8329,7 +8329,7 @@
       </c>
       <c r="B20">
         <f>SUM(C14:L14)</f>
-        <v>547.69497759977924</v>
+        <v>545.37754760185385</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.35">
@@ -8338,7 +8338,7 @@
       </c>
       <c r="B21">
         <f>B19+B20</f>
-        <v>1155.9822696152191</v>
+        <v>1127.6443106330778</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.35">
@@ -8383,7 +8383,7 @@
       </c>
       <c r="B26">
         <f>B21-B22-B24+B23+B25</f>
-        <v>1127.1172696152194</v>
+        <v>1098.7793106330778</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.35">
@@ -8401,7 +8401,7 @@
       </c>
       <c r="B28">
         <f>B26-B27</f>
-        <v>1127.1172696152194</v>
+        <v>1098.7793106330778</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.35">
@@ -8419,7 +8419,7 @@
       </c>
       <c r="B30">
         <f>B28/B29</f>
-        <v>82.674064867318947</v>
+        <v>80.595475245587053</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.35">
@@ -8428,7 +8428,7 @@
       </c>
       <c r="B31">
         <f>B19/B21</f>
-        <v>0.52620815042251001</v>
+        <v>0.51635676031951061</v>
       </c>
     </row>
   </sheetData>
@@ -8528,35 +8528,35 @@
       </c>
       <c r="D3">
         <f>'Scenario inputs'!D12</f>
-        <v>0.06</v>
+        <v>5.8096824069499453E-2</v>
       </c>
       <c r="E3">
         <f>'Scenario inputs'!D12</f>
-        <v>0.06</v>
+        <v>5.8096824069499453E-2</v>
       </c>
       <c r="F3">
         <f>'Scenario inputs'!D12</f>
-        <v>0.06</v>
+        <v>5.8096824069499453E-2</v>
       </c>
       <c r="G3">
         <f>'Scenario inputs'!D12</f>
-        <v>0.06</v>
+        <v>5.8096824069499453E-2</v>
       </c>
       <c r="H3">
         <f>G3-((G3-M3)/5)*1</f>
-        <v>5.2999999999999999E-2</v>
+        <v>5.1477459255599566E-2</v>
       </c>
       <c r="I3">
         <f>G3-((G3-M3)/5)*2</f>
-        <v>4.5999999999999999E-2</v>
+        <v>4.4858094441699671E-2</v>
       </c>
       <c r="J3">
         <f>G3-((G3-M3)/5)*3</f>
-        <v>3.9E-2</v>
+        <v>3.8238729627799783E-2</v>
       </c>
       <c r="K3">
         <f>G3-((G3-M3)/5)*4</f>
-        <v>3.2000000000000001E-2</v>
+        <v>3.1619364813899889E-2</v>
       </c>
       <c r="L3">
         <f>G3-((G3-M3)/5)*5</f>
@@ -8581,43 +8581,43 @@
       </c>
       <c r="D4">
         <f t="shared" si="0"/>
-        <v>681.05000000000007</v>
+        <v>679.82720946465338</v>
       </c>
       <c r="E4">
         <f t="shared" si="0"/>
-        <v>721.91300000000012</v>
+        <v>719.32301125058007</v>
       </c>
       <c r="F4">
         <f t="shared" si="0"/>
-        <v>765.22778000000017</v>
+        <v>761.11339368434756</v>
       </c>
       <c r="G4">
         <f t="shared" si="0"/>
-        <v>811.14144680000027</v>
+        <v>805.33166461416681</v>
       </c>
       <c r="H4">
         <f t="shared" si="0"/>
-        <v>854.1319434804002</v>
+        <v>846.78809256658678</v>
       </c>
       <c r="I4">
         <f t="shared" si="0"/>
-        <v>893.42201288049864</v>
+        <v>884.77339279504542</v>
       </c>
       <c r="J4">
         <f t="shared" si="0"/>
-        <v>928.26547138283797</v>
+        <v>918.60600334400624</v>
       </c>
       <c r="K4">
         <f t="shared" si="0"/>
-        <v>957.96996646708885</v>
+        <v>947.6517416839788</v>
       </c>
       <c r="L4">
         <f t="shared" si="0"/>
-        <v>981.91921562876598</v>
+        <v>971.3430352260782</v>
       </c>
       <c r="M4">
         <f t="shared" si="0"/>
-        <v>1006.4671960194851</v>
+        <v>995.62661110673002</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.35">
@@ -8687,43 +8687,43 @@
       </c>
       <c r="D6">
         <f t="shared" si="1"/>
-        <v>118.21119999999999</v>
+        <v>117.99895782023056</v>
       </c>
       <c r="E6">
         <f t="shared" si="1"/>
-        <v>126.85069466666668</v>
+        <v>126.39559568376599</v>
       </c>
       <c r="F6">
         <f t="shared" si="1"/>
-        <v>136.10136837333334</v>
+        <v>135.36959461627393</v>
       </c>
       <c r="G6">
         <f t="shared" si="1"/>
-        <v>146.00546042400003</v>
+        <v>144.95969963055003</v>
       </c>
       <c r="H6">
         <f t="shared" si="1"/>
-        <v>153.74374982647203</v>
+        <v>152.42185666198563</v>
       </c>
       <c r="I6">
         <f t="shared" si="1"/>
-        <v>160.81596231848974</v>
+        <v>159.25921070310818</v>
       </c>
       <c r="J6">
         <f t="shared" si="1"/>
-        <v>167.08778484891084</v>
+        <v>165.34908060192112</v>
       </c>
       <c r="K6">
         <f t="shared" si="1"/>
-        <v>172.43459396407599</v>
+        <v>170.57731350311619</v>
       </c>
       <c r="L6">
         <f t="shared" si="1"/>
-        <v>176.74545881317786</v>
+        <v>174.84174634069407</v>
       </c>
       <c r="M6">
         <f t="shared" si="1"/>
-        <v>181.16409528350729</v>
+        <v>179.2127899992114</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.35">
@@ -8793,43 +8793,43 @@
       </c>
       <c r="D8">
         <f t="shared" si="2"/>
-        <v>91.022623999999993</v>
+        <v>90.859197521577528</v>
       </c>
       <c r="E8">
         <f t="shared" si="2"/>
-        <v>97.675034893333347</v>
+        <v>97.324608676499821</v>
       </c>
       <c r="F8">
         <f t="shared" si="2"/>
-        <v>104.79805364746667</v>
+        <v>104.23458785453093</v>
       </c>
       <c r="G8">
         <f t="shared" si="2"/>
-        <v>112.42420452648003</v>
+        <v>111.61896871552352</v>
       </c>
       <c r="H8">
         <f t="shared" si="2"/>
-        <v>117.76771236707758</v>
+        <v>116.75514220308099</v>
       </c>
       <c r="I8">
         <f t="shared" si="2"/>
-        <v>122.54176328668919</v>
+        <v>121.35551855576844</v>
       </c>
       <c r="J8">
         <f t="shared" si="2"/>
-        <v>126.65254091547442</v>
+        <v>125.3346030962562</v>
       </c>
       <c r="K8">
         <f t="shared" si="2"/>
-        <v>130.01568384891328</v>
+        <v>128.6152943813496</v>
       </c>
       <c r="L8">
         <f t="shared" si="2"/>
-        <v>132.5590941098834</v>
+        <v>131.13130975552056</v>
       </c>
       <c r="M8">
         <f>M6*(1-M7)</f>
-        <v>135.87307146263046</v>
+        <v>134.40959249940855</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.35">
@@ -8883,47 +8883,47 @@
       </c>
       <c r="C10">
         <f t="shared" ref="C10:L10" si="3">(D4-C4)/C9</f>
-        <v>19.275000000000034</v>
+        <v>18.663604732326689</v>
       </c>
       <c r="D10">
         <f t="shared" si="3"/>
-        <v>20.431500000000028</v>
+        <v>19.747900892963344</v>
       </c>
       <c r="E10">
         <f t="shared" si="3"/>
-        <v>21.657390000000021</v>
+        <v>20.895191216883745</v>
       </c>
       <c r="F10">
         <f t="shared" si="3"/>
-        <v>22.95683340000005</v>
+        <v>22.109135464909627</v>
       </c>
       <c r="G10">
         <f t="shared" si="3"/>
-        <v>21.495248340199964</v>
+        <v>20.728213976209986</v>
       </c>
       <c r="H10">
         <f t="shared" si="3"/>
-        <v>19.645034700049223</v>
+        <v>18.99265011422932</v>
       </c>
       <c r="I10">
         <f t="shared" si="3"/>
-        <v>17.421729251169666</v>
+        <v>16.916305274480408</v>
       </c>
       <c r="J10">
         <f t="shared" si="3"/>
-        <v>14.85224754212544</v>
+        <v>14.522869169986279</v>
       </c>
       <c r="K10">
         <f t="shared" si="3"/>
-        <v>11.974624580838565</v>
+        <v>11.845646771049701</v>
       </c>
       <c r="L10">
         <f t="shared" si="3"/>
-        <v>12.273990195359545</v>
+        <v>12.141787940325912</v>
       </c>
       <c r="M10">
         <f>IF(M3&gt;0,(M3/B17)*M8,0)</f>
-        <v>22.645511910438412</v>
+        <v>22.401598749901428</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.35">
@@ -8932,47 +8932,47 @@
       </c>
       <c r="C11">
         <f t="shared" ref="C11:M11" si="4">C8-C10</f>
-        <v>64.475333333333282</v>
+        <v>65.086728601006627</v>
       </c>
       <c r="D11">
         <f t="shared" si="4"/>
-        <v>70.591123999999965</v>
+        <v>71.111296628614184</v>
       </c>
       <c r="E11">
         <f t="shared" si="4"/>
-        <v>76.017644893333326</v>
+        <v>76.429417459616076</v>
       </c>
       <c r="F11">
         <f t="shared" si="4"/>
-        <v>81.841220247466623</v>
+        <v>82.125452389621302</v>
       </c>
       <c r="G11">
         <f t="shared" si="4"/>
-        <v>90.928956186280061</v>
+        <v>90.890754739313536</v>
       </c>
       <c r="H11">
         <f t="shared" si="4"/>
-        <v>98.122677667028356</v>
+        <v>97.762492088851673</v>
       </c>
       <c r="I11">
         <f t="shared" si="4"/>
-        <v>105.12003403551952</v>
+        <v>104.43921328128803</v>
       </c>
       <c r="J11">
         <f t="shared" si="4"/>
-        <v>111.80029337334898</v>
+        <v>110.81173392626992</v>
       </c>
       <c r="K11">
         <f t="shared" si="4"/>
-        <v>118.04105926807472</v>
+        <v>116.7696476102999</v>
       </c>
       <c r="L11">
         <f t="shared" si="4"/>
-        <v>120.28510391452386</v>
+        <v>118.98952181519465</v>
       </c>
       <c r="M11">
         <f t="shared" si="4"/>
-        <v>113.22755955219205</v>
+        <v>112.00799374950712</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.35">
@@ -9075,43 +9075,43 @@
       </c>
       <c r="C14">
         <f t="shared" ref="C14:L14" si="6">C11*C13</f>
-        <v>60.032131967790264</v>
+        <v>60.601394032767807</v>
       </c>
       <c r="D14">
         <f t="shared" si="6"/>
-        <v>61.197043169480402</v>
+        <v>61.647992594919309</v>
       </c>
       <c r="E14">
         <f t="shared" si="6"/>
-        <v>61.359939609262753</v>
+        <v>61.692314281423592</v>
       </c>
       <c r="F14">
         <f t="shared" si="6"/>
-        <v>61.508166309279858</v>
+        <v>61.721782355292248</v>
       </c>
       <c r="G14">
         <f t="shared" si="6"/>
-        <v>63.628701509107948</v>
+        <v>63.60196955739314</v>
       </c>
       <c r="H14">
         <f t="shared" si="6"/>
-        <v>63.93084092089687</v>
+        <v>63.696165640442793</v>
       </c>
       <c r="I14">
         <f t="shared" si="6"/>
-        <v>63.770040039637038</v>
+        <v>63.35702679096849</v>
       </c>
       <c r="J14">
         <f t="shared" si="6"/>
-        <v>63.148684956374218</v>
+        <v>62.590312279517505</v>
       </c>
       <c r="K14">
         <f t="shared" si="6"/>
-        <v>62.078989194690195</v>
+        <v>61.410340920484536</v>
       </c>
       <c r="L14">
         <f t="shared" si="6"/>
-        <v>58.899764384397301</v>
+        <v>58.265359309223903</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.35">
@@ -9124,43 +9124,43 @@
       </c>
       <c r="C15">
         <f t="shared" ref="C15:L15" si="7">B15+C10</f>
-        <v>332.71200000000005</v>
+        <v>332.1006047323267</v>
       </c>
       <c r="D15">
         <f t="shared" si="7"/>
-        <v>353.14350000000007</v>
+        <v>351.84850562529004</v>
       </c>
       <c r="E15">
         <f t="shared" si="7"/>
-        <v>374.80089000000009</v>
+        <v>372.74369684217379</v>
       </c>
       <c r="F15">
         <f t="shared" si="7"/>
-        <v>397.75772340000015</v>
+        <v>394.85283230708342</v>
       </c>
       <c r="G15">
         <f t="shared" si="7"/>
-        <v>419.25297174020011</v>
+        <v>415.5810462832934</v>
       </c>
       <c r="H15">
         <f t="shared" si="7"/>
-        <v>438.89800644024933</v>
+        <v>434.57369639752272</v>
       </c>
       <c r="I15">
         <f t="shared" si="7"/>
-        <v>456.319735691419</v>
+        <v>451.49000167200313</v>
       </c>
       <c r="J15">
         <f t="shared" si="7"/>
-        <v>471.17198323354444</v>
+        <v>466.01287084198941</v>
       </c>
       <c r="K15">
         <f t="shared" si="7"/>
-        <v>483.146607814383</v>
+        <v>477.85851761303911</v>
       </c>
       <c r="L15">
         <f t="shared" si="7"/>
-        <v>495.42059800974255</v>
+        <v>490.00030555336502</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.35">
@@ -9177,39 +9177,39 @@
       </c>
       <c r="D16">
         <f t="shared" si="8"/>
-        <v>0.27357782105845291</v>
+        <v>0.27358937691429408</v>
       </c>
       <c r="E16">
         <f t="shared" si="8"/>
-        <v>0.27658737848306236</v>
+        <v>0.27660941320054411</v>
       </c>
       <c r="F16">
         <f t="shared" si="8"/>
-        <v>0.27960993808597051</v>
+        <v>0.27964144997645846</v>
       </c>
       <c r="G16">
         <f t="shared" si="8"/>
-        <v>0.28264493160682641</v>
+        <v>0.28268498940059683</v>
       </c>
       <c r="H16">
         <f t="shared" si="8"/>
-        <v>0.28089893287639017</v>
+        <v>0.28094433864890778</v>
       </c>
       <c r="I16">
         <f t="shared" si="8"/>
-        <v>0.27920328069061706</v>
+        <v>0.27925187272438934</v>
       </c>
       <c r="J16">
         <f t="shared" si="8"/>
-        <v>0.27755218766413764</v>
+        <v>0.27760216756097478</v>
       </c>
       <c r="K16">
         <f t="shared" si="8"/>
-        <v>0.27594103315873258</v>
+        <v>0.27599086297545433</v>
       </c>
       <c r="L16">
         <f t="shared" si="8"/>
-        <v>0.27436619023269732</v>
+        <v>0.27441450747919544</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.35">
@@ -9227,7 +9227,7 @@
       </c>
       <c r="B18">
         <f>M11/(M12-M3)</f>
-        <v>2310.1197200907486</v>
+        <v>2285.2375887273847</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.35">
@@ -9236,7 +9236,7 @@
       </c>
       <c r="B19">
         <f>B18*L13</f>
-        <v>1131.191667006289</v>
+        <v>1119.0076838945879</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.35">
@@ -9245,7 +9245,7 @@
       </c>
       <c r="B20">
         <f>SUM(C14:L14)</f>
-        <v>619.55430206091683</v>
+        <v>618.58465776243327</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.35">
@@ -9254,7 +9254,7 @@
       </c>
       <c r="B21">
         <f>B19+B20</f>
-        <v>1750.7459690672058</v>
+        <v>1737.5923416570213</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.35">
@@ -9299,7 +9299,7 @@
       </c>
       <c r="B26">
         <f>B21-B22-B24+B23+B25</f>
-        <v>1721.880969067206</v>
+        <v>1708.7273416570215</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.35">
@@ -9317,7 +9317,7 @@
       </c>
       <c r="B28">
         <f>B26-B27</f>
-        <v>1721.880969067206</v>
+        <v>1708.7273416570215</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.35">
@@ -9335,7 +9335,7 @@
       </c>
       <c r="B30">
         <f>B28/B29</f>
-        <v>126.29998915646284</v>
+        <v>125.33517043256788</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.35">
@@ -9344,7 +9344,7 @@
       </c>
       <c r="B31">
         <f>B19/B21</f>
-        <v>0.64611981806188923</v>
+        <v>0.64399897321570143</v>
       </c>
     </row>
   </sheetData>
@@ -9444,35 +9444,35 @@
       </c>
       <c r="D3">
         <f>'Scenario inputs'!E12</f>
-        <v>7.0000000000000007E-2</v>
+        <v>7.9772924907641762E-2</v>
       </c>
       <c r="E3">
         <f>'Scenario inputs'!E12</f>
-        <v>7.0000000000000007E-2</v>
+        <v>7.9772924907641762E-2</v>
       </c>
       <c r="F3">
         <f>'Scenario inputs'!E12</f>
-        <v>7.0000000000000007E-2</v>
+        <v>7.9772924907641762E-2</v>
       </c>
       <c r="G3">
         <f>'Scenario inputs'!E12</f>
-        <v>7.0000000000000007E-2</v>
+        <v>7.9772924907641762E-2</v>
       </c>
       <c r="H3">
         <f>G3-((G3-M3)/5)*1</f>
-        <v>6.2000000000000006E-2</v>
+        <v>6.9818339926113415E-2</v>
       </c>
       <c r="I3">
         <f>G3-((G3-M3)/5)*2</f>
-        <v>5.4000000000000006E-2</v>
+        <v>5.9863754944585054E-2</v>
       </c>
       <c r="J3">
         <f>G3-((G3-M3)/5)*3</f>
-        <v>4.5999999999999999E-2</v>
+        <v>4.9909169963056707E-2</v>
       </c>
       <c r="K3">
         <f>G3-((G3-M3)/5)*4</f>
-        <v>3.7999999999999999E-2</v>
+        <v>3.9954584981528353E-2</v>
       </c>
       <c r="L3">
         <f>G3-((G3-M3)/5)*5</f>
@@ -9497,43 +9497,43 @@
       </c>
       <c r="D4">
         <f t="shared" si="0"/>
-        <v>700.85</v>
+        <v>707.25126581450536</v>
       </c>
       <c r="E4">
         <f t="shared" si="0"/>
-        <v>749.90950000000009</v>
+        <v>763.6707679331605</v>
       </c>
       <c r="F4">
         <f t="shared" si="0"/>
-        <v>802.40316500000017</v>
+        <v>824.59101875765361</v>
       </c>
       <c r="G4">
         <f t="shared" si="0"/>
-        <v>858.57138655000028</v>
+        <v>890.37105617652378</v>
       </c>
       <c r="H4">
         <f t="shared" si="0"/>
-        <v>911.8028125161004</v>
+        <v>952.53528523702892</v>
       </c>
       <c r="I4">
         <f t="shared" si="0"/>
-        <v>961.04016439196982</v>
+        <v>1009.5576241285288</v>
       </c>
       <c r="J4">
         <f t="shared" si="0"/>
-        <v>1005.2480119540005</v>
+        <v>1059.9438071786592</v>
       </c>
       <c r="K4">
         <f t="shared" si="0"/>
-        <v>1043.4474364082525</v>
+        <v>1102.2934220982236</v>
       </c>
       <c r="L4">
         <f t="shared" si="0"/>
-        <v>1074.7508595005002</v>
+        <v>1135.3622247611704</v>
       </c>
       <c r="M4">
         <f t="shared" si="0"/>
-        <v>1106.9933852855152</v>
+        <v>1169.4230915040055</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.35">
@@ -9603,43 +9603,43 @@
       </c>
       <c r="D6">
         <f t="shared" si="1"/>
-        <v>128.14320000000001</v>
+        <v>129.3136054869392</v>
       </c>
       <c r="E6">
         <f t="shared" si="1"/>
-        <v>141.4027826666667</v>
+        <v>143.99760454686751</v>
       </c>
       <c r="F6">
         <f t="shared" si="1"/>
-        <v>155.89080522666671</v>
+        <v>160.20145919639788</v>
       </c>
       <c r="G6">
         <f t="shared" si="1"/>
-        <v>171.71427731000006</v>
+        <v>178.07421123530477</v>
       </c>
       <c r="H6">
         <f t="shared" si="1"/>
-        <v>182.36056250322008</v>
+        <v>190.50705704740579</v>
       </c>
       <c r="I6">
         <f t="shared" si="1"/>
-        <v>192.20803287839396</v>
+        <v>201.91152482570578</v>
       </c>
       <c r="J6">
         <f t="shared" si="1"/>
-        <v>201.04960239080012</v>
+        <v>211.98876143573185</v>
       </c>
       <c r="K6">
         <f t="shared" si="1"/>
-        <v>208.68948728165051</v>
+        <v>220.45868441964473</v>
       </c>
       <c r="L6">
         <f t="shared" si="1"/>
-        <v>214.95017190010003</v>
+        <v>227.07244495223409</v>
       </c>
       <c r="M6">
         <f t="shared" si="1"/>
-        <v>221.39867705710304</v>
+        <v>233.88461830080109</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.35">
@@ -9709,43 +9709,43 @@
       </c>
       <c r="D8">
         <f t="shared" si="2"/>
-        <v>99.310980000000015</v>
+        <v>100.21804425237788</v>
       </c>
       <c r="E8">
         <f t="shared" si="2"/>
-        <v>109.58715656666669</v>
+        <v>111.59814352382232</v>
       </c>
       <c r="F8">
         <f t="shared" si="2"/>
-        <v>120.8153740506667</v>
+        <v>124.15613087720835</v>
       </c>
       <c r="G8">
         <f t="shared" si="2"/>
-        <v>133.07856491525004</v>
+        <v>138.0075137073612</v>
       </c>
       <c r="H8">
         <f t="shared" si="2"/>
-        <v>140.41763312747946</v>
+        <v>146.69043392650246</v>
       </c>
       <c r="I8">
         <f t="shared" si="2"/>
-        <v>147.03914515197138</v>
+        <v>154.46231649166492</v>
       </c>
       <c r="J8">
         <f t="shared" si="2"/>
-        <v>152.7976978170081</v>
+        <v>161.1114586911562</v>
       </c>
       <c r="K8">
         <f t="shared" si="2"/>
-        <v>157.56056289764615</v>
+        <v>166.44630673683176</v>
       </c>
       <c r="L8">
         <f t="shared" si="2"/>
-        <v>161.21262892507502</v>
+        <v>170.30433371417558</v>
       </c>
       <c r="M8">
         <f>M6*(1-M7)</f>
-        <v>166.0490077928273</v>
+        <v>175.41346372560082</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.35">
@@ -9799,47 +9799,47 @@
       </c>
       <c r="C10">
         <f t="shared" ref="C10:L10" si="3">(D4-C4)/C9</f>
-        <v>22.925000000000011</v>
+        <v>26.12563290725268</v>
       </c>
       <c r="D10">
         <f t="shared" si="3"/>
-        <v>24.529750000000035</v>
+        <v>28.209751059327573</v>
       </c>
       <c r="E10">
         <f t="shared" si="3"/>
-        <v>26.246832500000039</v>
+        <v>30.460125412246555</v>
       </c>
       <c r="F10">
         <f t="shared" si="3"/>
-        <v>28.084110775000056</v>
+        <v>32.890018709435083</v>
       </c>
       <c r="G10">
         <f t="shared" si="3"/>
-        <v>26.615712983050059</v>
+        <v>31.082114530252568</v>
       </c>
       <c r="H10">
         <f t="shared" si="3"/>
-        <v>24.618675937934711</v>
+        <v>28.511169445749942</v>
       </c>
       <c r="I10">
         <f t="shared" si="3"/>
-        <v>22.10392378101534</v>
+        <v>25.193091525065199</v>
       </c>
       <c r="J10">
         <f t="shared" si="3"/>
-        <v>19.09971222712602</v>
+        <v>21.174807459782187</v>
       </c>
       <c r="K10">
         <f t="shared" si="3"/>
-        <v>15.651711546123806</v>
+        <v>16.534401331473418</v>
       </c>
       <c r="L10">
         <f t="shared" si="3"/>
-        <v>16.121262892507502</v>
+        <v>17.03043337141753</v>
       </c>
       <c r="M10">
         <f>IF(M3&gt;0,(M3/B17)*M8,0)</f>
-        <v>24.907351168924095</v>
+        <v>26.312019558840124</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.35">
@@ -9848,47 +9848,47 @@
       </c>
       <c r="C11">
         <f t="shared" ref="C11:M11" si="4">C8-C10</f>
-        <v>64.081666666666663</v>
+        <v>60.881033759413995</v>
       </c>
       <c r="D11">
         <f t="shared" si="4"/>
-        <v>74.781229999999979</v>
+        <v>72.008293193050307</v>
       </c>
       <c r="E11">
         <f t="shared" si="4"/>
-        <v>83.340324066666653</v>
+        <v>81.138018111575761</v>
       </c>
       <c r="F11">
         <f t="shared" si="4"/>
-        <v>92.731263275666649</v>
+        <v>91.266112167773272</v>
       </c>
       <c r="G11">
         <f t="shared" si="4"/>
-        <v>106.46285193219998</v>
+        <v>106.92539917710863</v>
       </c>
       <c r="H11">
         <f t="shared" si="4"/>
-        <v>115.79895718954475</v>
+        <v>118.17926448075252</v>
       </c>
       <c r="I11">
         <f t="shared" si="4"/>
-        <v>124.93522137095604</v>
+        <v>129.26922496659972</v>
       </c>
       <c r="J11">
         <f t="shared" si="4"/>
-        <v>133.69798558988208</v>
+        <v>139.93665123137401</v>
       </c>
       <c r="K11">
         <f t="shared" si="4"/>
-        <v>141.90885135152234</v>
+        <v>149.91190540535834</v>
       </c>
       <c r="L11">
         <f t="shared" si="4"/>
-        <v>145.09136603256752</v>
+        <v>153.27390034275805</v>
       </c>
       <c r="M11">
         <f t="shared" si="4"/>
-        <v>141.1416566239032</v>
+        <v>149.1014441667607</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.35">
@@ -9991,43 +9991,43 @@
       </c>
       <c r="C14">
         <f t="shared" ref="C14:L14" si="6">C11*C13</f>
-        <v>60.124842316563665</v>
+        <v>57.121837574774204</v>
       </c>
       <c r="D14">
         <f t="shared" si="6"/>
-        <v>65.831372219969126</v>
+        <v>63.390301979739633</v>
       </c>
       <c r="E14">
         <f t="shared" si="6"/>
-        <v>68.836002294205642</v>
+        <v>67.016979636507415</v>
       </c>
       <c r="F14">
         <f t="shared" si="6"/>
-        <v>71.863238314646836</v>
+        <v>70.727801359361237</v>
       </c>
       <c r="G14">
         <f t="shared" si="6"/>
-        <v>77.41031863539358</v>
+        <v>77.746641859527244</v>
       </c>
       <c r="H14">
         <f t="shared" si="6"/>
-        <v>78.999721357286916</v>
+        <v>80.623601375846448</v>
       </c>
       <c r="I14">
         <f t="shared" si="6"/>
-        <v>79.96978962816145</v>
+        <v>82.743942120853902</v>
       </c>
       <c r="J14">
         <f t="shared" si="6"/>
-        <v>80.294551863066147</v>
+        <v>84.041286413306153</v>
       </c>
       <c r="K14">
         <f t="shared" si="6"/>
-        <v>79.963326264795541</v>
+        <v>84.472916866980455</v>
       </c>
       <c r="L14">
         <f t="shared" si="6"/>
-        <v>76.708428926330299</v>
+        <v>81.0344571989542</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.35">
@@ -10040,43 +10040,43 @@
       </c>
       <c r="C15">
         <f t="shared" ref="C15:L15" si="7">B15+C10</f>
-        <v>336.36200000000002</v>
+        <v>339.56263290725269</v>
       </c>
       <c r="D15">
         <f t="shared" si="7"/>
-        <v>360.89175000000006</v>
+        <v>367.77238396658026</v>
       </c>
       <c r="E15">
         <f t="shared" si="7"/>
-        <v>387.1385825000001</v>
+        <v>398.23250937882682</v>
       </c>
       <c r="F15">
         <f t="shared" si="7"/>
-        <v>415.22269327500015</v>
+        <v>431.1225280882619</v>
       </c>
       <c r="G15">
         <f t="shared" si="7"/>
-        <v>441.83840625805021</v>
+        <v>462.20464261851447</v>
       </c>
       <c r="H15">
         <f t="shared" si="7"/>
-        <v>466.45708219598492</v>
+        <v>490.71581206426441</v>
       </c>
       <c r="I15">
         <f t="shared" si="7"/>
-        <v>488.56100597700026</v>
+        <v>515.90890358932961</v>
       </c>
       <c r="J15">
         <f t="shared" si="7"/>
-        <v>507.66071820412628</v>
+        <v>537.0837110491118</v>
       </c>
       <c r="K15">
         <f t="shared" si="7"/>
-        <v>523.31242975025009</v>
+        <v>553.61811238058522</v>
       </c>
       <c r="L15">
         <f t="shared" si="7"/>
-        <v>539.43369264275759</v>
+        <v>570.64854575200275</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.35">
@@ -10093,39 +10093,39 @@
       </c>
       <c r="D16">
         <f t="shared" si="8"/>
-        <v>0.29525029581224993</v>
+        <v>0.29513861226229565</v>
       </c>
       <c r="E16">
         <f t="shared" si="8"/>
-        <v>0.30365658557355957</v>
+        <v>0.30344351122884561</v>
       </c>
       <c r="F16">
         <f t="shared" si="8"/>
-        <v>0.31207267761969104</v>
+        <v>0.31176794448768191</v>
       </c>
       <c r="G16">
         <f t="shared" si="8"/>
-        <v>0.32049925755650521</v>
+        <v>0.32011204406165361</v>
       </c>
       <c r="H16">
         <f t="shared" si="8"/>
-        <v>0.31780314055693543</v>
+        <v>0.31737118237381051</v>
       </c>
       <c r="I16">
         <f t="shared" si="8"/>
-        <v>0.31522545323942996</v>
+        <v>0.31476938931700138</v>
       </c>
       <c r="J16">
         <f t="shared" si="8"/>
-        <v>0.31275049778369191</v>
+        <v>0.31228664124665517</v>
       </c>
       <c r="K16">
         <f t="shared" si="8"/>
-        <v>0.31036587478153532</v>
+        <v>0.30990756806179071</v>
       </c>
       <c r="L16">
         <f t="shared" si="8"/>
-        <v>0.30806191437496233</v>
+        <v>0.30762059604924874</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.35">
@@ -10143,7 +10143,7 @@
       </c>
       <c r="B18">
         <f>M11/(M12-M3)</f>
-        <v>3941.3879059295468</v>
+        <v>4163.6653759948513</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.35">
@@ -10152,7 +10152,7 @@
       </c>
       <c r="B19">
         <f>B18*L13</f>
-        <v>2083.7743989896067</v>
+        <v>2201.2903889527979</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.35">
@@ -10161,7 +10161,7 @@
       </c>
       <c r="B20">
         <f>SUM(C14:L14)</f>
-        <v>740.00159182041921</v>
+        <v>748.91976638585095</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.35">
@@ -10170,7 +10170,7 @@
       </c>
       <c r="B21">
         <f>B19+B20</f>
-        <v>2823.7759908100261</v>
+        <v>2950.2101553386487</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.35">
@@ -10215,7 +10215,7 @@
       </c>
       <c r="B26">
         <f>B21-B22-B24+B23+B25</f>
-        <v>2794.9109908100263</v>
+        <v>2921.345155338649</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.35">
@@ -10233,7 +10233,7 @@
       </c>
       <c r="B28">
         <f>B26-B27</f>
-        <v>2794.9109908100263</v>
+        <v>2921.345155338649</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.35">
@@ -10251,7 +10251,7 @@
       </c>
       <c r="B30">
         <f>B28/B29</f>
-        <v>205.00675376173893</v>
+        <v>214.28070120400736</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.35">
@@ -10260,7 +10260,7 @@
       </c>
       <c r="B31">
         <f>B19/B21</f>
-        <v>0.73793898870563623</v>
+        <v>0.74614697701090249</v>
       </c>
     </row>
   </sheetData>
@@ -10806,39 +10806,39 @@
       </c>
       <c r="D2">
         <f>'DCF Bear'!D8</f>
-        <v>83.750160000000008</v>
+        <v>83.143410149889149</v>
       </c>
       <c r="E2">
         <f>'DCF Bear'!E8</f>
-        <v>87.100166400000006</v>
+        <v>85.842698299403821</v>
       </c>
       <c r="F2">
         <f>'DCF Bear'!F8</f>
-        <v>90.584173056000026</v>
+        <v>88.629620050919854</v>
       </c>
       <c r="G2">
         <f>'DCF Bear'!G8</f>
-        <v>94.207539978240021</v>
+        <v>91.507020468681688</v>
       </c>
       <c r="H2">
         <f>'DCF Bear'!H8</f>
-        <v>97.216270196211724</v>
+        <v>93.88009508861164</v>
       </c>
       <c r="I2">
         <f>'DCF Bear'!I8</f>
-        <v>99.932201902165744</v>
+        <v>96.080088323050305</v>
       </c>
       <c r="J2">
         <f>'DCF Bear'!J8</f>
-        <v>102.32425492477253</v>
+        <v>98.091510643029068</v>
       </c>
       <c r="K2">
         <f>'DCF Bear'!K8</f>
-        <v>104.36424324517752</v>
+        <v>99.899884295183284</v>
       </c>
       <c r="L2">
         <f>'DCF Bear'!L8</f>
-        <v>106.02741843633572</v>
+        <v>101.49191432379178</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.35">
@@ -10851,39 +10851,39 @@
       </c>
       <c r="D3">
         <f>'DCF Bear'!C15</f>
-        <v>326.03700000000003</v>
+        <v>323.66361646382154</v>
       </c>
       <c r="E3">
         <f>'DCF Bear'!D15</f>
-        <v>339.14100000000002</v>
+        <v>334.22224462382752</v>
       </c>
       <c r="F3">
         <f>'DCF Bear'!E15</f>
-        <v>352.76916000000006</v>
+        <v>345.12366338883822</v>
       </c>
       <c r="G3">
         <f>'DCF Bear'!F15</f>
-        <v>366.94244640000005</v>
+        <v>356.37900160978944</v>
       </c>
       <c r="H3">
         <f>'DCF Bear'!G15</f>
-        <v>380.20864247040004</v>
+        <v>367.10736788100547</v>
       </c>
       <c r="I3">
         <f>'DCF Bear'!H15</f>
-        <v>392.42533502945287</v>
+        <v>377.23816026004408</v>
       </c>
       <c r="J3">
         <f>'DCF Bear'!I15</f>
-        <v>403.45700841027758</v>
+        <v>386.70295409685355</v>
       </c>
       <c r="K3">
         <f>'DCF Bear'!J15</f>
-        <v>413.17748861212425</v>
+        <v>395.43625507574177</v>
       </c>
       <c r="L3">
         <f>'DCF Bear'!K15</f>
-        <v>421.47229838436675</v>
+        <v>403.37624017725659</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.35">
@@ -10941,39 +10941,39 @@
       </c>
       <c r="D5">
         <f t="shared" si="0"/>
-        <v>25.111640237565513</v>
+        <v>24.928840268524343</v>
       </c>
       <c r="E5">
         <f t="shared" si="0"/>
-        <v>26.120921189338034</v>
+        <v>25.742074569405222</v>
       </c>
       <c r="F5">
         <f t="shared" si="0"/>
-        <v>27.170573379181462</v>
+        <v>26.581710887080806</v>
       </c>
       <c r="G5">
         <f t="shared" si="0"/>
-        <v>28.262211656618625</v>
+        <v>27.448606374883255</v>
       </c>
       <c r="H5">
         <f t="shared" si="0"/>
-        <v>29.754877038649397</v>
+        <v>28.729579949335164</v>
       </c>
       <c r="I5">
         <f t="shared" si="0"/>
-        <v>31.19696976515705</v>
+        <v>29.989622048772119</v>
       </c>
       <c r="J5">
         <f t="shared" si="0"/>
-        <v>32.573649335091154</v>
+        <v>31.220988013636106</v>
       </c>
       <c r="K5">
         <f t="shared" si="0"/>
-        <v>33.870169679564114</v>
+        <v>32.415834419866194</v>
       </c>
       <c r="L5">
         <f t="shared" si="0"/>
-        <v>35.072132985045521</v>
+        <v>33.566298883070687</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.35">
@@ -10986,39 +10986,39 @@
       </c>
       <c r="D6">
         <f t="shared" si="1"/>
-        <v>58.638519762434498</v>
+        <v>58.21456988136481</v>
       </c>
       <c r="E6">
         <f t="shared" si="1"/>
-        <v>60.979245210661972</v>
+        <v>60.100623729998603</v>
       </c>
       <c r="F6">
         <f t="shared" si="1"/>
-        <v>63.413599676818563</v>
+        <v>62.047909163839051</v>
       </c>
       <c r="G6">
         <f t="shared" si="1"/>
-        <v>65.945328321621389</v>
+        <v>64.058414093798433</v>
       </c>
       <c r="H6">
         <f t="shared" si="1"/>
-        <v>67.461393157562327</v>
+        <v>65.150515139276479</v>
       </c>
       <c r="I6">
         <f t="shared" si="1"/>
-        <v>68.735232137008694</v>
+        <v>66.090466274278185</v>
       </c>
       <c r="J6">
         <f t="shared" si="1"/>
-        <v>69.750605589681385</v>
+        <v>66.870522629392966</v>
       </c>
       <c r="K6">
         <f t="shared" si="1"/>
-        <v>70.494073565613405</v>
+        <v>67.484049875317083</v>
       </c>
       <c r="L6">
         <f t="shared" si="1"/>
-        <v>70.955285451290194</v>
+        <v>67.925615440721089</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.35">
@@ -11076,39 +11076,39 @@
       </c>
       <c r="D8">
         <f t="shared" si="2"/>
-        <v>50.551586897807717</v>
+        <v>50.186104628813965</v>
       </c>
       <c r="E8">
         <f t="shared" si="2"/>
-        <v>48.810104387683872</v>
+        <v>48.106822376890108</v>
       </c>
       <c r="F8">
         <f t="shared" si="2"/>
-        <v>47.1287581287216</v>
+        <v>46.113781874528136</v>
       </c>
       <c r="G8">
         <f t="shared" si="2"/>
-        <v>45.505461323981912</v>
+        <v>44.203399379622518</v>
       </c>
       <c r="H8">
         <f t="shared" si="2"/>
-        <v>43.172934000805306</v>
+        <v>41.694052828957126</v>
       </c>
       <c r="I8">
         <f t="shared" si="2"/>
-        <v>40.748711540235156</v>
+        <v>39.180799453795281</v>
       </c>
       <c r="J8">
         <f t="shared" si="2"/>
-        <v>38.261562181058558</v>
+        <v>36.681698144896203</v>
       </c>
       <c r="K8">
         <f t="shared" si="2"/>
-        <v>35.73963805067573</v>
+        <v>34.213592643255474</v>
       </c>
       <c r="L8">
         <f t="shared" si="2"/>
-        <v>33.209954431560526</v>
+        <v>31.79194585963058</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.35">
@@ -11126,7 +11126,7 @@
       </c>
       <c r="B10">
         <f>SUM(C8:L8)</f>
-        <v>435.48407925442342</v>
+        <v>424.52756550228247</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.35">
@@ -11135,7 +11135,7 @@
       </c>
       <c r="B11">
         <f>'DCF Bear'!M8</f>
-        <v>108.14796680506244</v>
+        <v>103.52175261026761</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.35">
@@ -11171,7 +11171,7 @@
       </c>
       <c r="B15">
         <f>'DCF Bear'!L15</f>
-        <v>429.93300435205407</v>
+        <v>411.47502498080172</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.35">
@@ -11180,7 +11180,7 @@
       </c>
       <c r="B16">
         <f>B11-B12*B15</f>
-        <v>72.371789910171429</v>
+        <v>69.281526499390935</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.35">
@@ -11189,7 +11189,7 @@
       </c>
       <c r="B17">
         <f>B11*(B13/B14)*(B14-B12)/(B12*(B12-B13))</f>
-        <v>6.8576185280839236E-14</v>
+        <v>6.5642721701787948E-14</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.35">
@@ -11198,7 +11198,7 @@
       </c>
       <c r="B18">
         <f>B16/B12+B17</f>
-        <v>869.71341733440045</v>
+        <v>832.57679884273</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.35">
@@ -11207,7 +11207,7 @@
       </c>
       <c r="B19">
         <f>B18*L7</f>
-        <v>407.06119036079548</v>
+        <v>389.67974513079537</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.35">
@@ -11216,7 +11216,7 @@
       </c>
       <c r="B20">
         <f>B9+B10+B19</f>
-        <v>1155.9822696152189</v>
+        <v>1127.644310633078</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.35">
@@ -11225,7 +11225,7 @@
       </c>
       <c r="B21">
         <f>'DCF Bear'!B21</f>
-        <v>1155.9822696152191</v>
+        <v>1127.6443106330778</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.35">
@@ -11293,39 +11293,39 @@
       </c>
       <c r="D2">
         <f>'DCF Base'!D8</f>
-        <v>91.022623999999993</v>
+        <v>90.859197521577528</v>
       </c>
       <c r="E2">
         <f>'DCF Base'!E8</f>
-        <v>97.675034893333347</v>
+        <v>97.324608676499821</v>
       </c>
       <c r="F2">
         <f>'DCF Base'!F8</f>
-        <v>104.79805364746667</v>
+        <v>104.23458785453093</v>
       </c>
       <c r="G2">
         <f>'DCF Base'!G8</f>
-        <v>112.42420452648003</v>
+        <v>111.61896871552352</v>
       </c>
       <c r="H2">
         <f>'DCF Base'!H8</f>
-        <v>117.76771236707758</v>
+        <v>116.75514220308099</v>
       </c>
       <c r="I2">
         <f>'DCF Base'!I8</f>
-        <v>122.54176328668919</v>
+        <v>121.35551855576844</v>
       </c>
       <c r="J2">
         <f>'DCF Base'!J8</f>
-        <v>126.65254091547442</v>
+        <v>125.3346030962562</v>
       </c>
       <c r="K2">
         <f>'DCF Base'!K8</f>
-        <v>130.01568384891328</v>
+        <v>128.6152943813496</v>
       </c>
       <c r="L2">
         <f>'DCF Base'!L8</f>
-        <v>132.5590941098834</v>
+        <v>131.13130975552056</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.35">
@@ -11338,39 +11338,39 @@
       </c>
       <c r="D3">
         <f>'DCF Base'!C15</f>
-        <v>332.71200000000005</v>
+        <v>332.1006047323267</v>
       </c>
       <c r="E3">
         <f>'DCF Base'!D15</f>
-        <v>353.14350000000007</v>
+        <v>351.84850562529004</v>
       </c>
       <c r="F3">
         <f>'DCF Base'!E15</f>
-        <v>374.80089000000009</v>
+        <v>372.74369684217379</v>
       </c>
       <c r="G3">
         <f>'DCF Base'!F15</f>
-        <v>397.75772340000015</v>
+        <v>394.85283230708342</v>
       </c>
       <c r="H3">
         <f>'DCF Base'!G15</f>
-        <v>419.25297174020011</v>
+        <v>415.5810462832934</v>
       </c>
       <c r="I3">
         <f>'DCF Base'!H15</f>
-        <v>438.89800644024933</v>
+        <v>434.57369639752272</v>
       </c>
       <c r="J3">
         <f>'DCF Base'!I15</f>
-        <v>456.319735691419</v>
+        <v>451.49000167200313</v>
       </c>
       <c r="K3">
         <f>'DCF Base'!J15</f>
-        <v>471.17198323354444</v>
+        <v>466.01287084198941</v>
       </c>
       <c r="L3">
         <f>'DCF Base'!K15</f>
-        <v>483.146607814383</v>
+        <v>477.85851761303911</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.35">
@@ -11428,39 +11428,39 @@
       </c>
       <c r="D5">
         <f t="shared" si="0"/>
-        <v>24.625252581829418</v>
+        <v>24.580000944095307</v>
       </c>
       <c r="E5">
         <f t="shared" si="0"/>
-        <v>26.137463888081214</v>
+        <v>26.041616537912653</v>
       </c>
       <c r="F5">
         <f t="shared" si="0"/>
-        <v>27.740407872708122</v>
+        <v>27.588147355741242</v>
       </c>
       <c r="G5">
         <f t="shared" si="0"/>
-        <v>29.439528496412642</v>
+        <v>29.224526702411282</v>
       </c>
       <c r="H5">
         <f t="shared" si="0"/>
-        <v>31.030471773741304</v>
+        <v>30.758698913616101</v>
       </c>
       <c r="I5">
         <f t="shared" si="0"/>
-        <v>32.484473858028963</v>
+        <v>32.164415588281301</v>
       </c>
       <c r="J5">
         <f t="shared" si="0"/>
-        <v>33.773920836864406</v>
+        <v>33.416454258769328</v>
       </c>
       <c r="K5">
         <f t="shared" si="0"/>
-        <v>34.873190917693158</v>
+        <v>34.491345821213052</v>
       </c>
       <c r="L5">
         <f t="shared" si="0"/>
-        <v>35.759477420361328</v>
+        <v>35.368086196469221</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.35">
@@ -11473,39 +11473,39 @@
       </c>
       <c r="D6">
         <f t="shared" si="1"/>
-        <v>66.397371418170579</v>
+        <v>66.279196577482224</v>
       </c>
       <c r="E6">
         <f t="shared" si="1"/>
-        <v>71.537571005252133</v>
+        <v>71.282992138587161</v>
       </c>
       <c r="F6">
         <f t="shared" si="1"/>
-        <v>77.057645774758555</v>
+        <v>76.646440498789687</v>
       </c>
       <c r="G6">
         <f t="shared" si="1"/>
-        <v>82.984676030067391</v>
+        <v>82.39444201311224</v>
       </c>
       <c r="H6">
         <f t="shared" si="1"/>
-        <v>86.737240593336281</v>
+        <v>85.996443289464892</v>
       </c>
       <c r="I6">
         <f t="shared" si="1"/>
-        <v>90.057289428660226</v>
+        <v>89.19110296748714</v>
       </c>
       <c r="J6">
         <f t="shared" si="1"/>
-        <v>92.878620078610012</v>
+        <v>91.918148837486882</v>
       </c>
       <c r="K6">
         <f t="shared" si="1"/>
-        <v>95.142492931220119</v>
+        <v>94.12394856013654</v>
       </c>
       <c r="L6">
         <f t="shared" si="1"/>
-        <v>96.799616689522082</v>
+        <v>95.76322355905134</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.35">
@@ -11563,39 +11563,39 @@
       </c>
       <c r="D8">
         <f t="shared" si="2"/>
-        <v>57.561384134042278</v>
+        <v>57.458935689856126</v>
       </c>
       <c r="E8">
         <f t="shared" si="2"/>
-        <v>57.743712566141014</v>
+        <v>57.538221539600059</v>
       </c>
       <c r="F8">
         <f t="shared" si="2"/>
-        <v>57.91304769630608</v>
+        <v>57.604004375286813</v>
       </c>
       <c r="G8">
         <f t="shared" si="2"/>
-        <v>58.069589736958775</v>
+        <v>57.656565925177382</v>
       </c>
       <c r="H8">
         <f t="shared" si="2"/>
-        <v>56.512774234589187</v>
+        <v>56.030115223293727</v>
       </c>
       <c r="I8">
         <f t="shared" si="2"/>
-        <v>54.632373414056623</v>
+        <v>54.106909873090345</v>
       </c>
       <c r="J8">
         <f t="shared" si="2"/>
-        <v>52.461067333165495</v>
+        <v>51.918559849640403</v>
       </c>
       <c r="K8">
         <f t="shared" si="2"/>
-        <v>50.036401123947961</v>
+        <v>49.500738318150766</v>
       </c>
       <c r="L8">
         <f t="shared" si="2"/>
-        <v>47.399673192819989</v>
+        <v>46.892184657600261</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.35">
@@ -11613,7 +11613,7 @@
       </c>
       <c r="B10">
         <f>SUM(C8:L8)</f>
-        <v>548.7089077071721</v>
+        <v>545.08511972684062</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.35">
@@ -11622,7 +11622,7 @@
       </c>
       <c r="B11">
         <f>'DCF Base'!M8</f>
-        <v>135.87307146263046</v>
+        <v>134.40959249940855</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.35">
@@ -11658,7 +11658,7 @@
       </c>
       <c r="B15">
         <f>'DCF Base'!L15</f>
-        <v>495.42059800974255</v>
+        <v>490.00030555336502</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.35">
@@ -11667,7 +11667,7 @@
       </c>
       <c r="B16">
         <f>B11-B12*B15</f>
-        <v>99.205150377034258</v>
+        <v>98.142847418301756</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.35">
@@ -11676,7 +11676,7 @@
       </c>
       <c r="B17">
         <f>B11*(B13/B14)*(B14-B12)/(B12*(B12-B13))</f>
-        <v>474.33747979681783</v>
+        <v>469.22842532651202</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.35">
@@ -11685,7 +11685,7 @@
       </c>
       <c r="B18">
         <f>B16/B12+B17</f>
-        <v>1814.6991220810062</v>
+        <v>1795.2372831740199</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.35">
@@ -11694,7 +11694,7 @@
       </c>
       <c r="B19">
         <f>B18*L7</f>
-        <v>888.60006136003346</v>
+        <v>879.07022193018042</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.35">
@@ -11703,7 +11703,7 @@
       </c>
       <c r="B20">
         <f>B9+B10+B19</f>
-        <v>1750.7459690672056</v>
+        <v>1737.5923416570211</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.35">
@@ -11712,7 +11712,7 @@
       </c>
       <c r="B21">
         <f>'DCF Base'!B21</f>
-        <v>1750.7459690672058</v>
+        <v>1737.5923416570213</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.35">
@@ -11780,39 +11780,39 @@
       </c>
       <c r="D2">
         <f>'DCF Bull'!D8</f>
-        <v>99.310980000000015</v>
+        <v>100.21804425237788</v>
       </c>
       <c r="E2">
         <f>'DCF Bull'!E8</f>
-        <v>109.58715656666669</v>
+        <v>111.59814352382232</v>
       </c>
       <c r="F2">
         <f>'DCF Bull'!F8</f>
-        <v>120.8153740506667</v>
+        <v>124.15613087720835</v>
       </c>
       <c r="G2">
         <f>'DCF Bull'!G8</f>
-        <v>133.07856491525004</v>
+        <v>138.0075137073612</v>
       </c>
       <c r="H2">
         <f>'DCF Bull'!H8</f>
-        <v>140.41763312747946</v>
+        <v>146.69043392650246</v>
       </c>
       <c r="I2">
         <f>'DCF Bull'!I8</f>
-        <v>147.03914515197138</v>
+        <v>154.46231649166492</v>
       </c>
       <c r="J2">
         <f>'DCF Bull'!J8</f>
-        <v>152.7976978170081</v>
+        <v>161.1114586911562</v>
       </c>
       <c r="K2">
         <f>'DCF Bull'!K8</f>
-        <v>157.56056289764615</v>
+        <v>166.44630673683176</v>
       </c>
       <c r="L2">
         <f>'DCF Bull'!L8</f>
-        <v>161.21262892507502</v>
+        <v>170.30433371417558</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.35">
@@ -11825,39 +11825,39 @@
       </c>
       <c r="D3">
         <f>'DCF Bull'!C15</f>
-        <v>336.36200000000002</v>
+        <v>339.56263290725269</v>
       </c>
       <c r="E3">
         <f>'DCF Bull'!D15</f>
-        <v>360.89175000000006</v>
+        <v>367.77238396658026</v>
       </c>
       <c r="F3">
         <f>'DCF Bull'!E15</f>
-        <v>387.1385825000001</v>
+        <v>398.23250937882682</v>
       </c>
       <c r="G3">
         <f>'DCF Bull'!F15</f>
-        <v>415.22269327500015</v>
+        <v>431.1225280882619</v>
       </c>
       <c r="H3">
         <f>'DCF Bull'!G15</f>
-        <v>441.83840625805021</v>
+        <v>462.20464261851447</v>
       </c>
       <c r="I3">
         <f>'DCF Bull'!H15</f>
-        <v>466.45708219598492</v>
+        <v>490.71581206426441</v>
       </c>
       <c r="J3">
         <f>'DCF Bull'!I15</f>
-        <v>488.56100597700026</v>
+        <v>515.90890358932961</v>
       </c>
       <c r="K3">
         <f>'DCF Bull'!J15</f>
-        <v>507.66071820412628</v>
+        <v>537.0837110491118</v>
       </c>
       <c r="L3">
         <f>'DCF Bull'!K15</f>
-        <v>523.31242975025009</v>
+        <v>553.61811238058522</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.35">
@@ -11915,39 +11915,39 @@
       </c>
       <c r="D5">
         <f t="shared" si="0"/>
-        <v>22.136030645068182</v>
+        <v>22.34666474796494</v>
       </c>
       <c r="E5">
         <f t="shared" si="0"/>
-        <v>23.750336951118992</v>
+        <v>24.20315244258865</v>
       </c>
       <c r="F5">
         <f t="shared" si="0"/>
-        <v>25.477644698593355</v>
+        <v>26.207737590667534</v>
       </c>
       <c r="G5">
         <f t="shared" si="0"/>
-        <v>27.325863988390928</v>
+        <v>28.37223435923509</v>
       </c>
       <c r="H5">
         <f t="shared" si="0"/>
-        <v>29.077447812464797</v>
+        <v>30.417752698866767</v>
       </c>
       <c r="I5">
         <f t="shared" si="0"/>
-        <v>30.697606347029122</v>
+        <v>32.294076779999152</v>
       </c>
       <c r="J5">
         <f t="shared" si="0"/>
-        <v>32.152268687581284</v>
+        <v>33.952037685341764</v>
       </c>
       <c r="K5">
         <f t="shared" si="0"/>
-        <v>33.409223442195795</v>
+        <v>35.345554749793628</v>
       </c>
       <c r="L5">
         <f t="shared" si="0"/>
-        <v>34.439264785845687</v>
+        <v>36.433686032671453</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.35">
@@ -11960,39 +11960,39 @@
       </c>
       <c r="D6">
         <f t="shared" si="1"/>
-        <v>77.17494935493184</v>
+        <v>77.871379504412943</v>
       </c>
       <c r="E6">
         <f t="shared" si="1"/>
-        <v>85.836819615547697</v>
+        <v>87.39499108123367</v>
       </c>
       <c r="F6">
         <f t="shared" si="1"/>
-        <v>95.337729352073353</v>
+        <v>97.948393286540821</v>
       </c>
       <c r="G6">
         <f t="shared" si="1"/>
-        <v>105.75270092685912</v>
+        <v>109.6352793481261</v>
       </c>
       <c r="H6">
         <f t="shared" si="1"/>
-        <v>111.34018531501466</v>
+        <v>116.2726812276357</v>
       </c>
       <c r="I6">
         <f t="shared" si="1"/>
-        <v>116.34153880494226</v>
+        <v>122.16823971166576</v>
       </c>
       <c r="J6">
         <f t="shared" si="1"/>
-        <v>120.64542912942682</v>
+        <v>127.15942100581444</v>
       </c>
       <c r="K6">
         <f t="shared" si="1"/>
-        <v>124.15133945545035</v>
+        <v>131.10075198703814</v>
       </c>
       <c r="L6">
         <f t="shared" si="1"/>
-        <v>126.77336413922933</v>
+        <v>133.87064768150412</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.35">
@@ -12050,39 +12050,39 @@
       </c>
       <c r="D8">
         <f t="shared" si="2"/>
-        <v>67.938609956559759</v>
+        <v>68.551690971617944</v>
       </c>
       <c r="E8">
         <f t="shared" si="2"/>
-        <v>70.898014594431189</v>
+        <v>72.185006165293416</v>
       </c>
       <c r="F8">
         <f t="shared" si="2"/>
-        <v>73.88315140750565</v>
+        <v>75.906317682339747</v>
       </c>
       <c r="G8">
         <f t="shared" si="2"/>
-        <v>76.893959975025453</v>
+        <v>79.717025741745516</v>
       </c>
       <c r="H8">
         <f t="shared" si="2"/>
-        <v>75.957882775726816</v>
+        <v>79.322902739207109</v>
       </c>
       <c r="I8">
         <f t="shared" si="2"/>
-        <v>74.469059094417162</v>
+        <v>78.198672254131125</v>
       </c>
       <c r="J8">
         <f t="shared" si="2"/>
-        <v>72.455621702409047</v>
+        <v>76.367708008321046</v>
       </c>
       <c r="K8">
         <f t="shared" si="2"/>
-        <v>69.957257553272839</v>
+        <v>73.873138319832591</v>
       </c>
       <c r="L8">
         <f t="shared" si="2"/>
-        <v>67.023875084635023</v>
+        <v>70.776141570639425</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.35">
@@ -12100,7 +12100,7 @@
       </c>
       <c r="B10">
         <f>SUM(C8:L8)</f>
-        <v>711.75806820733828</v>
+        <v>737.17923951648334</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.35">
@@ -12109,7 +12109,7 @@
       </c>
       <c r="B11">
         <f>'DCF Bull'!M8</f>
-        <v>166.0490077928273</v>
+        <v>175.41346372560082</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.35">
@@ -12145,7 +12145,7 @@
       </c>
       <c r="B15">
         <f>'DCF Bull'!L15</f>
-        <v>539.43369264275759</v>
+        <v>570.64854575200275</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.35">
@@ -12154,7 +12154,7 @@
       </c>
       <c r="B16">
         <f>B11-B12*B15</f>
-        <v>130.54880042302221</v>
+        <v>137.85900247156522</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.35">
@@ -12163,7 +12163,7 @@
       </c>
       <c r="B17">
         <f>B11*(B13/B14)*(B14-B12)/(B12*(B12-B13))</f>
-        <v>1418.2356183872137</v>
+        <v>1498.218059277478</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.35">
@@ -12172,7 +12172,7 @@
       </c>
       <c r="B18">
         <f>B16/B12+B17</f>
-        <v>3401.9542132867891</v>
+        <v>3593.0168302428492</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.35">
@@ -12181,7 +12181,7 @@
       </c>
       <c r="B19">
         <f>B18*L7</f>
-        <v>1798.5809226026877</v>
+        <v>1899.5939158221661</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.35">
@@ -12190,7 +12190,7 @@
       </c>
       <c r="B20">
         <f>B9+B10+B19</f>
-        <v>2823.7759908100261</v>
+        <v>2950.2101553386492</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.35">
@@ -12199,7 +12199,7 @@
       </c>
       <c r="B21">
         <f>'DCF Bull'!B21</f>
-        <v>2823.7759908100261</v>
+        <v>2950.2101553386487</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Check the bases of the other methods
Each Damodaran premium is now paired with the risk-free rate it is
measured against; Bear uses the smoothed ERP with the T-bond rate
instead of the adjusted-risk-free premium with the T-bond rate, which
implied an unsupported market return. The report adds a Base beta
sensitivity. Comps show each peer's trailing period and filing date and
the range without Quaker Houghton (one estimated amortization quarter).
Precedents record the EV basis of each deal; Waterpik becomes context
because its cash price has no disclosed bridge to enterprise value.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/models/excel/wd40_valuation.xlsx
+++ b/models/excel/wd40_valuation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\sunesis-ai\models\out\valuation_book\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{93ED054F-6A65-4899-B0FE-F88E6D8A444F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{709FA7D1-AD82-4C29-890F-0A990A72DB47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4310" yWindow="4570" windowWidth="7500" windowHeight="6000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1397,7 +1397,7 @@
         <v>0.09</v>
       </c>
       <c r="C21">
-        <v>7.7020829652970399E-2</v>
+        <v>8.6579251013891551E-2</v>
       </c>
       <c r="D21">
         <v>7.4013719318297547E-2</v>
@@ -1414,7 +1414,7 @@
         <v>0.08</v>
       </c>
       <c r="C22">
-        <v>8.3213376346411877E-2</v>
+        <v>9.4478057603863227E-2</v>
       </c>
       <c r="D22">
         <v>7.4013719318297547E-2</v>
@@ -1692,43 +1692,43 @@
       </c>
       <c r="C6">
         <f>1/(1+B8)^C2</f>
-        <v>0.92762389152796965</v>
+        <v>0.91923080407695568</v>
       </c>
       <c r="D6">
         <f>1/(1+B8)^D2</f>
-        <v>0.86048608413349448</v>
+        <v>0.84498527116396649</v>
       </c>
       <c r="E6">
         <f>1/(1+B8)^E2</f>
-        <v>0.79820744996957604</v>
+        <v>0.77673649024523739</v>
       </c>
       <c r="F6">
         <f>1/(1+B8)^F2</f>
-        <v>0.74043630098739543</v>
+        <v>0.71400010848404205</v>
       </c>
       <c r="G6">
         <f>1/(1+B8)^G2</f>
-        <v>0.68684640295050281</v>
+        <v>0.65633089383281962</v>
       </c>
       <c r="H6">
         <f>1/(1+B8)^H2</f>
-        <v>0.63713513318693338</v>
+        <v>0.60331957527848978</v>
       </c>
       <c r="I6">
         <f>1/(1+B8)^I2</f>
-        <v>0.59102177167605441</v>
+        <v>0.55458993829861358</v>
       </c>
       <c r="J6">
         <f>1/(1+B8)^J2</f>
-        <v>0.54824591581989679</v>
+        <v>0.5097961549152239</v>
       </c>
       <c r="K6">
         <f>1/(1+B8)^K2</f>
-        <v>0.50856600994716838</v>
+        <v>0.46862032939806147</v>
       </c>
       <c r="L6">
         <f>1/(1+B8)^L2</f>
-        <v>0.47175798124604446</v>
+        <v>0.43077024219938792</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.35">
@@ -1737,43 +1737,43 @@
       </c>
       <c r="C7">
         <f t="shared" ref="C7:L7" si="2">C5*C6</f>
-        <v>3.627380465430972</v>
+        <v>3.594560136262527</v>
       </c>
       <c r="D7">
         <f t="shared" si="2"/>
-        <v>3.4994385747314416</v>
+        <v>3.4363996205339578</v>
       </c>
       <c r="E7">
         <f t="shared" si="2"/>
-        <v>3.3760093420096906</v>
+        <v>3.2851981617657029</v>
       </c>
       <c r="F7">
         <f t="shared" si="2"/>
-        <v>3.2569336006166028</v>
+        <v>3.1406495617037051</v>
       </c>
       <c r="G7">
         <f t="shared" si="2"/>
-        <v>3.1420577978942621</v>
+        <v>3.0024610948059887</v>
       </c>
       <c r="H7">
         <f t="shared" si="2"/>
-        <v>3.0312337971640182</v>
+        <v>2.8703529154438177</v>
       </c>
       <c r="I7">
         <f t="shared" si="2"/>
-        <v>2.9243186866986468</v>
+        <v>2.744057491185977</v>
       </c>
       <c r="J7">
         <f t="shared" si="2"/>
-        <v>2.8211745954322947</v>
+        <v>2.6233190610185311</v>
       </c>
       <c r="K7">
         <f t="shared" si="2"/>
-        <v>2.7216685151705406</v>
+        <v>2.5078931174028871</v>
       </c>
       <c r="L7">
         <f t="shared" si="2"/>
-        <v>2.6256721290713143</v>
+        <v>2.3975459111232924</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.35">
@@ -1781,7 +1781,7 @@
         <v>93</v>
       </c>
       <c r="B8">
-        <v>7.8023118133377742E-2</v>
+        <v>8.7866067547800103E-2</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.35">
@@ -1805,7 +1805,7 @@
         <v>95</v>
       </c>
       <c r="B11">
-        <v>7.8023118133377742E-2</v>
+        <v>8.7866067547800103E-2</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.35">
@@ -1814,7 +1814,7 @@
       </c>
       <c r="B12">
         <f>1-B10/B11</f>
-        <v>0.74366571756577693</v>
+        <v>0.7723808455508745</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.35">
@@ -1823,7 +1823,7 @@
       </c>
       <c r="B13">
         <f>L3*(1+B10)*B12</f>
-        <v>6.5348302492577224</v>
+        <v>6.787159330101395</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.35">
@@ -1832,7 +1832,7 @@
       </c>
       <c r="B14">
         <f>B13/(B8-B10)</f>
-        <v>112.62459618657702</v>
+        <v>100.00814214439337</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.35">
@@ -1841,7 +1841,7 @@
       </c>
       <c r="B15">
         <f>B14*L6</f>
-        <v>53.131552135630535</v>
+        <v>43.08053161345115</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.35">
@@ -1850,7 +1850,7 @@
       </c>
       <c r="B16">
         <f>SUM(C7:L7)</f>
-        <v>31.025887504219785</v>
+        <v>29.602437071246385</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.35">
@@ -1859,7 +1859,7 @@
       </c>
       <c r="B17">
         <f>B16+B15</f>
-        <v>84.157439639850324</v>
+        <v>72.682968684697528</v>
       </c>
     </row>
   </sheetData>
@@ -7266,7 +7266,7 @@
         <v>3.7735849056603772E-2</v>
       </c>
       <c r="I4">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.35">
@@ -7455,13 +7455,13 @@
         <v>203</v>
       </c>
       <c r="B6">
-        <v>10.68376068376068</v>
+        <v>10.102725875596541</v>
       </c>
       <c r="C6">
-        <v>11.83333333333333</v>
+        <v>11.25854700854701</v>
       </c>
       <c r="D6">
-        <v>12.5</v>
+        <v>14.24537037037037</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
@@ -7470,15 +7470,15 @@
       </c>
       <c r="B7">
         <f>B2*B6</f>
-        <v>1196.4102564102559</v>
+        <v>1131.3436544528029</v>
       </c>
       <c r="C7">
         <f>C2*C6</f>
-        <v>1325.1439999999996</v>
+        <v>1260.7771282051283</v>
       </c>
       <c r="D7">
         <f>D2*D6</f>
-        <v>1399.8</v>
+        <v>1595.2535555555555</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
@@ -7487,15 +7487,15 @@
       </c>
       <c r="B8">
         <f>B7-B3+B4</f>
-        <v>1167.5452564102561</v>
+        <v>1102.4786544528029</v>
       </c>
       <c r="C8">
         <f>C7-C3+C4</f>
-        <v>1296.2789999999995</v>
+        <v>1231.9121282051283</v>
       </c>
       <c r="D8">
         <f>D7-D3+D4</f>
-        <v>1370.9349999999999</v>
+        <v>1566.3885555555557</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
@@ -7504,15 +7504,15 @@
       </c>
       <c r="B9">
         <f>B8/B5</f>
-        <v>85.639458170084168</v>
+        <v>80.866822157894475</v>
       </c>
       <c r="C9">
         <f>C8/C5</f>
-        <v>95.082079763296548</v>
+        <v>90.360768966690387</v>
       </c>
       <c r="D9">
         <f>D8/D5</f>
-        <v>100.55809823370971</v>
+        <v>114.89461881249967</v>
       </c>
     </row>
   </sheetData>
@@ -8007,7 +8007,7 @@
       </c>
       <c r="M10">
         <f>IF(M3&gt;0,(M3/B17)*M8,0)</f>
-        <v>24.881036476470626</v>
+        <v>21.914454051187981</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.35">
@@ -8056,7 +8056,7 @@
       </c>
       <c r="M11">
         <f t="shared" si="4"/>
-        <v>78.640716133796985</v>
+        <v>81.607298559079624</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.35">
@@ -8065,47 +8065,47 @@
       </c>
       <c r="C12">
         <f>'Scenario inputs'!C21</f>
-        <v>7.7020829652970399E-2</v>
+        <v>8.6579251013891551E-2</v>
       </c>
       <c r="D12">
         <f>'Scenario inputs'!C21</f>
-        <v>7.7020829652970399E-2</v>
+        <v>8.6579251013891551E-2</v>
       </c>
       <c r="E12">
         <f>'Scenario inputs'!C21</f>
-        <v>7.7020829652970399E-2</v>
+        <v>8.6579251013891551E-2</v>
       </c>
       <c r="F12">
         <f>'Scenario inputs'!C21</f>
-        <v>7.7020829652970399E-2</v>
+        <v>8.6579251013891551E-2</v>
       </c>
       <c r="G12">
         <f>'Scenario inputs'!C21</f>
-        <v>7.7020829652970399E-2</v>
+        <v>8.6579251013891551E-2</v>
       </c>
       <c r="H12">
         <f>G12-(G12-M12)/5</f>
-        <v>7.8259338991658697E-2</v>
+        <v>8.8159012331885889E-2</v>
       </c>
       <c r="I12">
         <f>H12-(G12-M12)/5</f>
-        <v>7.9497848330346996E-2</v>
+        <v>8.9738773649880227E-2</v>
       </c>
       <c r="J12">
         <f>I12-(G12-M12)/5</f>
-        <v>8.0736357669035294E-2</v>
+        <v>9.1318534967874565E-2</v>
       </c>
       <c r="K12">
         <f>J12-(G12-M12)/5</f>
-        <v>8.1974867007723592E-2</v>
+        <v>9.2898296285868903E-2</v>
       </c>
       <c r="L12">
         <f>K12-(G12-M12)/5</f>
-        <v>8.3213376346411891E-2</v>
+        <v>9.4478057603863241E-2</v>
       </c>
       <c r="M12">
         <f>'Scenario inputs'!C22</f>
-        <v>8.3213376346411877E-2</v>
+        <v>9.4478057603863227E-2</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.35">
@@ -8114,43 +8114,43 @@
       </c>
       <c r="C13">
         <f>1/(1+C12)</f>
-        <v>0.92848714942886712</v>
+        <v>0.92031943281347939</v>
       </c>
       <c r="D13">
         <f t="shared" ref="D13:L13" si="5">C13*(1/(1+D12))</f>
-        <v>0.86208838665454346</v>
+        <v>0.84698785841412438</v>
       </c>
       <c r="E13">
         <f t="shared" si="5"/>
-        <v>0.80043798868060811</v>
+        <v>0.7794993854555905</v>
       </c>
       <c r="F13">
         <f t="shared" si="5"/>
-        <v>0.74319638640463359</v>
+        <v>0.71738843230094484</v>
       </c>
       <c r="G13">
         <f t="shared" si="5"/>
-        <v>0.69004829427867309</v>
+        <v>0.66022651512215669</v>
       </c>
       <c r="H13">
         <f t="shared" si="5"/>
-        <v>0.63996505230733858</v>
+        <v>0.60673716583692572</v>
       </c>
       <c r="I13">
         <f t="shared" si="5"/>
-        <v>0.59283587577054353</v>
+        <v>0.55677303635326358</v>
       </c>
       <c r="J13">
         <f t="shared" si="5"/>
-        <v>0.54854810015755351</v>
+        <v>0.51018379924212809</v>
       </c>
       <c r="K13">
         <f t="shared" si="5"/>
-        <v>0.50698783944455317</v>
+        <v>0.46681727016681113</v>
       </c>
       <c r="L13">
         <f t="shared" si="5"/>
-        <v>0.46804060078595117</v>
+        <v>0.42652044682267309</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.35">
@@ -8159,43 +8159,43 @@
       </c>
       <c r="C14">
         <f t="shared" ref="C14:L14" si="6">C11*C13</f>
-        <v>65.274859687561261</v>
+        <v>64.700649741451457</v>
       </c>
       <c r="D14">
         <f t="shared" si="6"/>
-        <v>62.574497601330144</v>
+        <v>61.478429051067252</v>
       </c>
       <c r="E14">
         <f t="shared" si="6"/>
-        <v>59.985847059660848</v>
+        <v>58.416681342315059</v>
       </c>
       <c r="F14">
         <f t="shared" si="6"/>
-        <v>57.504286656686389</v>
+        <v>55.507414742412685</v>
       </c>
       <c r="G14">
         <f t="shared" si="6"/>
-        <v>55.741172543087956</v>
+        <v>53.332209357050523</v>
       </c>
       <c r="H14">
         <f t="shared" si="6"/>
-        <v>53.59662688923504</v>
+        <v>50.813814566825101</v>
       </c>
       <c r="I14">
         <f t="shared" si="6"/>
-        <v>51.34865396187412</v>
+        <v>48.225060505736401</v>
       </c>
       <c r="J14">
         <f t="shared" si="6"/>
-        <v>49.017276144744798</v>
+        <v>45.58911089992602</v>
       </c>
       <c r="K14">
         <f t="shared" si="6"/>
-        <v>46.622550607736883</v>
+        <v>42.928469106403448</v>
       </c>
       <c r="L14">
         <f t="shared" si="6"/>
-        <v>43.711776449936394</v>
+        <v>39.834079333143379</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.35">
@@ -8302,7 +8302,7 @@
       </c>
       <c r="B17">
         <f>IF('Scenario inputs'!C23=1,'Scenario inputs'!C24,L12)</f>
-        <v>8.3213376346411891E-2</v>
+        <v>9.4478057603863241E-2</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.35">
@@ -8311,7 +8311,7 @@
       </c>
       <c r="B18">
         <f>M11/(M12-M3)</f>
-        <v>1244.0518238235315</v>
+        <v>1095.7227025593993</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.35">
@@ -8320,7 +8320,7 @@
       </c>
       <c r="B19">
         <f>B18*L13</f>
-        <v>582.26676303122395</v>
+        <v>467.34813668938193</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.35">
@@ -8329,7 +8329,7 @@
       </c>
       <c r="B20">
         <f>SUM(C14:L14)</f>
-        <v>545.37754760185385</v>
+        <v>520.82591864633127</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.35">
@@ -8338,7 +8338,7 @@
       </c>
       <c r="B21">
         <f>B19+B20</f>
-        <v>1127.6443106330778</v>
+        <v>988.17405533571321</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.35">
@@ -8383,7 +8383,7 @@
       </c>
       <c r="B26">
         <f>B21-B22-B24+B23+B25</f>
-        <v>1098.7793106330778</v>
+        <v>959.3090553357132</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.35">
@@ -8401,7 +8401,7 @@
       </c>
       <c r="B28">
         <f>B26-B27</f>
-        <v>1098.7793106330778</v>
+        <v>959.3090553357132</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.35">
@@ -8419,7 +8419,7 @@
       </c>
       <c r="B30">
         <f>B28/B29</f>
-        <v>80.595475245587053</v>
+        <v>70.365330393443827</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.35">
@@ -8428,7 +8428,7 @@
       </c>
       <c r="B31">
         <f>B19/B21</f>
-        <v>0.51635676031951061</v>
+        <v>0.47294111211066897</v>
       </c>
     </row>
   </sheetData>
@@ -10892,43 +10892,43 @@
       </c>
       <c r="C4">
         <f>'DCF Bear'!C12</f>
-        <v>7.7020829652970399E-2</v>
+        <v>8.6579251013891551E-2</v>
       </c>
       <c r="D4">
         <f>'DCF Bear'!D12</f>
-        <v>7.7020829652970399E-2</v>
+        <v>8.6579251013891551E-2</v>
       </c>
       <c r="E4">
         <f>'DCF Bear'!E12</f>
-        <v>7.7020829652970399E-2</v>
+        <v>8.6579251013891551E-2</v>
       </c>
       <c r="F4">
         <f>'DCF Bear'!F12</f>
-        <v>7.7020829652970399E-2</v>
+        <v>8.6579251013891551E-2</v>
       </c>
       <c r="G4">
         <f>'DCF Bear'!G12</f>
-        <v>7.7020829652970399E-2</v>
+        <v>8.6579251013891551E-2</v>
       </c>
       <c r="H4">
         <f>'DCF Bear'!H12</f>
-        <v>7.8259338991658697E-2</v>
+        <v>8.8159012331885889E-2</v>
       </c>
       <c r="I4">
         <f>'DCF Bear'!I12</f>
-        <v>7.9497848330346996E-2</v>
+        <v>8.9738773649880227E-2</v>
       </c>
       <c r="J4">
         <f>'DCF Bear'!J12</f>
-        <v>8.0736357669035294E-2</v>
+        <v>9.1318534967874565E-2</v>
       </c>
       <c r="K4">
         <f>'DCF Bear'!K12</f>
-        <v>8.1974867007723592E-2</v>
+        <v>9.2898296285868903E-2</v>
       </c>
       <c r="L4">
         <f>'DCF Bear'!L12</f>
-        <v>8.3213376346411891E-2</v>
+        <v>9.4478057603863241E-2</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.35">
@@ -10937,43 +10937,43 @@
       </c>
       <c r="C5">
         <f t="shared" ref="C5:L5" si="0">C4*C3</f>
-        <v>24.141177783938083</v>
+        <v>27.137140700041126</v>
       </c>
       <c r="D5">
         <f t="shared" si="0"/>
-        <v>24.928840268524343</v>
+        <v>28.022553493885127</v>
       </c>
       <c r="E5">
         <f t="shared" si="0"/>
-        <v>25.742074569405222</v>
+        <v>28.936711611712628</v>
       </c>
       <c r="F5">
         <f t="shared" si="0"/>
-        <v>26.581710887080806</v>
+        <v>29.880548283376037</v>
       </c>
       <c r="G5">
         <f t="shared" si="0"/>
-        <v>27.448606374883255</v>
+        <v>30.855027036454022</v>
       </c>
       <c r="H5">
         <f t="shared" si="0"/>
-        <v>28.729579949335164</v>
+        <v>32.36382297214773</v>
       </c>
       <c r="I5">
         <f t="shared" si="0"/>
-        <v>29.989622048772119</v>
+        <v>33.852889875673341</v>
       </c>
       <c r="J5">
         <f t="shared" si="0"/>
-        <v>31.220988013636106</v>
+        <v>35.313147235873913</v>
       </c>
       <c r="K5">
         <f t="shared" si="0"/>
-        <v>32.415834419866194</v>
+        <v>36.73535438620069</v>
       </c>
       <c r="L5">
         <f t="shared" si="0"/>
-        <v>33.566298883070687</v>
+        <v>38.110203655496619</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.35">
@@ -10982,43 +10982,43 @@
       </c>
       <c r="C6">
         <f t="shared" ref="C6:L6" si="1">C2-C5</f>
-        <v>56.387822216061913</v>
+        <v>53.391859299958867</v>
       </c>
       <c r="D6">
         <f t="shared" si="1"/>
-        <v>58.21456988136481</v>
+        <v>55.120856656004023</v>
       </c>
       <c r="E6">
         <f t="shared" si="1"/>
-        <v>60.100623729998603</v>
+        <v>56.905986687691197</v>
       </c>
       <c r="F6">
         <f t="shared" si="1"/>
-        <v>62.047909163839051</v>
+        <v>58.749071767543818</v>
       </c>
       <c r="G6">
         <f t="shared" si="1"/>
-        <v>64.058414093798433</v>
+        <v>60.65199343222767</v>
       </c>
       <c r="H6">
         <f t="shared" si="1"/>
-        <v>65.150515139276479</v>
+        <v>61.516272116463909</v>
       </c>
       <c r="I6">
         <f t="shared" si="1"/>
-        <v>66.090466274278185</v>
+        <v>62.227198447376963</v>
       </c>
       <c r="J6">
         <f t="shared" si="1"/>
-        <v>66.870522629392966</v>
+        <v>62.778363407155155</v>
       </c>
       <c r="K6">
         <f t="shared" si="1"/>
-        <v>67.484049875317083</v>
+        <v>63.164529908982594</v>
       </c>
       <c r="L6">
         <f t="shared" si="1"/>
-        <v>67.925615440721089</v>
+        <v>63.381710668295156</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.35">
@@ -11027,43 +11027,43 @@
       </c>
       <c r="C7">
         <f>'DCF Bear'!C13</f>
-        <v>0.92848714942886712</v>
+        <v>0.92031943281347939</v>
       </c>
       <c r="D7">
         <f>'DCF Bear'!D13</f>
-        <v>0.86208838665454346</v>
+        <v>0.84698785841412438</v>
       </c>
       <c r="E7">
         <f>'DCF Bear'!E13</f>
-        <v>0.80043798868060811</v>
+        <v>0.7794993854555905</v>
       </c>
       <c r="F7">
         <f>'DCF Bear'!F13</f>
-        <v>0.74319638640463359</v>
+        <v>0.71738843230094484</v>
       </c>
       <c r="G7">
         <f>'DCF Bear'!G13</f>
-        <v>0.69004829427867309</v>
+        <v>0.66022651512215669</v>
       </c>
       <c r="H7">
         <f>'DCF Bear'!H13</f>
-        <v>0.63996505230733858</v>
+        <v>0.60673716583692572</v>
       </c>
       <c r="I7">
         <f>'DCF Bear'!I13</f>
-        <v>0.59283587577054353</v>
+        <v>0.55677303635326358</v>
       </c>
       <c r="J7">
         <f>'DCF Bear'!J13</f>
-        <v>0.54854810015755351</v>
+        <v>0.51018379924212809</v>
       </c>
       <c r="K7">
         <f>'DCF Bear'!K13</f>
-        <v>0.50698783944455317</v>
+        <v>0.46681727016681113</v>
       </c>
       <c r="L7">
         <f>'DCF Bear'!L13</f>
-        <v>0.46804060078595117</v>
+        <v>0.42652044682267309</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.35">
@@ -11072,43 +11072,43 @@
       </c>
       <c r="C8">
         <f t="shared" ref="C8:L8" si="2">C6*C7</f>
-        <v>52.355368311893073</v>
+        <v>49.137565667795236</v>
       </c>
       <c r="D8">
         <f t="shared" si="2"/>
-        <v>50.186104628813965</v>
+        <v>46.686696333020784</v>
       </c>
       <c r="E8">
         <f t="shared" si="2"/>
-        <v>48.106822376890108</v>
+        <v>44.358181651799299</v>
       </c>
       <c r="F8">
         <f t="shared" si="2"/>
-        <v>46.113781874528136</v>
+        <v>42.145904494453958</v>
       </c>
       <c r="G8">
         <f t="shared" si="2"/>
-        <v>44.203399379622518</v>
+        <v>40.044054258971613</v>
       </c>
       <c r="H8">
         <f t="shared" si="2"/>
-        <v>41.694052828957126</v>
+        <v>37.32420859679641</v>
       </c>
       <c r="I8">
         <f t="shared" si="2"/>
-        <v>39.180799453795281</v>
+        <v>34.646426223303159</v>
       </c>
       <c r="J8">
         <f t="shared" si="2"/>
-        <v>36.681698144896203</v>
+        <v>32.028503953265407</v>
       </c>
       <c r="K8">
         <f t="shared" si="2"/>
-        <v>34.213592643255474</v>
+        <v>29.48629342348115</v>
       </c>
       <c r="L8">
         <f t="shared" si="2"/>
-        <v>31.79194585963058</v>
+        <v>27.033595554626636</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.35">
@@ -11126,7 +11126,7 @@
       </c>
       <c r="B10">
         <f>SUM(C8:L8)</f>
-        <v>424.52756550228247</v>
+        <v>382.89143015751358</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.35">
@@ -11144,7 +11144,7 @@
       </c>
       <c r="B12">
         <f>'DCF Bear'!M12</f>
-        <v>8.3213376346411877E-2</v>
+        <v>9.4478057603863227E-2</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.35">
@@ -11162,7 +11162,7 @@
       </c>
       <c r="B14">
         <f>'DCF Bear'!B17</f>
-        <v>8.3213376346411891E-2</v>
+        <v>9.4478057603863241E-2</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.35">
@@ -11180,7 +11180,7 @@
       </c>
       <c r="B16">
         <f>B11-B12*B15</f>
-        <v>69.281526499390935</v>
+        <v>64.646391497580368</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.35">
@@ -11189,7 +11189,7 @@
       </c>
       <c r="B17">
         <f>B11*(B13/B14)*(B14-B12)/(B12*(B12-B13))</f>
-        <v>6.5642721701787948E-14</v>
+        <v>4.3220680539997398E-14</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.35">
@@ -11198,7 +11198,7 @@
       </c>
       <c r="B18">
         <f>B16/B12+B17</f>
-        <v>832.57679884273</v>
+        <v>684.24767757859752</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.35">
@@ -11207,7 +11207,7 @@
       </c>
       <c r="B19">
         <f>B18*L7</f>
-        <v>389.67974513079537</v>
+        <v>291.84562517819978</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.35">
@@ -11216,7 +11216,7 @@
       </c>
       <c r="B20">
         <f>B9+B10+B19</f>
-        <v>1127.644310633078</v>
+        <v>988.17405533571332</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.35">
@@ -11225,7 +11225,7 @@
       </c>
       <c r="B21">
         <f>'DCF Bear'!B21</f>
-        <v>1127.6443106330778</v>
+        <v>988.17405533571321</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Model buyout repayments the way a lender would
Mandatory amortization of 1% of the original debt is paid first, then a
sweep of cash above the minimum, capped by the debt outstanding. A year
that cannot meet the mandatory payment makes the case infeasible instead
of turning a negative cash flow into new borrowing. A 2% exit fee comes
off the exit value; sources equal uses and balances stay non-negative
(asserted in Python and visible in the sheet). The solver reports
boundary found, no solution, infeasible or search ceiling reached.
Measured alone: LBO Base -0.99.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/models/excel/wd40_valuation.xlsx
+++ b/models/excel/wd40_valuation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\sunesis-ai\models\out\valuation_book\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{709FA7D1-AD82-4C29-890F-0A990A72DB47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E764D963-2E8B-43BE-9793-6A736A3A41E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4310" yWindow="4570" windowWidth="7500" windowHeight="6000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="694" uniqueCount="204">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="730" uniqueCount="216">
   <si>
     <t>Original</t>
   </si>
@@ -405,6 +405,18 @@
     <t>Financing fees (% of new debt)</t>
   </si>
   <si>
+    <t>Mandatory amortization (% of original debt a year)</t>
+  </si>
+  <si>
+    <t>Exit fee (% of exit EV)</t>
+  </si>
+  <si>
+    <t>Transaction fees</t>
+  </si>
+  <si>
+    <t>Financing fees</t>
+  </si>
+  <si>
     <t>Total uses</t>
   </si>
   <si>
@@ -414,6 +426,12 @@
     <t>Sponsor equity</t>
   </si>
   <si>
+    <t>Total sources</t>
+  </si>
+  <si>
+    <t>Sources minus uses</t>
+  </si>
+  <si>
     <t>EBITDA (reported basis)</t>
   </si>
   <si>
@@ -429,6 +447,18 @@
     <t>Cash flow after interest</t>
   </si>
   <si>
+    <t>Cash available above minimum</t>
+  </si>
+  <si>
+    <t>Mandatory repayment</t>
+  </si>
+  <si>
+    <t>Funding shortfall (1 = yes)</t>
+  </si>
+  <si>
+    <t>Cash sweep</t>
+  </si>
+  <si>
     <t>Debt repaid</t>
   </si>
   <si>
@@ -438,10 +468,16 @@
     <t>Cash, end of year</t>
   </si>
   <si>
+    <t>Feasible (1 = no funding shortfall)</t>
+  </si>
+  <si>
     <t>Exit EV / EBITDA</t>
   </si>
   <si>
     <t>Exit enterprise value</t>
+  </si>
+  <si>
+    <t>Exit fee</t>
   </si>
   <si>
     <t>Exit equity value</t>
@@ -2679,7 +2715,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
-  <dimension ref="A1:G39"/>
+  <dimension ref="A1:G51"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
@@ -2708,7 +2744,7 @@
         <v>101</v>
       </c>
       <c r="B2">
-        <v>65.8935546875</v>
+        <v>65.09765625</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
@@ -2725,7 +2761,7 @@
       </c>
       <c r="B4">
         <f>B2*B3</f>
-        <v>898.3441610595703</v>
+        <v>887.49346833984373</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
@@ -2758,7 +2794,7 @@
       </c>
       <c r="B8">
         <f>B4+B5-B6</f>
-        <v>927.20916105957031</v>
+        <v>916.35846833984374</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
@@ -2775,7 +2811,7 @@
       </c>
       <c r="B10">
         <f>B8/B9</f>
-        <v>8.2798360574686587</v>
+        <v>8.1829410303243666</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">
@@ -2841,8 +2877,7 @@
         <v>117</v>
       </c>
       <c r="B18">
-        <f>B4+B5+B8*B16+B12*B17</f>
-        <v>1016.4815442807617</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.35">
@@ -2850,8 +2885,7 @@
         <v>118</v>
       </c>
       <c r="B19">
-        <f>B6-B7</f>
-        <v>28.130000000000003</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.35">
@@ -2859,342 +2893,514 @@
         <v>119</v>
       </c>
       <c r="B20">
-        <f>B18-B12-B19</f>
-        <v>484.42354428076169</v>
+        <f>B8*B16</f>
+        <v>18.327169366796877</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="B21">
+        <f>B12*B17</f>
+        <v>12.5982</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A22" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="B22">
+        <f>B4+B5+B20+B21</f>
+        <v>1005.4138377066406</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A23" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="B23">
+        <f>B6-B7</f>
+        <v>28.130000000000003</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A24" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="B24">
+        <f>B22-B12-B23</f>
+        <v>473.35583770664061</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A25" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="B25">
+        <f>B12+B23+B24</f>
+        <v>1005.4138377066406</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A26" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="B26">
+        <f>B25-B22</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A27" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C21">
+      <c r="C27">
         <f>'DCF Base'!C4</f>
         <v>642.5</v>
       </c>
-      <c r="D21">
+      <c r="D27">
         <f>'DCF Base'!D4</f>
         <v>679.82720946465338</v>
       </c>
-      <c r="E21">
+      <c r="E27">
         <f>'DCF Base'!E4</f>
         <v>719.32301125058007</v>
       </c>
-      <c r="F21">
+      <c r="F27">
         <f>'DCF Base'!F4</f>
         <v>761.11339368434756</v>
       </c>
-      <c r="G21">
+      <c r="G27">
         <f>'DCF Base'!G4</f>
         <v>805.33166461416681</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A22" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="C22">
-        <f>'DCF Base'!C6+C21*(B39-B38)</f>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A28" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="C28">
+        <f>'DCF Base'!C6+C27*(B51-B50)</f>
         <v>114.90614450349602</v>
       </c>
-      <c r="D22">
-        <f>'DCF Base'!D6+D21*(B39-B38)</f>
+      <c r="D28">
+        <f>'DCF Base'!D6+D27*(B51-B50)</f>
         <v>124.49511982082481</v>
       </c>
-      <c r="E22">
-        <f>'DCF Base'!E6+E21*(B39-B38)</f>
+      <c r="E28">
+        <f>'DCF Base'!E6+E27*(B51-B50)</f>
         <v>133.26916406523574</v>
       </c>
-      <c r="F22">
-        <f>'DCF Base'!F6+F21*(B39-B38)</f>
+      <c r="F28">
+        <f>'DCF Base'!F6+F27*(B51-B50)</f>
         <v>142.64249549073159</v>
       </c>
-      <c r="G22">
-        <f>'DCF Base'!G6+G21*(B39-B38)</f>
+      <c r="G28">
+        <f>'DCF Base'!G6+G27*(B51-B50)</f>
         <v>152.65513294758597</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A23" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="C23">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A29" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="C29">
         <f>'DCF Base'!C11</f>
         <v>65.086728601006627</v>
       </c>
-      <c r="D23">
+      <c r="D29">
         <f>'DCF Base'!D11</f>
         <v>71.111296628614184</v>
       </c>
-      <c r="E23">
+      <c r="E29">
         <f>'DCF Base'!E11</f>
         <v>76.429417459616076</v>
       </c>
-      <c r="F23">
+      <c r="F29">
         <f>'DCF Base'!F11</f>
         <v>82.125452389621302</v>
       </c>
-      <c r="G23">
+      <c r="G29">
         <f>'DCF Base'!G11</f>
         <v>90.890754739313536</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A24" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="C24">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A30" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="C30">
         <f>B15*B12</f>
         <v>39.507955199999998</v>
       </c>
-      <c r="D24">
-        <f>B15*C29</f>
+      <c r="D30">
+        <f>B15*C39</f>
         <v>36.790171917194677</v>
       </c>
-      <c r="E24">
-        <f>B15*D29</f>
+      <c r="E30">
+        <f>B15*D39</f>
         <v>33.435995359808537</v>
       </c>
-      <c r="F24">
-        <f>B15*E29</f>
+      <c r="F30">
+        <f>B15*E39</f>
         <v>29.462393198855555</v>
       </c>
-      <c r="G24">
-        <f>B15*F29</f>
+      <c r="G30">
+        <f>B15*F39</f>
         <v>24.802343484137754</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A25" s="1" t="s">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A31" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="C25">
+      <c r="C31">
         <f>'DCF Base'!C7</f>
         <v>0.23</v>
       </c>
-      <c r="D25">
+      <c r="D31">
         <f>'DCF Base'!D7</f>
         <v>0.23</v>
       </c>
-      <c r="E25">
+      <c r="E31">
         <f>'DCF Base'!E7</f>
         <v>0.23</v>
       </c>
-      <c r="F25">
+      <c r="F31">
         <f>'DCF Base'!F7</f>
         <v>0.23</v>
       </c>
-      <c r="G25">
+      <c r="G31">
         <f>'DCF Base'!G7</f>
         <v>0.23</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A26" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="C26">
-        <f>C24*(1-C25)</f>
-        <v>30.421125503999999</v>
-      </c>
-      <c r="D26">
-        <f>D24*(1-D25)</f>
-        <v>28.328432376239903</v>
-      </c>
-      <c r="E26">
-        <f>E24*(1-E25)</f>
-        <v>25.745716427052574</v>
-      </c>
-      <c r="F26">
-        <f>F24*(1-F25)</f>
-        <v>22.686042763118778</v>
-      </c>
-      <c r="G26">
-        <f>G24*(1-G25)</f>
-        <v>19.097804482786071</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A27" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="C27">
-        <f>C23-C26</f>
-        <v>34.665603097006624</v>
-      </c>
-      <c r="D27">
-        <f>D23-D26</f>
-        <v>42.782864252374281</v>
-      </c>
-      <c r="E27">
-        <f>E23-E26</f>
-        <v>50.683701032563505</v>
-      </c>
-      <c r="F27">
-        <f>F23-F26</f>
-        <v>59.439409626502524</v>
-      </c>
-      <c r="G27">
-        <f>G23-G26</f>
-        <v>71.792950256527462</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A28" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="C28">
-        <f>IF(C27&gt;B12,B12,C27)</f>
-        <v>34.665603097006624</v>
-      </c>
-      <c r="D28">
-        <f>IF(D27&gt;C29,C29,D27)</f>
-        <v>42.782864252374281</v>
-      </c>
-      <c r="E28">
-        <f>IF(E27&gt;D29,D29,E27)</f>
-        <v>50.683701032563505</v>
-      </c>
-      <c r="F28">
-        <f>IF(F27&gt;E29,E29,F27)</f>
-        <v>59.439409626502524</v>
-      </c>
-      <c r="G28">
-        <f>IF(G27&gt;F29,F29,G27)</f>
-        <v>71.792950256527462</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A29" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="B29">
-        <f>B12</f>
-        <v>503.928</v>
-      </c>
-      <c r="C29">
-        <f>B12-C28</f>
-        <v>469.26239690299337</v>
-      </c>
-      <c r="D29">
-        <f>C29-D28</f>
-        <v>426.47953265061909</v>
-      </c>
-      <c r="E29">
-        <f>D29-E28</f>
-        <v>375.79583161805556</v>
-      </c>
-      <c r="F29">
-        <f>E29-F28</f>
-        <v>316.35642199155302</v>
-      </c>
-      <c r="G29">
-        <f>F29-G28</f>
-        <v>244.56347173502556</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A30" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="B30">
-        <f>B7</f>
-        <v>30</v>
-      </c>
-      <c r="C30">
-        <f>B7+C27-C28</f>
-        <v>30</v>
-      </c>
-      <c r="D30">
-        <f>C30+D27-D28</f>
-        <v>30</v>
-      </c>
-      <c r="E30">
-        <f>D30+E27-E28</f>
-        <v>30</v>
-      </c>
-      <c r="F30">
-        <f>E30+F27-F28</f>
-        <v>30</v>
-      </c>
-      <c r="G30">
-        <f>F30+G27-G28</f>
-        <v>30</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A31" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="B31">
-        <v>11.090646475186521</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="B32">
-        <f>B31*G22</f>
-        <v>1693.0441121442741</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C32">
+        <f>C30*(1-C31)</f>
+        <v>30.421125503999999</v>
+      </c>
+      <c r="D32">
+        <f>D30*(1-D31)</f>
+        <v>28.328432376239903</v>
+      </c>
+      <c r="E32">
+        <f>E30*(1-E31)</f>
+        <v>25.745716427052574</v>
+      </c>
+      <c r="F32">
+        <f>F30*(1-F31)</f>
+        <v>22.686042763118778</v>
+      </c>
+      <c r="G32">
+        <f>G30*(1-G31)</f>
+        <v>19.097804482786071</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A33" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="B33">
-        <f>B32-G29+G30</f>
-        <v>1478.4806404092485</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C33">
+        <f>C29-C32</f>
+        <v>34.665603097006624</v>
+      </c>
+      <c r="D33">
+        <f>D29-D32</f>
+        <v>42.782864252374281</v>
+      </c>
+      <c r="E33">
+        <f>E29-E32</f>
+        <v>50.683701032563505</v>
+      </c>
+      <c r="F33">
+        <f>F29-F32</f>
+        <v>59.439409626502524</v>
+      </c>
+      <c r="G33">
+        <f>G29-G32</f>
+        <v>71.792950256527462</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A34" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="B34">
-        <f>B33/B20</f>
-        <v>3.0520412516373323</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C34">
+        <f>B7+C33-B7</f>
+        <v>34.665603097006624</v>
+      </c>
+      <c r="D34">
+        <f>C40+D33-B7</f>
+        <v>42.782864252374281</v>
+      </c>
+      <c r="E34">
+        <f>D40+E33-B7</f>
+        <v>50.683701032563505</v>
+      </c>
+      <c r="F34">
+        <f>E40+F33-B7</f>
+        <v>59.439409626502524</v>
+      </c>
+      <c r="G34">
+        <f>F40+G33-B7</f>
+        <v>71.792950256527462</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A35" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="B35">
-        <f>B34^(1/5)-1</f>
-        <v>0.25002321847155828</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C35">
+        <f>IF(B18*B12&lt;B12,B18*B12,B12)</f>
+        <v>5.0392799999999998</v>
+      </c>
+      <c r="D35">
+        <f>IF(B18*B12&lt;C39,B18*B12,C39)</f>
+        <v>5.0392799999999998</v>
+      </c>
+      <c r="E35">
+        <f>IF(B18*B12&lt;D39,B18*B12,D39)</f>
+        <v>5.0392799999999998</v>
+      </c>
+      <c r="F35">
+        <f>IF(B18*B12&lt;E39,B18*B12,E39)</f>
+        <v>5.0392799999999998</v>
+      </c>
+      <c r="G35">
+        <f>IF(B18*B12&lt;F39,B18*B12,F39)</f>
+        <v>5.0392799999999998</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A36" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="B36">
-        <v>0.25</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C36">
+        <f>IF(C34&lt;C35,1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="D36">
+        <f>IF(D34&lt;D35,1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="E36">
+        <f>IF(E34&lt;E35,1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F36">
+        <f>IF(F34&lt;F35,1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="G36">
+        <f>IF(G34&lt;G35,1,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A37" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="B37">
-        <f>IF(B35&gt;=B36,1,0)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C37">
+        <f>IF(C34-C35&gt;0,IF(C34-C35&lt;B12-C35,C34-C35,B12-C35),0)</f>
+        <v>29.626323097006626</v>
+      </c>
+      <c r="D37">
+        <f>IF(D34-D35&gt;0,IF(D34-D35&lt;C39-D35,D34-D35,C39-D35),0)</f>
+        <v>37.743584252374283</v>
+      </c>
+      <c r="E37">
+        <f>IF(E34-E35&gt;0,IF(E34-E35&lt;D39-E35,E34-E35,D39-E35),0)</f>
+        <v>45.644421032563507</v>
+      </c>
+      <c r="F37">
+        <f>IF(F34-F35&gt;0,IF(F34-F35&lt;E39-F35,F34-F35,E39-F35),0)</f>
+        <v>54.400129626502526</v>
+      </c>
+      <c r="G37">
+        <f>IF(G34-G35&gt;0,IF(G34-G35&lt;F39-G35,G34-G35,F39-G35),0)</f>
+        <v>66.753670256527457</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A38" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="B38">
-        <v>3.656002430166319E-3</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C38">
+        <f>C35+C37</f>
+        <v>34.665603097006624</v>
+      </c>
+      <c r="D38">
+        <f>D35+D37</f>
+        <v>42.782864252374281</v>
+      </c>
+      <c r="E38">
+        <f>E35+E37</f>
+        <v>50.683701032563505</v>
+      </c>
+      <c r="F38">
+        <f>F35+F37</f>
+        <v>59.439409626502524</v>
+      </c>
+      <c r="G38">
+        <f>G35+G37</f>
+        <v>71.792950256527462</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A39" s="1" t="s">
         <v>136</v>
       </c>
       <c r="B39">
+        <f>B12</f>
+        <v>503.928</v>
+      </c>
+      <c r="C39">
+        <f>B12-C38</f>
+        <v>469.26239690299337</v>
+      </c>
+      <c r="D39">
+        <f>C39-D38</f>
+        <v>426.47953265061909</v>
+      </c>
+      <c r="E39">
+        <f>D39-E38</f>
+        <v>375.79583161805556</v>
+      </c>
+      <c r="F39">
+        <f>E39-F38</f>
+        <v>316.35642199155302</v>
+      </c>
+      <c r="G39">
+        <f>F39-G38</f>
+        <v>244.56347173502556</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A40" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="B40">
+        <f>B7</f>
+        <v>30</v>
+      </c>
+      <c r="C40">
+        <f>B7+C33-C38</f>
+        <v>30</v>
+      </c>
+      <c r="D40">
+        <f>C40+D33-D38</f>
+        <v>30</v>
+      </c>
+      <c r="E40">
+        <f>D40+E33-E38</f>
+        <v>30</v>
+      </c>
+      <c r="F40">
+        <f>E40+F33-F38</f>
+        <v>30</v>
+      </c>
+      <c r="G40">
+        <f>F40+G33-G38</f>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A41" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="B41">
+        <f>IF(SUM(C36:G36)&gt;0,0,1)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A42" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="B42">
+        <v>11.090646475186521</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A43" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="B43">
+        <f>B42*G28</f>
+        <v>1693.0441121442741</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A44" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="B44">
+        <f>B43*B19</f>
+        <v>33.860882242885481</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A45" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="B45">
+        <f>B43-B44-G39+G40</f>
+        <v>1444.619758166363</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A46" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="B46">
+        <f>B45/B24</f>
+        <v>3.0518684741808491</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A47" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="B47">
+        <f>IF(B46&gt;0,B46^(1/5)-1,-1)</f>
+        <v>0.25000906527340749</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A48" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="B48">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A49" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="B49">
+        <f>IF(B41=1,IF(B47&gt;=B48,1,0),0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A50" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="B50">
+        <v>3.656002430166319E-3</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A51" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="B51">
         <v>1.3211609958305439E-2</v>
       </c>
     </row>
@@ -3205,7 +3411,7 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
-  <dimension ref="A1:G39"/>
+  <dimension ref="A1:G51"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
@@ -3234,7 +3440,7 @@
         <v>101</v>
       </c>
       <c r="B2">
-        <v>75.859375</v>
+        <v>74.873046875</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
@@ -3251,7 +3457,7 @@
       </c>
       <c r="B4">
         <f>B2*B3</f>
-        <v>1034.2108103906251</v>
+        <v>1020.7639396582031</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
@@ -3284,7 +3490,7 @@
       </c>
       <c r="B8">
         <f>B4+B5-B6</f>
-        <v>1063.0758103906251</v>
+        <v>1049.6289396582029</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
@@ -3301,7 +3507,7 @@
       </c>
       <c r="B10">
         <f>B8/B9</f>
-        <v>9.4931044648398437</v>
+        <v>9.3730259649432313</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">
@@ -3367,8 +3573,7 @@
         <v>117</v>
       </c>
       <c r="B18">
-        <f>B4+B5+B8*B16+B12*B17</f>
-        <v>1156.4653265984377</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.35">
@@ -3376,8 +3581,7 @@
         <v>118</v>
       </c>
       <c r="B19">
-        <f>B6-B7</f>
-        <v>28.130000000000003</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.35">
@@ -3385,342 +3589,514 @@
         <v>119</v>
       </c>
       <c r="B20">
-        <f>B18-B12-B19</f>
-        <v>568.41532659843779</v>
+        <f>B8*B16</f>
+        <v>20.992578793164057</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="B21">
+        <f>B12*B17</f>
+        <v>13.997999999999999</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A22" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="B22">
+        <f>B4+B5+B20+B21</f>
+        <v>1142.7495184513671</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A23" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="B23">
+        <f>B6-B7</f>
+        <v>28.130000000000003</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A24" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="B24">
+        <f>B22-B12-B23</f>
+        <v>554.69951845136711</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A25" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="B25">
+        <f>B12+B23+B24</f>
+        <v>1142.7495184513671</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A26" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="B26">
+        <f>B25-B22</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A27" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C21">
+      <c r="C27">
         <f>'DCF Base'!C4</f>
         <v>642.5</v>
       </c>
-      <c r="D21">
+      <c r="D27">
         <f>'DCF Base'!D4</f>
         <v>679.82720946465338</v>
       </c>
-      <c r="E21">
+      <c r="E27">
         <f>'DCF Base'!E4</f>
         <v>719.32301125058007</v>
       </c>
-      <c r="F21">
+      <c r="F27">
         <f>'DCF Base'!F4</f>
         <v>761.11339368434756</v>
       </c>
-      <c r="G21">
+      <c r="G27">
         <f>'DCF Base'!G4</f>
         <v>805.33166461416681</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A22" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="C22">
-        <f>'DCF Base'!C6+C21*(B39-B38)</f>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A28" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="C28">
+        <f>'DCF Base'!C6+C27*(B51-B50)</f>
         <v>114.90614450349602</v>
       </c>
-      <c r="D22">
-        <f>'DCF Base'!D6+D21*(B39-B38)</f>
+      <c r="D28">
+        <f>'DCF Base'!D6+D27*(B51-B50)</f>
         <v>124.49511982082481</v>
       </c>
-      <c r="E22">
-        <f>'DCF Base'!E6+E21*(B39-B38)</f>
+      <c r="E28">
+        <f>'DCF Base'!E6+E27*(B51-B50)</f>
         <v>133.26916406523574</v>
       </c>
-      <c r="F22">
-        <f>'DCF Base'!F6+F21*(B39-B38)</f>
+      <c r="F28">
+        <f>'DCF Base'!F6+F27*(B51-B50)</f>
         <v>142.64249549073159</v>
       </c>
-      <c r="G22">
-        <f>'DCF Base'!G6+G21*(B39-B38)</f>
+      <c r="G28">
+        <f>'DCF Base'!G6+G27*(B51-B50)</f>
         <v>152.65513294758597</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A23" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="C23">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A29" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="C29">
         <f>'DCF Base'!C11</f>
         <v>65.086728601006627</v>
       </c>
-      <c r="D23">
+      <c r="D29">
         <f>'DCF Base'!D11</f>
         <v>71.111296628614184</v>
       </c>
-      <c r="E23">
+      <c r="E29">
         <f>'DCF Base'!E11</f>
         <v>76.429417459616076</v>
       </c>
-      <c r="F23">
+      <c r="F29">
         <f>'DCF Base'!F11</f>
         <v>82.125452389621302</v>
       </c>
-      <c r="G23">
+      <c r="G29">
         <f>'DCF Base'!G11</f>
         <v>90.890754739313536</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A24" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="C24">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A30" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="C30">
         <f>B15*B12</f>
         <v>43.897727999999994</v>
       </c>
-      <c r="D24">
-        <f>B15*C29</f>
+      <c r="D30">
+        <f>B15*C39</f>
         <v>41.444946521585074</v>
       </c>
-      <c r="E24">
-        <f>B15*D29</f>
+      <c r="E30">
+        <f>B15*D39</f>
         <v>38.371769397516772</v>
       </c>
-      <c r="F24">
-        <f>B15*E29</f>
+      <c r="F30">
+        <f>B15*E39</f>
         <v>34.696130043672163</v>
       </c>
-      <c r="G24">
-        <f>B15*F29</f>
+      <c r="G30">
+        <f>B15*F39</f>
         <v>30.352030554802255</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A25" s="1" t="s">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A31" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="C25">
+      <c r="C31">
         <f>'DCF Base'!C7</f>
         <v>0.23</v>
       </c>
-      <c r="D25">
+      <c r="D31">
         <f>'DCF Base'!D7</f>
         <v>0.23</v>
       </c>
-      <c r="E25">
+      <c r="E31">
         <f>'DCF Base'!E7</f>
         <v>0.23</v>
       </c>
-      <c r="F25">
+      <c r="F31">
         <f>'DCF Base'!F7</f>
         <v>0.23</v>
       </c>
-      <c r="G25">
+      <c r="G31">
         <f>'DCF Base'!G7</f>
         <v>0.23</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A26" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="C26">
-        <f>C24*(1-C25)</f>
-        <v>33.801250559999993</v>
-      </c>
-      <c r="D26">
-        <f>D24*(1-D25)</f>
-        <v>31.912608821620509</v>
-      </c>
-      <c r="E26">
-        <f>E24*(1-E25)</f>
-        <v>29.546262436087915</v>
-      </c>
-      <c r="F26">
-        <f>F24*(1-F25)</f>
-        <v>26.716020133627566</v>
-      </c>
-      <c r="G26">
-        <f>G24*(1-G25)</f>
-        <v>23.371063527197737</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A27" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="C27">
-        <f>C23-C26</f>
-        <v>31.285478041006634</v>
-      </c>
-      <c r="D27">
-        <f>D23-D26</f>
-        <v>39.198687806993675</v>
-      </c>
-      <c r="E27">
-        <f>E23-E26</f>
-        <v>46.883155023528161</v>
-      </c>
-      <c r="F27">
-        <f>F23-F26</f>
-        <v>55.409432255993735</v>
-      </c>
-      <c r="G27">
-        <f>G23-G26</f>
-        <v>67.519691212115802</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A28" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="C28">
-        <f>IF(C27&gt;B12,B12,C27)</f>
-        <v>31.285478041006634</v>
-      </c>
-      <c r="D28">
-        <f>IF(D27&gt;C29,C29,D27)</f>
-        <v>39.198687806993675</v>
-      </c>
-      <c r="E28">
-        <f>IF(E27&gt;D29,D29,E27)</f>
-        <v>46.883155023528161</v>
-      </c>
-      <c r="F28">
-        <f>IF(F27&gt;E29,E29,F27)</f>
-        <v>55.409432255993735</v>
-      </c>
-      <c r="G28">
-        <f>IF(G27&gt;F29,F29,G27)</f>
-        <v>67.519691212115802</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A29" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="B29">
-        <f>B12</f>
-        <v>559.91999999999996</v>
-      </c>
-      <c r="C29">
-        <f>B12-C28</f>
-        <v>528.63452195899333</v>
-      </c>
-      <c r="D29">
-        <f>C29-D28</f>
-        <v>489.43583415199964</v>
-      </c>
-      <c r="E29">
-        <f>D29-E28</f>
-        <v>442.55267912847148</v>
-      </c>
-      <c r="F29">
-        <f>E29-F28</f>
-        <v>387.14324687247773</v>
-      </c>
-      <c r="G29">
-        <f>F29-G28</f>
-        <v>319.62355566036194</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A30" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="B30">
-        <f>B7</f>
-        <v>30</v>
-      </c>
-      <c r="C30">
-        <f>B7+C27-C28</f>
-        <v>30</v>
-      </c>
-      <c r="D30">
-        <f>C30+D27-D28</f>
-        <v>30</v>
-      </c>
-      <c r="E30">
-        <f>D30+E27-E28</f>
-        <v>30</v>
-      </c>
-      <c r="F30">
-        <f>E30+F27-F28</f>
-        <v>30</v>
-      </c>
-      <c r="G30">
-        <f>F30+G27-G28</f>
-        <v>30</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A31" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="B31">
-        <v>11.162988929834521</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="B32">
-        <f>B31*G22</f>
-        <v>1704.0875591763192</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C32">
+        <f>C30*(1-C31)</f>
+        <v>33.801250559999993</v>
+      </c>
+      <c r="D32">
+        <f>D30*(1-D31)</f>
+        <v>31.912608821620509</v>
+      </c>
+      <c r="E32">
+        <f>E30*(1-E31)</f>
+        <v>29.546262436087915</v>
+      </c>
+      <c r="F32">
+        <f>F30*(1-F31)</f>
+        <v>26.716020133627566</v>
+      </c>
+      <c r="G32">
+        <f>G30*(1-G31)</f>
+        <v>23.371063527197737</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A33" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="B33">
-        <f>B32-G29+G30</f>
-        <v>1414.4640035159573</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C33">
+        <f>C29-C32</f>
+        <v>31.285478041006634</v>
+      </c>
+      <c r="D33">
+        <f>D29-D32</f>
+        <v>39.198687806993675</v>
+      </c>
+      <c r="E33">
+        <f>E29-E32</f>
+        <v>46.883155023528161</v>
+      </c>
+      <c r="F33">
+        <f>F29-F32</f>
+        <v>55.409432255993735</v>
+      </c>
+      <c r="G33">
+        <f>G29-G32</f>
+        <v>67.519691212115802</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A34" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="B34">
-        <f>B33/B20</f>
-        <v>2.488433962505058</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C34">
+        <f>B7+C33-B7</f>
+        <v>31.285478041006634</v>
+      </c>
+      <c r="D34">
+        <f>C40+D33-B7</f>
+        <v>39.198687806993675</v>
+      </c>
+      <c r="E34">
+        <f>D40+E33-B7</f>
+        <v>46.883155023528161</v>
+      </c>
+      <c r="F34">
+        <f>E40+F33-B7</f>
+        <v>55.409432255993735</v>
+      </c>
+      <c r="G34">
+        <f>F40+G33-B7</f>
+        <v>67.519691212115802</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A35" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="B35">
-        <f>B34^(1/5)-1</f>
-        <v>0.20001099155260116</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C35">
+        <f>IF(B18*B12&lt;B12,B18*B12,B12)</f>
+        <v>5.5991999999999997</v>
+      </c>
+      <c r="D35">
+        <f>IF(B18*B12&lt;C39,B18*B12,C39)</f>
+        <v>5.5991999999999997</v>
+      </c>
+      <c r="E35">
+        <f>IF(B18*B12&lt;D39,B18*B12,D39)</f>
+        <v>5.5991999999999997</v>
+      </c>
+      <c r="F35">
+        <f>IF(B18*B12&lt;E39,B18*B12,E39)</f>
+        <v>5.5991999999999997</v>
+      </c>
+      <c r="G35">
+        <f>IF(B18*B12&lt;F39,B18*B12,F39)</f>
+        <v>5.5991999999999997</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A36" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="B36">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C36">
+        <f>IF(C34&lt;C35,1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="D36">
+        <f>IF(D34&lt;D35,1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="E36">
+        <f>IF(E34&lt;E35,1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F36">
+        <f>IF(F34&lt;F35,1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="G36">
+        <f>IF(G34&lt;G35,1,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A37" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="B37">
-        <f>IF(B35&gt;=B36,1,0)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C37">
+        <f>IF(C34-C35&gt;0,IF(C34-C35&lt;B12-C35,C34-C35,B12-C35),0)</f>
+        <v>25.686278041006634</v>
+      </c>
+      <c r="D37">
+        <f>IF(D34-D35&gt;0,IF(D34-D35&lt;C39-D35,D34-D35,C39-D35),0)</f>
+        <v>33.599487806993679</v>
+      </c>
+      <c r="E37">
+        <f>IF(E34-E35&gt;0,IF(E34-E35&lt;D39-E35,E34-E35,D39-E35),0)</f>
+        <v>41.283955023528165</v>
+      </c>
+      <c r="F37">
+        <f>IF(F34-F35&gt;0,IF(F34-F35&lt;E39-F35,F34-F35,E39-F35),0)</f>
+        <v>49.810232255993739</v>
+      </c>
+      <c r="G37">
+        <f>IF(G34-G35&gt;0,IF(G34-G35&lt;F39-G35,G34-G35,F39-G35),0)</f>
+        <v>61.920491212115806</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A38" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="B38">
-        <v>3.656002430166319E-3</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C38">
+        <f>C35+C37</f>
+        <v>31.285478041006634</v>
+      </c>
+      <c r="D38">
+        <f>D35+D37</f>
+        <v>39.198687806993675</v>
+      </c>
+      <c r="E38">
+        <f>E35+E37</f>
+        <v>46.883155023528161</v>
+      </c>
+      <c r="F38">
+        <f>F35+F37</f>
+        <v>55.409432255993735</v>
+      </c>
+      <c r="G38">
+        <f>G35+G37</f>
+        <v>67.519691212115802</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A39" s="1" t="s">
         <v>136</v>
       </c>
       <c r="B39">
+        <f>B12</f>
+        <v>559.91999999999996</v>
+      </c>
+      <c r="C39">
+        <f>B12-C38</f>
+        <v>528.63452195899333</v>
+      </c>
+      <c r="D39">
+        <f>C39-D38</f>
+        <v>489.43583415199964</v>
+      </c>
+      <c r="E39">
+        <f>D39-E38</f>
+        <v>442.55267912847148</v>
+      </c>
+      <c r="F39">
+        <f>E39-F38</f>
+        <v>387.14324687247773</v>
+      </c>
+      <c r="G39">
+        <f>F39-G38</f>
+        <v>319.62355566036194</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A40" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="B40">
+        <f>B7</f>
+        <v>30</v>
+      </c>
+      <c r="C40">
+        <f>B7+C33-C38</f>
+        <v>30</v>
+      </c>
+      <c r="D40">
+        <f>C40+D33-D38</f>
+        <v>30</v>
+      </c>
+      <c r="E40">
+        <f>D40+E33-E38</f>
+        <v>30</v>
+      </c>
+      <c r="F40">
+        <f>E40+F33-F38</f>
+        <v>30</v>
+      </c>
+      <c r="G40">
+        <f>F40+G33-G38</f>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A41" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="B41">
+        <f>IF(SUM(C36:G36)&gt;0,0,1)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A42" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="B42">
+        <v>11.162988929834521</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A43" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="B43">
+        <f>B42*G28</f>
+        <v>1704.0875591763192</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A44" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="B44">
+        <f>B43*B19</f>
+        <v>34.081751183526386</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A45" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="B45">
+        <f>B43-B44-G39+G40</f>
+        <v>1380.3822523324309</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A46" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="B46">
+        <f>B45/B24</f>
+        <v>2.4885225359240239</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A47" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="B47">
+        <f>IF(B46&gt;0,B46^(1/5)-1,-1)</f>
+        <v>0.20001953407891682</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A48" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="B48">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A49" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="B49">
+        <f>IF(B41=1,IF(B47&gt;=B48,1,0),0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A50" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="B50">
+        <v>3.656002430166319E-3</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A51" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="B51">
         <v>1.3211609958305439E-2</v>
       </c>
     </row>
@@ -3731,7 +4107,7 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
-  <dimension ref="A1:G39"/>
+  <dimension ref="A1:G51"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
@@ -3760,7 +4136,7 @@
         <v>101</v>
       </c>
       <c r="B2">
-        <v>107.8955078125</v>
+        <v>106.2841796875</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
@@ -3777,7 +4153,7 @@
       </c>
       <c r="B4">
         <f>B2*B3</f>
-        <v>1470.9678345263671</v>
+        <v>1449.0001744189453</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
@@ -3810,7 +4186,7 @@
       </c>
       <c r="B8">
         <f>B4+B5-B6</f>
-        <v>1499.8328345263672</v>
+        <v>1477.8651744189451</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
@@ -3827,7 +4203,7 @@
       </c>
       <c r="B10">
         <f>B8/B9</f>
-        <v>13.393277919402479</v>
+        <v>13.197110073036731</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">
@@ -3893,8 +4269,7 @@
         <v>117</v>
       </c>
       <c r="B18">
-        <f>B4+B5+B8*B16+B12*B17</f>
-        <v>1603.3572912168945</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.35">
@@ -3902,8 +4277,7 @@
         <v>118</v>
       </c>
       <c r="B19">
-        <f>B6-B7</f>
-        <v>28.130000000000003</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.35">
@@ -3911,342 +4285,514 @@
         <v>119</v>
       </c>
       <c r="B20">
-        <f>B18-B12-B19</f>
-        <v>959.31529121689459</v>
+        <f>B8*B16</f>
+        <v>29.557303488378903</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="B21">
+        <f>B12*B17</f>
+        <v>15.397799999999998</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A22" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="B22">
+        <f>B4+B5+B20+B21</f>
+        <v>1580.9502779073241</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A23" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="B23">
+        <f>B6-B7</f>
+        <v>28.130000000000003</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A24" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="B24">
+        <f>B22-B12-B23</f>
+        <v>936.90827790732419</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A25" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="B25">
+        <f>B12+B23+B24</f>
+        <v>1580.9502779073241</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A26" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="B26">
+        <f>B25-B22</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A27" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C21">
+      <c r="C27">
         <f>'DCF Base'!C4</f>
         <v>642.5</v>
       </c>
-      <c r="D21">
+      <c r="D27">
         <f>'DCF Base'!D4</f>
         <v>679.82720946465338</v>
       </c>
-      <c r="E21">
+      <c r="E27">
         <f>'DCF Base'!E4</f>
         <v>719.32301125058007</v>
       </c>
-      <c r="F21">
+      <c r="F27">
         <f>'DCF Base'!F4</f>
         <v>761.11339368434756</v>
       </c>
-      <c r="G21">
+      <c r="G27">
         <f>'DCF Base'!G4</f>
         <v>805.33166461416681</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A22" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="C22">
-        <f>'DCF Base'!C6+C21*(B39-B38)</f>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A28" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="C28">
+        <f>'DCF Base'!C6+C27*(B51-B50)</f>
         <v>114.90614450349602</v>
       </c>
-      <c r="D22">
-        <f>'DCF Base'!D6+D21*(B39-B38)</f>
+      <c r="D28">
+        <f>'DCF Base'!D6+D27*(B51-B50)</f>
         <v>124.49511982082481</v>
       </c>
-      <c r="E22">
-        <f>'DCF Base'!E6+E21*(B39-B38)</f>
+      <c r="E28">
+        <f>'DCF Base'!E6+E27*(B51-B50)</f>
         <v>133.26916406523574</v>
       </c>
-      <c r="F22">
-        <f>'DCF Base'!F6+F21*(B39-B38)</f>
+      <c r="F28">
+        <f>'DCF Base'!F6+F27*(B51-B50)</f>
         <v>142.64249549073159</v>
       </c>
-      <c r="G22">
-        <f>'DCF Base'!G6+G21*(B39-B38)</f>
+      <c r="G28">
+        <f>'DCF Base'!G6+G27*(B51-B50)</f>
         <v>152.65513294758597</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A23" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="C23">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A29" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="C29">
         <f>'DCF Base'!C11</f>
         <v>65.086728601006627</v>
       </c>
-      <c r="D23">
+      <c r="D29">
         <f>'DCF Base'!D11</f>
         <v>71.111296628614184</v>
       </c>
-      <c r="E23">
+      <c r="E29">
         <f>'DCF Base'!E11</f>
         <v>76.429417459616076</v>
       </c>
-      <c r="F23">
+      <c r="F29">
         <f>'DCF Base'!F11</f>
         <v>82.125452389621302</v>
       </c>
-      <c r="G23">
+      <c r="G29">
         <f>'DCF Base'!G11</f>
         <v>90.890754739313536</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A24" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="C24">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A30" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="C30">
         <f>B15*B12</f>
         <v>48.287500799999989</v>
       </c>
-      <c r="D24">
-        <f>B15*C29</f>
+      <c r="D30">
+        <f>B15*C39</f>
         <v>46.099721125975471</v>
       </c>
-      <c r="E24">
-        <f>B15*D29</f>
+      <c r="E30">
+        <f>B15*D39</f>
         <v>43.307543435225007</v>
       </c>
-      <c r="F24">
-        <f>B15*E29</f>
+      <c r="F30">
+        <f>B15*E39</f>
         <v>39.929866888488775</v>
       </c>
-      <c r="G24">
-        <f>B15*F29</f>
+      <c r="G30">
+        <f>B15*F39</f>
         <v>35.901717625466752</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A25" s="1" t="s">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A31" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="C25">
+      <c r="C31">
         <f>'DCF Base'!C7</f>
         <v>0.23</v>
       </c>
-      <c r="D25">
+      <c r="D31">
         <f>'DCF Base'!D7</f>
         <v>0.23</v>
       </c>
-      <c r="E25">
+      <c r="E31">
         <f>'DCF Base'!E7</f>
         <v>0.23</v>
       </c>
-      <c r="F25">
+      <c r="F31">
         <f>'DCF Base'!F7</f>
         <v>0.23</v>
       </c>
-      <c r="G25">
+      <c r="G31">
         <f>'DCF Base'!G7</f>
         <v>0.23</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A26" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="C26">
-        <f>C24*(1-C25)</f>
-        <v>37.18137561599999</v>
-      </c>
-      <c r="D26">
-        <f>D24*(1-D25)</f>
-        <v>35.496785267001115</v>
-      </c>
-      <c r="E26">
-        <f>E24*(1-E25)</f>
-        <v>33.346808445123258</v>
-      </c>
-      <c r="F26">
-        <f>F24*(1-F25)</f>
-        <v>30.745997504136358</v>
-      </c>
-      <c r="G26">
-        <f>G24*(1-G25)</f>
-        <v>27.644322571609401</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A27" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="C27">
-        <f>C23-C26</f>
-        <v>27.905352985006637</v>
-      </c>
-      <c r="D27">
-        <f>D23-D26</f>
-        <v>35.614511361613069</v>
-      </c>
-      <c r="E27">
-        <f>E23-E26</f>
-        <v>43.082609014492817</v>
-      </c>
-      <c r="F27">
-        <f>F23-F26</f>
-        <v>51.379454885484947</v>
-      </c>
-      <c r="G27">
-        <f>G23-G26</f>
-        <v>63.246432167704135</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A28" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="C28">
-        <f>IF(C27&gt;B12,B12,C27)</f>
-        <v>27.905352985006637</v>
-      </c>
-      <c r="D28">
-        <f>IF(D27&gt;C29,C29,D27)</f>
-        <v>35.614511361613069</v>
-      </c>
-      <c r="E28">
-        <f>IF(E27&gt;D29,D29,E27)</f>
-        <v>43.082609014492817</v>
-      </c>
-      <c r="F28">
-        <f>IF(F27&gt;E29,E29,F27)</f>
-        <v>51.379454885484947</v>
-      </c>
-      <c r="G28">
-        <f>IF(G27&gt;F29,F29,G27)</f>
-        <v>63.246432167704135</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A29" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="B29">
-        <f>B12</f>
-        <v>615.91199999999992</v>
-      </c>
-      <c r="C29">
-        <f>B12-C28</f>
-        <v>588.00664701499329</v>
-      </c>
-      <c r="D29">
-        <f>C29-D28</f>
-        <v>552.39213565338025</v>
-      </c>
-      <c r="E29">
-        <f>D29-E28</f>
-        <v>509.30952663888741</v>
-      </c>
-      <c r="F29">
-        <f>E29-F28</f>
-        <v>457.93007175340244</v>
-      </c>
-      <c r="G29">
-        <f>F29-G28</f>
-        <v>394.6836395856983</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A30" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="B30">
-        <f>B7</f>
-        <v>30</v>
-      </c>
-      <c r="C30">
-        <f>B7+C27-C28</f>
-        <v>30</v>
-      </c>
-      <c r="D30">
-        <f>C30+D27-D28</f>
-        <v>30</v>
-      </c>
-      <c r="E30">
-        <f>D30+E27-E28</f>
-        <v>30</v>
-      </c>
-      <c r="F30">
-        <f>E30+F27-F28</f>
-        <v>30</v>
-      </c>
-      <c r="G30">
-        <f>F30+G27-G28</f>
-        <v>30.000000000000007</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A31" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="B31">
-        <v>16.46425504632656</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="B32">
-        <f>B31*G22</f>
-        <v>2513.3530429799443</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C32">
+        <f>C30*(1-C31)</f>
+        <v>37.18137561599999</v>
+      </c>
+      <c r="D32">
+        <f>D30*(1-D31)</f>
+        <v>35.496785267001115</v>
+      </c>
+      <c r="E32">
+        <f>E30*(1-E31)</f>
+        <v>33.346808445123258</v>
+      </c>
+      <c r="F32">
+        <f>F30*(1-F31)</f>
+        <v>30.745997504136358</v>
+      </c>
+      <c r="G32">
+        <f>G30*(1-G31)</f>
+        <v>27.644322571609401</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A33" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="B33">
-        <f>B32-G29+G30</f>
-        <v>2148.6694033942458</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C33">
+        <f>C29-C32</f>
+        <v>27.905352985006637</v>
+      </c>
+      <c r="D33">
+        <f>D29-D32</f>
+        <v>35.614511361613069</v>
+      </c>
+      <c r="E33">
+        <f>E29-E32</f>
+        <v>43.082609014492817</v>
+      </c>
+      <c r="F33">
+        <f>F29-F32</f>
+        <v>51.379454885484947</v>
+      </c>
+      <c r="G33">
+        <f>G29-G32</f>
+        <v>63.246432167704135</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A34" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="B34">
-        <f>B33/B20</f>
-        <v>2.2397948026749908</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C34">
+        <f>B7+C33-B7</f>
+        <v>27.905352985006637</v>
+      </c>
+      <c r="D34">
+        <f>C40+D33-B7</f>
+        <v>35.614511361613069</v>
+      </c>
+      <c r="E34">
+        <f>D40+E33-B7</f>
+        <v>43.082609014492817</v>
+      </c>
+      <c r="F34">
+        <f>E40+F33-B7</f>
+        <v>51.379454885484947</v>
+      </c>
+      <c r="G34">
+        <f>F40+G33-B7</f>
+        <v>63.246432167704143</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A35" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="B35">
-        <f>B34^(1/5)-1</f>
-        <v>0.17501022671377831</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C35">
+        <f>IF(B18*B12&lt;B12,B18*B12,B12)</f>
+        <v>6.1591199999999997</v>
+      </c>
+      <c r="D35">
+        <f>IF(B18*B12&lt;C39,B18*B12,C39)</f>
+        <v>6.1591199999999997</v>
+      </c>
+      <c r="E35">
+        <f>IF(B18*B12&lt;D39,B18*B12,D39)</f>
+        <v>6.1591199999999997</v>
+      </c>
+      <c r="F35">
+        <f>IF(B18*B12&lt;E39,B18*B12,E39)</f>
+        <v>6.1591199999999997</v>
+      </c>
+      <c r="G35">
+        <f>IF(B18*B12&lt;F39,B18*B12,F39)</f>
+        <v>6.1591199999999997</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A36" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="B36">
-        <v>0.17499999999999999</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C36">
+        <f>IF(C34&lt;C35,1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="D36">
+        <f>IF(D34&lt;D35,1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="E36">
+        <f>IF(E34&lt;E35,1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F36">
+        <f>IF(F34&lt;F35,1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="G36">
+        <f>IF(G34&lt;G35,1,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A37" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="B37">
-        <f>IF(B35&gt;=B36,1,0)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C37">
+        <f>IF(C34-C35&gt;0,IF(C34-C35&lt;B12-C35,C34-C35,B12-C35),0)</f>
+        <v>21.746232985006635</v>
+      </c>
+      <c r="D37">
+        <f>IF(D34-D35&gt;0,IF(D34-D35&lt;C39-D35,D34-D35,C39-D35),0)</f>
+        <v>29.455391361613067</v>
+      </c>
+      <c r="E37">
+        <f>IF(E34-E35&gt;0,IF(E34-E35&lt;D39-E35,E34-E35,D39-E35),0)</f>
+        <v>36.923489014492816</v>
+      </c>
+      <c r="F37">
+        <f>IF(F34-F35&gt;0,IF(F34-F35&lt;E39-F35,F34-F35,E39-F35),0)</f>
+        <v>45.220334885484945</v>
+      </c>
+      <c r="G37">
+        <f>IF(G34-G35&gt;0,IF(G34-G35&lt;F39-G35,G34-G35,F39-G35),0)</f>
+        <v>57.087312167704141</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A38" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="B38">
-        <v>3.656002430166319E-3</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C38">
+        <f>C35+C37</f>
+        <v>27.905352985006637</v>
+      </c>
+      <c r="D38">
+        <f>D35+D37</f>
+        <v>35.614511361613069</v>
+      </c>
+      <c r="E38">
+        <f>E35+E37</f>
+        <v>43.082609014492817</v>
+      </c>
+      <c r="F38">
+        <f>F35+F37</f>
+        <v>51.379454885484947</v>
+      </c>
+      <c r="G38">
+        <f>G35+G37</f>
+        <v>63.246432167704143</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A39" s="1" t="s">
         <v>136</v>
       </c>
       <c r="B39">
+        <f>B12</f>
+        <v>615.91199999999992</v>
+      </c>
+      <c r="C39">
+        <f>B12-C38</f>
+        <v>588.00664701499329</v>
+      </c>
+      <c r="D39">
+        <f>C39-D38</f>
+        <v>552.39213565338025</v>
+      </c>
+      <c r="E39">
+        <f>D39-E38</f>
+        <v>509.30952663888741</v>
+      </c>
+      <c r="F39">
+        <f>E39-F38</f>
+        <v>457.93007175340244</v>
+      </c>
+      <c r="G39">
+        <f>F39-G38</f>
+        <v>394.6836395856983</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A40" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="B40">
+        <f>B7</f>
+        <v>30</v>
+      </c>
+      <c r="C40">
+        <f>B7+C33-C38</f>
+        <v>30</v>
+      </c>
+      <c r="D40">
+        <f>C40+D33-D38</f>
+        <v>30</v>
+      </c>
+      <c r="E40">
+        <f>D40+E33-E38</f>
+        <v>30</v>
+      </c>
+      <c r="F40">
+        <f>E40+F33-F38</f>
+        <v>30</v>
+      </c>
+      <c r="G40">
+        <f>F40+G33-G38</f>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A41" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="B41">
+        <f>IF(SUM(C36:G36)&gt;0,0,1)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A42" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="B42">
+        <v>16.46425504632656</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A43" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="B43">
+        <f>B42*G28</f>
+        <v>2513.3530429799443</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A44" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="B44">
+        <f>B43*B19</f>
+        <v>50.267060859598885</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A45" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="B45">
+        <f>B43-B44-G39+G40</f>
+        <v>2098.4023425346468</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A46" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="B46">
+        <f>B45/B24</f>
+        <v>2.2397094699831586</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A47" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="B47">
+        <f>IF(B46&gt;0,B46^(1/5)-1,-1)</f>
+        <v>0.17500127336559701</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A48" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="B48">
+        <v>0.17499999999999999</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A49" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="B49">
+        <f>IF(B41=1,IF(B47&gt;=B48,1,0),0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A50" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="B50">
+        <v>3.656002430166319E-3</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A51" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="B51">
         <v>1.3211609958305439E-2</v>
       </c>
     </row>
@@ -4298,7 +4844,7 @@
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>137</v>
+        <v>149</v>
       </c>
       <c r="C2">
         <f>'DCF Base'!C4</f>
@@ -4343,7 +4889,7 @@
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>138</v>
+        <v>150</v>
       </c>
       <c r="C3">
         <v>0.5</v>
@@ -4378,7 +4924,7 @@
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
-        <v>139</v>
+        <v>151</v>
       </c>
       <c r="C4">
         <f>C2*B10*C3</f>
@@ -4423,7 +4969,7 @@
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
-        <v>140</v>
+        <v>152</v>
       </c>
       <c r="C5">
         <f>0.5*B11*D2*B10</f>
@@ -4460,7 +5006,7 @@
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
-        <v>141</v>
+        <v>153</v>
       </c>
       <c r="C6">
         <f>'DCF Base'!C7</f>
@@ -4505,7 +5051,7 @@
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
-        <v>142</v>
+        <v>154</v>
       </c>
       <c r="C7">
         <f t="shared" ref="C7:L7" si="0">(C4-C5)*(1-C6)</f>
@@ -4550,7 +5096,7 @@
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
-        <v>143</v>
+        <v>155</v>
       </c>
       <c r="C8">
         <f>'DCF Base'!C13</f>
@@ -4595,7 +5141,7 @@
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
-        <v>144</v>
+        <v>156</v>
       </c>
       <c r="C9">
         <f t="shared" ref="C9:L9" si="1">C7*C8</f>
@@ -4640,7 +5186,7 @@
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
-        <v>145</v>
+        <v>157</v>
       </c>
       <c r="B10">
         <v>3.2258064516129031E-2</v>
@@ -4648,7 +5194,7 @@
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
-        <v>146</v>
+        <v>158</v>
       </c>
       <c r="B11">
         <v>1</v>
@@ -4656,7 +5202,7 @@
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
-        <v>147</v>
+        <v>159</v>
       </c>
       <c r="B12">
         <f>'DCF Base'!M3</f>
@@ -4665,7 +5211,7 @@
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
-        <v>148</v>
+        <v>160</v>
       </c>
       <c r="B13">
         <f>'DCF Base'!M12</f>
@@ -4674,7 +5220,7 @@
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
-        <v>149</v>
+        <v>161</v>
       </c>
       <c r="B14">
         <f>L4*(1+B12)*(1-'DCF Base'!M7)/(B13-B12)</f>
@@ -4692,7 +5238,7 @@
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
-        <v>150</v>
+        <v>162</v>
       </c>
       <c r="B16">
         <f>SUM(C9:L9)</f>
@@ -4701,7 +5247,7 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
-        <v>151</v>
+        <v>163</v>
       </c>
       <c r="B17">
         <f>B16+B15</f>
@@ -4710,7 +5256,7 @@
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
-        <v>152</v>
+        <v>164</v>
       </c>
       <c r="B18">
         <v>13.633262999999999</v>
@@ -4718,7 +5264,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
-        <v>153</v>
+        <v>165</v>
       </c>
       <c r="B19">
         <f>B17/B18</f>
@@ -4727,7 +5273,7 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
-        <v>154</v>
+        <v>166</v>
       </c>
       <c r="B20">
         <f>'DCF Base'!B30</f>
@@ -4736,7 +5282,7 @@
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
-        <v>155</v>
+        <v>167</v>
       </c>
       <c r="B21">
         <f>B20+B19</f>
@@ -4791,7 +5337,7 @@
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>137</v>
+        <v>149</v>
       </c>
       <c r="C2">
         <f>'DCF Base'!C4</f>
@@ -4836,7 +5382,7 @@
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>138</v>
+        <v>150</v>
       </c>
       <c r="C3">
         <v>0.5</v>
@@ -4871,7 +5417,7 @@
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
-        <v>139</v>
+        <v>151</v>
       </c>
       <c r="C4">
         <f>C2*B10*C3</f>
@@ -4916,7 +5462,7 @@
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
-        <v>140</v>
+        <v>152</v>
       </c>
       <c r="C5">
         <f>0.5*B11*D2*B10</f>
@@ -4953,7 +5499,7 @@
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
-        <v>141</v>
+        <v>153</v>
       </c>
       <c r="C6">
         <f>'DCF Base'!C7</f>
@@ -4998,7 +5544,7 @@
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
-        <v>142</v>
+        <v>154</v>
       </c>
       <c r="C7">
         <f t="shared" ref="C7:L7" si="0">(C4-C5)*(1-C6)</f>
@@ -5043,7 +5589,7 @@
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
-        <v>143</v>
+        <v>155</v>
       </c>
       <c r="C8">
         <f>'DCF Base'!C13</f>
@@ -5088,7 +5634,7 @@
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
-        <v>144</v>
+        <v>156</v>
       </c>
       <c r="C9">
         <f t="shared" ref="C9:L9" si="1">C7*C8</f>
@@ -5133,7 +5679,7 @@
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
-        <v>145</v>
+        <v>157</v>
       </c>
       <c r="B10">
         <v>4.8202996236254951E-2</v>
@@ -5141,7 +5687,7 @@
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
-        <v>146</v>
+        <v>158</v>
       </c>
       <c r="B11">
         <v>1</v>
@@ -5149,7 +5695,7 @@
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
-        <v>147</v>
+        <v>159</v>
       </c>
       <c r="B12">
         <f>'DCF Base'!M3</f>
@@ -5158,7 +5704,7 @@
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
-        <v>148</v>
+        <v>160</v>
       </c>
       <c r="B13">
         <f>'DCF Base'!M12</f>
@@ -5167,7 +5713,7 @@
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
-        <v>149</v>
+        <v>161</v>
       </c>
       <c r="B14">
         <f>L4*(1+B12)*(1-'DCF Base'!M7)/(B13-B12)</f>
@@ -5185,7 +5731,7 @@
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
-        <v>150</v>
+        <v>162</v>
       </c>
       <c r="B16">
         <f>SUM(C9:L9)</f>
@@ -5194,7 +5740,7 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
-        <v>151</v>
+        <v>163</v>
       </c>
       <c r="B17">
         <f>B16+B15</f>
@@ -5203,7 +5749,7 @@
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
-        <v>152</v>
+        <v>164</v>
       </c>
       <c r="B18">
         <v>13.633262999999999</v>
@@ -5211,7 +5757,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
-        <v>153</v>
+        <v>165</v>
       </c>
       <c r="B19">
         <f>B17/B18</f>
@@ -5220,7 +5766,7 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
-        <v>154</v>
+        <v>166</v>
       </c>
       <c r="B20">
         <f>'DCF Base'!B30</f>
@@ -5229,7 +5775,7 @@
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
-        <v>155</v>
+        <v>167</v>
       </c>
       <c r="B21">
         <f>B20+B19</f>
@@ -5284,7 +5830,7 @@
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>137</v>
+        <v>149</v>
       </c>
       <c r="C2">
         <f>'DCF Base'!C4</f>
@@ -5329,7 +5875,7 @@
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>138</v>
+        <v>150</v>
       </c>
       <c r="C3">
         <v>0.5</v>
@@ -5364,7 +5910,7 @@
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
-        <v>139</v>
+        <v>151</v>
       </c>
       <c r="C4">
         <f>C2*B10*C3</f>
@@ -5409,7 +5955,7 @@
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
-        <v>140</v>
+        <v>152</v>
       </c>
       <c r="C5">
         <f>0.5*B11*D2*B10</f>
@@ -5446,7 +5992,7 @@
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
-        <v>141</v>
+        <v>153</v>
       </c>
       <c r="C6">
         <f>'DCF Base'!C7</f>
@@ -5491,7 +6037,7 @@
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
-        <v>142</v>
+        <v>154</v>
       </c>
       <c r="C7">
         <f t="shared" ref="C7:L7" si="0">(C4-C5)*(1-C6)</f>
@@ -5536,7 +6082,7 @@
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
-        <v>143</v>
+        <v>155</v>
       </c>
       <c r="C8">
         <f>'DCF Base'!C13</f>
@@ -5581,7 +6127,7 @@
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
-        <v>144</v>
+        <v>156</v>
       </c>
       <c r="C9">
         <f t="shared" ref="C9:L9" si="1">C7*C8</f>
@@ -5626,7 +6172,7 @@
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
-        <v>145</v>
+        <v>157</v>
       </c>
       <c r="B10">
         <v>6.9767441860465115E-2</v>
@@ -5634,7 +6180,7 @@
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
-        <v>146</v>
+        <v>158</v>
       </c>
       <c r="B11">
         <v>1</v>
@@ -5642,7 +6188,7 @@
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
-        <v>147</v>
+        <v>159</v>
       </c>
       <c r="B12">
         <f>'DCF Base'!M3</f>
@@ -5651,7 +6197,7 @@
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
-        <v>148</v>
+        <v>160</v>
       </c>
       <c r="B13">
         <f>'DCF Base'!M12</f>
@@ -5660,7 +6206,7 @@
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
-        <v>149</v>
+        <v>161</v>
       </c>
       <c r="B14">
         <f>L4*(1+B12)*(1-'DCF Base'!M7)/(B13-B12)</f>
@@ -5678,7 +6224,7 @@
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
-        <v>150</v>
+        <v>162</v>
       </c>
       <c r="B16">
         <f>SUM(C9:L9)</f>
@@ -5687,7 +6233,7 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
-        <v>151</v>
+        <v>163</v>
       </c>
       <c r="B17">
         <f>B16+B15</f>
@@ -5696,7 +6242,7 @@
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
-        <v>152</v>
+        <v>164</v>
       </c>
       <c r="B18">
         <v>13.633262999999999</v>
@@ -5704,7 +6250,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
-        <v>153</v>
+        <v>165</v>
       </c>
       <c r="B19">
         <f>B17/B18</f>
@@ -5713,7 +6259,7 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
-        <v>154</v>
+        <v>166</v>
       </c>
       <c r="B20">
         <f>'DCF Base'!B30</f>
@@ -5722,7 +6268,7 @@
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
-        <v>155</v>
+        <v>167</v>
       </c>
       <c r="B21">
         <f>B20+B19</f>
@@ -5742,13 +6288,13 @@
     <row r="1" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A1" s="1"/>
       <c r="B1" s="1" t="s">
-        <v>156</v>
+        <v>168</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>152</v>
+        <v>164</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>157</v>
+        <v>169</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>59</v>
@@ -5757,36 +6303,36 @@
         <v>60</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>158</v>
+        <v>170</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>159</v>
+        <v>171</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>160</v>
+        <v>172</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>161</v>
+        <v>173</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>162</v>
+        <v>174</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>163</v>
+        <v>175</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>164</v>
+        <v>176</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>165</v>
+        <v>177</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>166</v>
+        <v>178</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>167</v>
+        <v>179</v>
       </c>
       <c r="B2">
         <v>93.160003662109375</v>
@@ -5839,7 +6385,7 @@
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>168</v>
+        <v>180</v>
       </c>
       <c r="B3">
         <v>118.1999969482422</v>
@@ -5892,7 +6438,7 @@
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
-        <v>169</v>
+        <v>181</v>
       </c>
       <c r="B4">
         <v>27.559999465942379</v>
@@ -5945,7 +6491,7 @@
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
-        <v>170</v>
+        <v>182</v>
       </c>
       <c r="B5">
         <v>125.30999755859381</v>
@@ -5998,7 +6544,7 @@
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
-        <v>171</v>
+        <v>183</v>
       </c>
       <c r="B6">
         <v>145.07000732421881</v>
@@ -6978,18 +7524,18 @@
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="1"/>
       <c r="B1" s="1" t="s">
-        <v>172</v>
+        <v>184</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>173</v>
+        <v>185</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>174</v>
+        <v>186</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>175</v>
+        <v>187</v>
       </c>
       <c r="B2">
         <v>103.79300000000001</v>
@@ -7003,7 +7549,7 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>176</v>
+        <v>188</v>
       </c>
       <c r="B3">
         <v>8.1910000000000007</v>
@@ -7062,7 +7608,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
-        <v>177</v>
+        <v>189</v>
       </c>
       <c r="B7">
         <v>13.633262999999999</v>
@@ -7076,7 +7622,7 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
-        <v>178</v>
+        <v>190</v>
       </c>
       <c r="B8">
         <v>11.090646475186521</v>
@@ -7090,7 +7636,7 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
-        <v>179</v>
+        <v>191</v>
       </c>
       <c r="B9">
         <f>B4*B8</f>
@@ -7107,7 +7653,7 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
-        <v>180</v>
+        <v>192</v>
       </c>
       <c r="B10">
         <f>B9-B5+B6</f>
@@ -7152,36 +7698,36 @@
     <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" s="1"/>
       <c r="B1" s="1" t="s">
-        <v>188</v>
+        <v>200</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>189</v>
+        <v>201</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>190</v>
+        <v>202</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>191</v>
+        <v>203</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>192</v>
+        <v>204</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>193</v>
+        <v>205</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>194</v>
+        <v>206</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>195</v>
+        <v>207</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>196</v>
+        <v>208</v>
       </c>
       <c r="B2" t="s">
-        <v>181</v>
+        <v>193</v>
       </c>
       <c r="C2">
         <v>1250</v>
@@ -7209,10 +7755,10 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>197</v>
+        <v>209</v>
       </c>
       <c r="B3" t="s">
-        <v>182</v>
+        <v>194</v>
       </c>
       <c r="C3">
         <v>1420</v>
@@ -7240,10 +7786,10 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
-        <v>198</v>
+        <v>210</v>
       </c>
       <c r="B4" t="s">
-        <v>183</v>
+        <v>195</v>
       </c>
       <c r="C4">
         <v>1000</v>
@@ -7271,10 +7817,10 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
-        <v>199</v>
+        <v>211</v>
       </c>
       <c r="B5" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="C5">
         <v>2650</v>
@@ -7295,10 +7841,10 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
-        <v>200</v>
+        <v>212</v>
       </c>
       <c r="B6" t="s">
-        <v>185</v>
+        <v>197</v>
       </c>
       <c r="C6">
         <v>580</v>
@@ -7326,10 +7872,10 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
-        <v>201</v>
+        <v>213</v>
       </c>
       <c r="B7" t="s">
-        <v>186</v>
+        <v>198</v>
       </c>
       <c r="C7">
         <v>692</v>
@@ -7350,10 +7896,10 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
-        <v>202</v>
+        <v>214</v>
       </c>
       <c r="B8" t="s">
-        <v>187</v>
+        <v>199</v>
       </c>
       <c r="C8">
         <v>1400</v>
@@ -7385,13 +7931,13 @@
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="1"/>
       <c r="B1" s="1" t="s">
-        <v>172</v>
+        <v>184</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>173</v>
+        <v>185</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>174</v>
+        <v>186</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
@@ -7438,7 +7984,7 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
-        <v>177</v>
+        <v>189</v>
       </c>
       <c r="B5">
         <v>13.633262999999999</v>
@@ -7452,7 +7998,7 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
-        <v>203</v>
+        <v>215</v>
       </c>
       <c r="B6">
         <v>10.102725875596541</v>
@@ -7466,7 +8012,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
-        <v>179</v>
+        <v>191</v>
       </c>
       <c r="B7">
         <f>B2*B6</f>
@@ -7483,7 +8029,7 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
-        <v>180</v>
+        <v>192</v>
       </c>
       <c r="B8">
         <f>B7-B3+B4</f>

</xml_diff>